<commit_message>
Fill 5 more approved rows, add anatomical-region candidate matches sheet
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E9QvuhBZminJvrtKVH8YY8
</commit_message>
<xml_diff>
--- a/kirill/outputs/2026-09-03-קופח-מכרזים-מולא-מטבלאות-אביזרים.xlsx
+++ b/kirill/outputs/2026-09-03-קופח-מכרזים-מולא-מטבלאות-אביזרים.xlsx
@@ -9,6 +9,7 @@
     <sheet name="נספח יא" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="גיליון1" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="לוג התאמות (מיפוי)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="הצעות לפי אזור אנטומי" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'נספח יא'!$A$4:$K$79</definedName>
@@ -21,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="17">
     <font>
       <name val="Carlito"/>
       <sz val="11"/>
@@ -88,8 +89,29 @@
       <name val="Arial"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -132,8 +154,18 @@
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E2F3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF9E6"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -170,11 +202,55 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -238,6 +314,15 @@
     <xf numFmtId="0" fontId="10" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1542,6 +1627,21 @@
           <t>קיים במגוון</t>
         </is>
       </c>
+      <c r="M27" t="n">
+        <v>31</v>
+      </c>
+      <c r="N27" t="n">
+        <v>72</v>
+      </c>
+      <c r="O27" t="n">
+        <v>103</v>
+      </c>
+      <c r="P27" t="n">
+        <v>45</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>53</v>
+      </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="10">
       <c r="A28" s="15" t="inlineStr">
@@ -2222,6 +2322,21 @@
           <t>קיים במגוון</t>
         </is>
       </c>
+      <c r="M45" t="n">
+        <v>28</v>
+      </c>
+      <c r="N45" t="n">
+        <v>67</v>
+      </c>
+      <c r="O45" t="n">
+        <v>95</v>
+      </c>
+      <c r="P45" t="n">
+        <v>38</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>45</v>
+      </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="10">
       <c r="A46" s="15" t="inlineStr">
@@ -2387,6 +2502,21 @@
           <t>המוצר מכילים כרית ג'ל ולא סיליקון</t>
         </is>
       </c>
+      <c r="M49" t="n">
+        <v>28</v>
+      </c>
+      <c r="N49" t="n">
+        <v>67</v>
+      </c>
+      <c r="O49" t="n">
+        <v>95</v>
+      </c>
+      <c r="P49" t="n">
+        <v>38</v>
+      </c>
+      <c r="Q49" t="n">
+        <v>45</v>
+      </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="10">
       <c r="A50" s="15" t="inlineStr">
@@ -3229,6 +3359,21 @@
           <t>פרוייקט סורסינג נעצר - קיימות הצעות ודוגמאות</t>
         </is>
       </c>
+      <c r="M71" t="n">
+        <v>89</v>
+      </c>
+      <c r="N71" t="n">
+        <v>209</v>
+      </c>
+      <c r="O71" t="n">
+        <v>298</v>
+      </c>
+      <c r="P71" t="n">
+        <v>210</v>
+      </c>
+      <c r="Q71" t="n">
+        <v>248</v>
+      </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="10">
       <c r="A72" s="15" t="inlineStr">
@@ -3265,6 +3410,21 @@
         <is>
           <t>חדש במגוון</t>
         </is>
+      </c>
+      <c r="M72" t="n">
+        <v>96</v>
+      </c>
+      <c r="N72" t="n">
+        <v>225</v>
+      </c>
+      <c r="O72" t="n">
+        <v>321</v>
+      </c>
+      <c r="P72" t="n">
+        <v>230</v>
+      </c>
+      <c r="Q72" t="n">
+        <v>271</v>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="10">
@@ -4742,25 +4902,29 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="22" t="n">
+      <c r="A24" s="25" t="n">
         <v>27</v>
       </c>
-      <c r="B24" s="22" t="inlineStr">
+      <c r="B24" s="25" t="inlineStr">
         <is>
           <t>חגורת גב עם תמיכות לנשים בהיריון</t>
         </is>
       </c>
-      <c r="C24" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — נמצאה התאמה קרובה (לא מדויקת) בטבלת המחירים, ייתכן טעות כתיב/ניסוח שונה — דורש אימות ידני</t>
-        </is>
-      </c>
-      <c r="D24" s="24" t="inlineStr">
-        <is>
-          <t>חגורת גב עם תמיכה לנשים בהריון</t>
-        </is>
-      </c>
-      <c r="E24" s="24" t="inlineStr"/>
+      <c r="C24" s="26" t="inlineStr">
+        <is>
+          <t>מולא (אושר ידנית 03/09 - הבדל קוסמטי בלבד באיות/ניסוח)</t>
+        </is>
+      </c>
+      <c r="D24" s="27" t="inlineStr">
+        <is>
+          <t>דף 02!17</t>
+        </is>
+      </c>
+      <c r="E24" s="27" t="inlineStr">
+        <is>
+          <t>(31, 72, 103, 45, 53)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="22" t="n">
@@ -5108,25 +5272,29 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="22" t="n">
+      <c r="A42" s="25" t="n">
         <v>45</v>
       </c>
-      <c r="B42" s="22" t="inlineStr">
+      <c r="B42" s="25" t="inlineStr">
         <is>
           <t>מייצבים חצי קשיחים עם כריות אוויר</t>
         </is>
       </c>
-      <c r="C42" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — נמצאה התאמה קרובה (לא מדויקת) בטבלת המחירים, ייתכן טעות כתיב/ניסוח שונה — דורש אימות ידני</t>
-        </is>
-      </c>
-      <c r="D42" s="24" t="inlineStr">
-        <is>
-          <t>מייצבים חצי קשיחים עם כריות אויר; מייצבים חצי קשיחים עם שרוכים ו/או רצועות</t>
-        </is>
-      </c>
-      <c r="E42" s="24" t="inlineStr"/>
+      <c r="C42" s="26" t="inlineStr">
+        <is>
+          <t>מולא (אושר ידנית 03/09 - הבדל קוסמטי בלבד באיות/ניסוח)</t>
+        </is>
+      </c>
+      <c r="D42" s="27" t="inlineStr">
+        <is>
+          <t>דף 02!36</t>
+        </is>
+      </c>
+      <c r="E42" s="27" t="inlineStr">
+        <is>
+          <t>(28, 67, 95, 38, 45)</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="28" t="n">
@@ -5196,25 +5364,29 @@
       <c r="E45" s="24" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="22" t="n">
+      <c r="A46" s="25" t="n">
         <v>49</v>
       </c>
-      <c r="B46" s="22" t="inlineStr">
+      <c r="B46" s="25" t="inlineStr">
         <is>
           <t>קרסוליה עם סיליקון עם או בלי רצועות</t>
         </is>
       </c>
-      <c r="C46" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — נמצאה התאמה קרובה (לא מדויקת) בטבלת המחירים, ייתכן טעות כתיב/ניסוח שונה — דורש אימות ידני</t>
-        </is>
-      </c>
-      <c r="D46" s="24" t="inlineStr">
-        <is>
-          <t>קרסוליה עם סיליקון או בלי רצועות</t>
-        </is>
-      </c>
-      <c r="E46" s="24" t="inlineStr"/>
+      <c r="C46" s="26" t="inlineStr">
+        <is>
+          <t>מולא (אושר ידנית 03/09 - הבדל קוסמטי בלבד באיות/ניסוח)</t>
+        </is>
+      </c>
+      <c r="D46" s="27" t="inlineStr">
+        <is>
+          <t>דף 01!6,7</t>
+        </is>
+      </c>
+      <c r="E46" s="27" t="inlineStr">
+        <is>
+          <t>(28, 67, 95, 38, 45)</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="22" t="n">
@@ -5626,46 +5798,54 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="22" t="n">
+      <c r="A68" s="25" t="n">
         <v>71</v>
       </c>
-      <c r="B68" s="22" t="inlineStr">
+      <c r="B68" s="25" t="inlineStr">
         <is>
           <t>גרביים אלסטיות להריון AT - ורידים, בצקות ורידיות, בצקות ליפאדמה</t>
         </is>
       </c>
-      <c r="C68" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — נמצאה התאמה קרובה (לא מדויקת) בטבלת המחירים, ייתכן טעות כתיב/ניסוח שונה — דורש אימות ידני</t>
-        </is>
-      </c>
-      <c r="D68" s="24" t="inlineStr">
-        <is>
-          <t>גרביים אלסטיות להריון AT - ורידים, בצקות ורידיות, בצקות לימפאדמה; גרביים אלסטיות עד הברך AD - ורידים, בצקות ורידיות, בצקות לימפאדמה; גרביים אלסטיות מכנסיים AT - ורידים, בצקות ורידיות, בצקות לימפאדמה</t>
-        </is>
-      </c>
-      <c r="E68" s="24" t="inlineStr"/>
+      <c r="C68" s="26" t="inlineStr">
+        <is>
+          <t>מולא (אושר ידנית 03/09 - הבדל קוסמטי בלבד באיות/ניסוח)</t>
+        </is>
+      </c>
+      <c r="D68" s="27" t="inlineStr">
+        <is>
+          <t>דף 01!23</t>
+        </is>
+      </c>
+      <c r="E68" s="27" t="inlineStr">
+        <is>
+          <t>(89, 209, 298, 210, 248)</t>
+        </is>
+      </c>
     </row>
     <row r="69">
-      <c r="A69" s="22" t="n">
+      <c r="A69" s="25" t="n">
         <v>72</v>
       </c>
-      <c r="B69" s="22" t="inlineStr">
+      <c r="B69" s="25" t="inlineStr">
         <is>
           <t>חגורת שבר הרניה חד צדדית</t>
         </is>
       </c>
-      <c r="C69" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — נמצאה התאמה קרובה (לא מדויקת) בטבלת המחירים, ייתכן טעות כתיב/ניסוח שונה — דורש אימות ידני</t>
-        </is>
-      </c>
-      <c r="D69" s="24" t="inlineStr">
-        <is>
-          <t>חגורת שבר הבקע חד צדדית; חגורת שבר הרניה דו"צ</t>
-        </is>
-      </c>
-      <c r="E69" s="24" t="inlineStr"/>
+      <c r="C69" s="26" t="inlineStr">
+        <is>
+          <t>מולא (אושר ידנית 03/09 - הבדל קוסמטי בלבד באיות/ניסוח)</t>
+        </is>
+      </c>
+      <c r="D69" s="27" t="inlineStr">
+        <is>
+          <t>דף 01!24</t>
+        </is>
+      </c>
+      <c r="E69" s="27" t="inlineStr">
+        <is>
+          <t>(96, 225, 321, 230, 271)</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="25" t="n">
@@ -5806,4 +5986,3381 @@
   <autoFilter ref="A1:E76"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F199"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" style="10" min="1" max="1"/>
+    <col width="6" customWidth="1" style="10" min="2" max="2"/>
+    <col width="55" customWidth="1" style="10" min="3" max="3"/>
+    <col width="22" customWidth="1" style="10" min="4" max="4"/>
+    <col width="20" customWidth="1" style="10" min="5" max="5"/>
+    <col width="10" customWidth="1" style="10" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="31" t="inlineStr">
+        <is>
+          <t>הצעות התאמה לפי אזור אנטומי — לשורות שלא נמצאה להן התאמת טקסט (35 שורות, סבב 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="32" t="inlineStr">
+        <is>
+          <t>חשוב: ההתאמה כאן לפי אזור אנטומי בלבד (לא ניסוח דומה) — לא מולא כלום אוטומטית. יש לבחור ידנית לכל שורה במכרז, אם בכלל, איזה מועמד/ים למטה מתאימים לה, ולבקש מילוי בפירוש.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="33" t="inlineStr">
+        <is>
+          <t>אזור אנטומי: שורש כף יד  (מקורות מחיר שנבדקו: שורש כף יד)</t>
+        </is>
+      </c>
+      <c r="B4" s="34" t="n"/>
+      <c r="C4" s="34" t="n"/>
+      <c r="D4" s="34" t="n"/>
+      <c r="E4" s="34" t="n"/>
+      <c r="F4" s="34" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="35" t="inlineStr">
+        <is>
+          <t>שורות במכרז שטרם מולאו:</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="22" t="inlineStr">
+        <is>
+          <t>שורה 10</t>
+        </is>
+      </c>
+      <c r="B6" s="22" t="inlineStr">
+        <is>
+          <t>אימבלוייזר לתינוקות לשורש כף יד</t>
+        </is>
+      </c>
+      <c r="C6" s="36" t="n"/>
+      <c r="D6" s="36" t="n"/>
+      <c r="E6" s="36" t="n"/>
+      <c r="F6" s="37" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="22" t="inlineStr">
+        <is>
+          <t>שורה 11</t>
+        </is>
+      </c>
+      <c r="B7" s="22" t="inlineStr">
+        <is>
+          <t>חבק שורש כף יד ללא סד</t>
+        </is>
+      </c>
+      <c r="C7" s="36" t="n"/>
+      <c r="D7" s="36" t="n"/>
+      <c r="E7" s="36" t="n"/>
+      <c r="F7" s="37" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="35" t="inlineStr">
+        <is>
+          <t>מועמדים אפשריים מטבלת האביזרים (אותו אזור אנטומי):</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="38" t="inlineStr">
+        <is>
+          <t>גיליון</t>
+        </is>
+      </c>
+      <c r="B10" s="38" t="inlineStr">
+        <is>
+          <t>שורה</t>
+        </is>
+      </c>
+      <c r="C10" s="38" t="inlineStr">
+        <is>
+          <t>התוויה רפואית (טבלת המחירים)</t>
+        </is>
+      </c>
+      <c r="D10" s="38" t="inlineStr">
+        <is>
+          <t>עצמית / כללית / כולל</t>
+        </is>
+      </c>
+      <c r="E10" s="38" t="inlineStr">
+        <is>
+          <t>ליבואן ללא/כולל מע"מ</t>
+        </is>
+      </c>
+      <c r="F10" s="38" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="39" t="inlineStr">
+        <is>
+          <t>דף 03</t>
+        </is>
+      </c>
+      <c r="B11" s="39" t="n">
+        <v>17</v>
+      </c>
+      <c r="C11" s="39" t="inlineStr">
+        <is>
+          <t>תומך/מייצב פעיל לשורש כף היד עם אגודל (עם סיליקון)</t>
+        </is>
+      </c>
+      <c r="D11" s="39" t="inlineStr">
+        <is>
+          <t>40 / 95 / 135</t>
+        </is>
+      </c>
+      <c r="E11" s="39" t="inlineStr">
+        <is>
+          <t>72 / 85</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="39" t="inlineStr">
+        <is>
+          <t>דף 03</t>
+        </is>
+      </c>
+      <c r="B12" s="39" t="n">
+        <v>18</v>
+      </c>
+      <c r="C12" s="39" t="inlineStr">
+        <is>
+          <t>תומך/מייצב פעיל לשורש כף היד עם אגודל (עם סיליקון)</t>
+        </is>
+      </c>
+      <c r="D12" s="39" t="inlineStr">
+        <is>
+          <t>39 / 91 / 130</t>
+        </is>
+      </c>
+      <c r="E12" s="39" t="inlineStr">
+        <is>
+          <t>68 / 80</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="39" t="inlineStr">
+        <is>
+          <t>דף 03</t>
+        </is>
+      </c>
+      <c r="B13" s="39" t="n">
+        <v>19</v>
+      </c>
+      <c r="C13" s="39" t="inlineStr">
+        <is>
+          <t>תומך/מייצב פעיל לשורש כף היד ללא אגודל (עם סיליקון)</t>
+        </is>
+      </c>
+      <c r="D13" s="39" t="inlineStr">
+        <is>
+          <t>40 / 93 / 133</t>
+        </is>
+      </c>
+      <c r="E13" s="39" t="inlineStr">
+        <is>
+          <t>70 / 83</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="39" t="inlineStr">
+        <is>
+          <t>דף 03</t>
+        </is>
+      </c>
+      <c r="B14" s="39" t="n">
+        <v>20</v>
+      </c>
+      <c r="C14" s="39" t="inlineStr">
+        <is>
+          <t>תומך/מייצב פעיל לשורש כף היד ללא אגודל (עם סיליקון)</t>
+        </is>
+      </c>
+      <c r="D14" s="39" t="inlineStr">
+        <is>
+          <t>27 / 63 / 90</t>
+        </is>
+      </c>
+      <c r="E14" s="39" t="inlineStr">
+        <is>
+          <t>34 / 40</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="39" t="inlineStr">
+        <is>
+          <t>דף 03</t>
+        </is>
+      </c>
+      <c r="B15" s="39" t="n">
+        <v>21</v>
+      </c>
+      <c r="C15" s="39" t="inlineStr">
+        <is>
+          <t>מגן שורש כף יד עם קיבוע של האגודל (מקבע קשיח)</t>
+        </is>
+      </c>
+      <c r="D15" s="39" t="inlineStr">
+        <is>
+          <t>30 / 70 / 100</t>
+        </is>
+      </c>
+      <c r="E15" s="39" t="inlineStr">
+        <is>
+          <t>42 / 50</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="39" t="inlineStr">
+        <is>
+          <t>דף 03</t>
+        </is>
+      </c>
+      <c r="B16" s="39" t="n">
+        <v>22</v>
+      </c>
+      <c r="C16" s="39" t="inlineStr">
+        <is>
+          <t>מגן שורש כף יד ללא קיבוע של האגודל (מקבע קשיח)</t>
+        </is>
+      </c>
+      <c r="D16" s="39" t="inlineStr">
+        <is>
+          <t>27 / 64 / 91</t>
+        </is>
+      </c>
+      <c r="E16" s="39" t="inlineStr">
+        <is>
+          <t>35 / 41</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="39" t="inlineStr">
+        <is>
+          <t>דף 03</t>
+        </is>
+      </c>
+      <c r="B17" s="39" t="n">
+        <v>23</v>
+      </c>
+      <c r="C17" s="39" t="inlineStr">
+        <is>
+          <t>מגן שורש כף יד ללא קיבוע של האגודל (מקבע קשיח)</t>
+        </is>
+      </c>
+      <c r="D17" s="39" t="inlineStr">
+        <is>
+          <t>30 / 68 / 98</t>
+        </is>
+      </c>
+      <c r="E17" s="39" t="inlineStr">
+        <is>
+          <t>41 / 48</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="39" t="inlineStr">
+        <is>
+          <t>דף 03</t>
+        </is>
+      </c>
+      <c r="B18" s="39" t="n">
+        <v>24</v>
+      </c>
+      <c r="C18" s="39" t="inlineStr">
+        <is>
+          <t>מגן שורש כף יד ללא קיבוע של האגודל (מקבע קשיח)</t>
+        </is>
+      </c>
+      <c r="D18" s="39" t="inlineStr">
+        <is>
+          <t>28 / 67 / 95</t>
+        </is>
+      </c>
+      <c r="E18" s="39" t="inlineStr">
+        <is>
+          <t>38 / 45</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="39" t="inlineStr">
+        <is>
+          <t>דף 03</t>
+        </is>
+      </c>
+      <c r="B19" s="39" t="n">
+        <v>25</v>
+      </c>
+      <c r="C19" s="39" t="inlineStr">
+        <is>
+          <t>מגן שורש כף יד ללא קיבוע של האגודל (מקבע קשיח)</t>
+        </is>
+      </c>
+      <c r="D19" s="39" t="inlineStr">
+        <is>
+          <t>28 / 65 / 93</t>
+        </is>
+      </c>
+      <c r="E19" s="39" t="inlineStr">
+        <is>
+          <t>37 / 43</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="39" t="inlineStr">
+        <is>
+          <t>דף 03</t>
+        </is>
+      </c>
+      <c r="B20" s="39" t="n">
+        <v>26</v>
+      </c>
+      <c r="C20" s="39" t="inlineStr">
+        <is>
+          <t>מגן שורש כף יד ללא קיבוע של האגודל (מקבע קשיח)</t>
+        </is>
+      </c>
+      <c r="D20" s="39" t="inlineStr">
+        <is>
+          <t>53 / 123 / 176</t>
+        </is>
+      </c>
+      <c r="E20" s="39" t="inlineStr">
+        <is>
+          <t>107 / 126</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="33" t="inlineStr">
+        <is>
+          <t>אזור אנטומי: מרפק  (מקורות מחיר שנבדקו: מרפק)</t>
+        </is>
+      </c>
+      <c r="B23" s="34" t="n"/>
+      <c r="C23" s="34" t="n"/>
+      <c r="D23" s="34" t="n"/>
+      <c r="E23" s="34" t="n"/>
+      <c r="F23" s="34" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="35" t="inlineStr">
+        <is>
+          <t>שורות במכרז שטרם מולאו:</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="22" t="inlineStr">
+        <is>
+          <t>שורה 12</t>
+        </is>
+      </c>
+      <c r="B25" s="22" t="inlineStr">
+        <is>
+          <t>תומך פעיל למרפק עם סיליקון (לפחות 10 ס"מ מעל ומתחת לקו המפרק)</t>
+        </is>
+      </c>
+      <c r="C25" s="36" t="n"/>
+      <c r="D25" s="36" t="n"/>
+      <c r="E25" s="36" t="n"/>
+      <c r="F25" s="37" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="22" t="inlineStr">
+        <is>
+          <t>שורה 14</t>
+        </is>
+      </c>
+      <c r="B26" s="22" t="inlineStr">
+        <is>
+          <t>מגן מרפק עם חיזוקי מתכת וציר יישור/ כיפוף מייצב POST OP</t>
+        </is>
+      </c>
+      <c r="C26" s="36" t="n"/>
+      <c r="D26" s="36" t="n"/>
+      <c r="E26" s="36" t="n"/>
+      <c r="F26" s="37" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="22" t="inlineStr">
+        <is>
+          <t>שורה 15</t>
+        </is>
+      </c>
+      <c r="B27" s="22" t="inlineStr">
+        <is>
+          <t>שרוול למרפק אלסטי</t>
+        </is>
+      </c>
+      <c r="C27" s="36" t="n"/>
+      <c r="D27" s="36" t="n"/>
+      <c r="E27" s="36" t="n"/>
+      <c r="F27" s="37" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="35" t="inlineStr">
+        <is>
+          <t>מועמדים אפשריים מטבלת האביזרים (אותו אזור אנטומי):</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="38" t="inlineStr">
+        <is>
+          <t>גיליון</t>
+        </is>
+      </c>
+      <c r="B30" s="38" t="inlineStr">
+        <is>
+          <t>שורה</t>
+        </is>
+      </c>
+      <c r="C30" s="38" t="inlineStr">
+        <is>
+          <t>התוויה רפואית (טבלת המחירים)</t>
+        </is>
+      </c>
+      <c r="D30" s="38" t="inlineStr">
+        <is>
+          <t>עצמית / כללית / כולל</t>
+        </is>
+      </c>
+      <c r="E30" s="38" t="inlineStr">
+        <is>
+          <t>ליבואן ללא/כולל מע"מ</t>
+        </is>
+      </c>
+      <c r="F30" s="38" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B31" s="39" t="n">
+        <v>2</v>
+      </c>
+      <c r="C31" s="39" t="inlineStr">
+        <is>
+          <t>מייצב אגודל ללא שורש כף יד</t>
+        </is>
+      </c>
+      <c r="D31" s="39" t="inlineStr">
+        <is>
+          <t>27 / 64 / 91</t>
+        </is>
+      </c>
+      <c r="E31" s="39" t="inlineStr">
+        <is>
+          <t>35 / 41</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B32" s="39" t="n">
+        <v>3</v>
+      </c>
+      <c r="C32" s="39" t="inlineStr">
+        <is>
+          <t>מייצב אגודל ללא שורש כף יד</t>
+        </is>
+      </c>
+      <c r="D32" s="39" t="inlineStr">
+        <is>
+          <t>34 / 81 / 115</t>
+        </is>
+      </c>
+      <c r="E32" s="39" t="inlineStr">
+        <is>
+          <t>55 / 65</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B33" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="C33" s="39" t="inlineStr">
+        <is>
+          <t>תומך פעיל למרפק עם כרית למרפק טניס</t>
+        </is>
+      </c>
+      <c r="D33" s="39" t="inlineStr">
+        <is>
+          <t>37 / 85 / 122</t>
+        </is>
+      </c>
+      <c r="E33" s="39" t="inlineStr">
+        <is>
+          <t>61 / 72</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B34" s="39" t="n">
+        <v>5</v>
+      </c>
+      <c r="C34" s="39" t="inlineStr">
+        <is>
+          <t>תומך פעיל למרפק עם כרית למרפק טניס</t>
+        </is>
+      </c>
+      <c r="D34" s="39" t="inlineStr">
+        <is>
+          <t>46 / 107 / 153</t>
+        </is>
+      </c>
+      <c r="E34" s="39" t="inlineStr">
+        <is>
+          <t>87 / 103</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B35" s="39" t="n">
+        <v>6</v>
+      </c>
+      <c r="C35" s="39" t="inlineStr">
+        <is>
+          <t>תומך פעיל למרפק עם כרית למרפק טניס</t>
+        </is>
+      </c>
+      <c r="D35" s="39" t="inlineStr">
+        <is>
+          <t>29 / 68 / 97</t>
+        </is>
+      </c>
+      <c r="E35" s="39" t="inlineStr">
+        <is>
+          <t>40 / 47</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B36" s="39" t="n">
+        <v>7</v>
+      </c>
+      <c r="C36" s="39" t="inlineStr">
+        <is>
+          <t>תומך פעיל למרפק עם כרית למרפק טניס</t>
+        </is>
+      </c>
+      <c r="D36" s="39" t="inlineStr">
+        <is>
+          <t>39 / 90 / 129</t>
+        </is>
+      </c>
+      <c r="E36" s="39" t="inlineStr">
+        <is>
+          <t>67 / 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B37" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="C37" s="39" t="inlineStr">
+        <is>
+          <t>רצועה למרפק עם כרית ורצועה מתחת למרפק טניס</t>
+        </is>
+      </c>
+      <c r="D37" s="39" t="inlineStr">
+        <is>
+          <t>30 / 68 / 98</t>
+        </is>
+      </c>
+      <c r="E37" s="39" t="inlineStr">
+        <is>
+          <t>41 / 48</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B38" s="39" t="n">
+        <v>9</v>
+      </c>
+      <c r="C38" s="39" t="inlineStr">
+        <is>
+          <t>רצועה למרפק עם כרית ורצועה מתחת למרפק טניס</t>
+        </is>
+      </c>
+      <c r="D38" s="39" t="inlineStr">
+        <is>
+          <t>24 / 56 / 80</t>
+        </is>
+      </c>
+      <c r="E38" s="39" t="inlineStr">
+        <is>
+          <t>26 / 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="33" t="inlineStr">
+        <is>
+          <t>אזור אנטומי: כתף  (מקורות מחיר שנבדקו: כתף)</t>
+        </is>
+      </c>
+      <c r="B41" s="34" t="n"/>
+      <c r="C41" s="34" t="n"/>
+      <c r="D41" s="34" t="n"/>
+      <c r="E41" s="34" t="n"/>
+      <c r="F41" s="34" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="35" t="inlineStr">
+        <is>
+          <t>שורות במכרז שטרם מולאו:</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="22" t="inlineStr">
+        <is>
+          <t>שורה 16</t>
+        </is>
+      </c>
+      <c r="B43" s="22" t="inlineStr">
+        <is>
+          <t>קיבוע אמה צמודה לבטן לאחר ניתוח</t>
+        </is>
+      </c>
+      <c r="C43" s="36" t="n"/>
+      <c r="D43" s="36" t="n"/>
+      <c r="E43" s="36" t="n"/>
+      <c r="F43" s="37" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="22" t="inlineStr">
+        <is>
+          <t>שורה 21</t>
+        </is>
+      </c>
+      <c r="B44" s="22" t="inlineStr">
+        <is>
+          <t>שמינייה לכתף / עצם הבריח</t>
+        </is>
+      </c>
+      <c r="C44" s="36" t="n"/>
+      <c r="D44" s="36" t="n"/>
+      <c r="E44" s="36" t="n"/>
+      <c r="F44" s="37" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="22" t="inlineStr">
+        <is>
+          <t>שורה 22</t>
+        </is>
+      </c>
+      <c r="B45" s="22" t="inlineStr">
+        <is>
+          <t>מתלה ליד /זרוע</t>
+        </is>
+      </c>
+      <c r="C45" s="36" t="n"/>
+      <c r="D45" s="36" t="n"/>
+      <c r="E45" s="36" t="n"/>
+      <c r="F45" s="37" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="35" t="inlineStr">
+        <is>
+          <t>מועמדים אפשריים מטבלת האביזרים (אותו אזור אנטומי):</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="38" t="inlineStr">
+        <is>
+          <t>גיליון</t>
+        </is>
+      </c>
+      <c r="B48" s="38" t="inlineStr">
+        <is>
+          <t>שורה</t>
+        </is>
+      </c>
+      <c r="C48" s="38" t="inlineStr">
+        <is>
+          <t>התוויה רפואית (טבלת המחירים)</t>
+        </is>
+      </c>
+      <c r="D48" s="38" t="inlineStr">
+        <is>
+          <t>עצמית / כללית / כולל</t>
+        </is>
+      </c>
+      <c r="E48" s="38" t="inlineStr">
+        <is>
+          <t>ליבואן ללא/כולל מע"מ</t>
+        </is>
+      </c>
+      <c r="F48" s="38" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B49" s="39" t="n">
+        <v>21</v>
+      </c>
+      <c r="C49" s="39" t="inlineStr">
+        <is>
+          <t>קיבוע אחרי צניחה/ניתוח לאחר ניתוח</t>
+        </is>
+      </c>
+      <c r="D49" s="39" t="inlineStr">
+        <is>
+          <t>32 / 73 / 105</t>
+        </is>
+      </c>
+      <c r="E49" s="39" t="inlineStr">
+        <is>
+          <t>47 / 55</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B50" s="39" t="n">
+        <v>22</v>
+      </c>
+      <c r="C50" s="39" t="inlineStr">
+        <is>
+          <t>קיבוע אחרי צניחה/ניתוח לאחר ניתוח</t>
+        </is>
+      </c>
+      <c r="D50" s="39" t="inlineStr">
+        <is>
+          <t>30 / 70 / 100</t>
+        </is>
+      </c>
+      <c r="E50" s="39" t="inlineStr">
+        <is>
+          <t>42 / 50</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B51" s="39" t="n">
+        <v>23</v>
+      </c>
+      <c r="C51" s="39" t="inlineStr">
+        <is>
+          <t>קיבוע אחרי צניחה/ניתוח לאחר ניתוח</t>
+        </is>
+      </c>
+      <c r="D51" s="39" t="inlineStr">
+        <is>
+          <t>32 / 74 / 106</t>
+        </is>
+      </c>
+      <c r="E51" s="39" t="inlineStr">
+        <is>
+          <t>48 / 56</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B52" s="39" t="n">
+        <v>24</v>
+      </c>
+      <c r="C52" s="39" t="inlineStr">
+        <is>
+          <t>קיבוע אחרי צניחה/ניתוח לאחר ניתוח</t>
+        </is>
+      </c>
+      <c r="D52" s="39" t="inlineStr">
+        <is>
+          <t>32 / 73 / 105</t>
+        </is>
+      </c>
+      <c r="E52" s="39" t="inlineStr">
+        <is>
+          <t>47 / 55</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B53" s="39" t="n">
+        <v>25</v>
+      </c>
+      <c r="C53" s="39" t="inlineStr">
+        <is>
+          <t>מקבע לזרוע (הומרוס) לאחר שבר</t>
+        </is>
+      </c>
+      <c r="D53" s="39" t="inlineStr">
+        <is>
+          <t>57 / 135 / 192</t>
+        </is>
+      </c>
+      <c r="E53" s="39" t="inlineStr">
+        <is>
+          <t>120 / 142</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B54" s="39" t="n">
+        <v>26</v>
+      </c>
+      <c r="C54" s="39" t="inlineStr">
+        <is>
+          <t>תומך כתף עם סיליקון</t>
+        </is>
+      </c>
+      <c r="D54" s="39" t="inlineStr">
+        <is>
+          <t>42 / 97 / 139</t>
+        </is>
+      </c>
+      <c r="E54" s="39" t="inlineStr">
+        <is>
+          <t>75 / 89</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B55" s="39" t="n">
+        <v>27</v>
+      </c>
+      <c r="C55" s="39" t="inlineStr">
+        <is>
+          <t>מקבע כתף בדרגות רוטציה (סיבוב) משתנות לאחר שבר, פריקה או ניתוח</t>
+        </is>
+      </c>
+      <c r="D55" s="39" t="inlineStr">
+        <is>
+          <t>165 / 387 / 552</t>
+        </is>
+      </c>
+      <c r="E55" s="39" t="inlineStr">
+        <is>
+          <t>425 / 502</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B56" s="39" t="n">
+        <v>28</v>
+      </c>
+      <c r="C56" s="39" t="inlineStr">
+        <is>
+          <t>מקבע כתף בדרגות רוטציה (סיבוב) משתנות לאחר שבר, פריקה או ניתוח</t>
+        </is>
+      </c>
+      <c r="D56" s="39" t="inlineStr">
+        <is>
+          <t>167 / 390 / 557</t>
+        </is>
+      </c>
+      <c r="E56" s="39" t="inlineStr">
+        <is>
+          <t>430 / 507</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B57" s="39" t="n">
+        <v>29</v>
+      </c>
+      <c r="C57" s="39" t="inlineStr">
+        <is>
+          <t>מקבע כתף בדרגות אבדוקציה שונות לאחר שבר, פריקה או ניתוח</t>
+        </is>
+      </c>
+      <c r="D57" s="39" t="inlineStr">
+        <is>
+          <t>101 / 236 / 337</t>
+        </is>
+      </c>
+      <c r="E57" s="39" t="inlineStr">
+        <is>
+          <t>243 / 287</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B58" s="39" t="n">
+        <v>30</v>
+      </c>
+      <c r="C58" s="39" t="inlineStr">
+        <is>
+          <t>מקבע כתף בדרגות אבדוקציה שונות לאחר שבר, פריקה או ניתוח</t>
+        </is>
+      </c>
+      <c r="D58" s="39" t="inlineStr">
+        <is>
+          <t>77 / 180 / 257</t>
+        </is>
+      </c>
+      <c r="E58" s="39" t="inlineStr">
+        <is>
+          <t>175 / 207</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="33" t="inlineStr">
+        <is>
+          <t>אזור אנטומי: גב  (מקורות מחיר שנבדקו: גב, צוואר)</t>
+        </is>
+      </c>
+      <c r="B61" s="34" t="n"/>
+      <c r="C61" s="34" t="n"/>
+      <c r="D61" s="34" t="n"/>
+      <c r="E61" s="34" t="n"/>
+      <c r="F61" s="34" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="35" t="inlineStr">
+        <is>
+          <t>שורות במכרז שטרם מולאו:</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="22" t="inlineStr">
+        <is>
+          <t>שורה 25</t>
+        </is>
+      </c>
+      <c r="B63" s="22" t="inlineStr">
+        <is>
+          <t>חגורת Jewett 3 POINTS</t>
+        </is>
+      </c>
+      <c r="C63" s="36" t="n"/>
+      <c r="D63" s="36" t="n"/>
+      <c r="E63" s="36" t="n"/>
+      <c r="F63" s="37" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="22" t="inlineStr">
+        <is>
+          <t>שורה 28</t>
+        </is>
+      </c>
+      <c r="B64" s="22" t="inlineStr">
+        <is>
+          <t>כיסוי למחוכים לספונדליזיס (ניתן בשב"ן רק בהתוויות שאינן בסל)</t>
+        </is>
+      </c>
+      <c r="C64" s="36" t="n"/>
+      <c r="D64" s="36" t="n"/>
+      <c r="E64" s="36" t="n"/>
+      <c r="F64" s="37" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="22" t="inlineStr">
+        <is>
+          <t>שורה 31</t>
+        </is>
+      </c>
+      <c r="B65" s="22" t="inlineStr">
+        <is>
+          <t>חגורה מייצבת -חזה צוואר /SOMI</t>
+        </is>
+      </c>
+      <c r="C65" s="36" t="n"/>
+      <c r="D65" s="36" t="n"/>
+      <c r="E65" s="36" t="n"/>
+      <c r="F65" s="37" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="22" t="inlineStr">
+        <is>
+          <t>שורה 32</t>
+        </is>
+      </c>
+      <c r="B66" s="22" t="inlineStr">
+        <is>
+          <t>צווארון רך</t>
+        </is>
+      </c>
+      <c r="C66" s="36" t="n"/>
+      <c r="D66" s="36" t="n"/>
+      <c r="E66" s="36" t="n"/>
+      <c r="F66" s="37" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="22" t="inlineStr">
+        <is>
+          <t>שורה 33</t>
+        </is>
+      </c>
+      <c r="B67" s="22" t="inlineStr">
+        <is>
+          <t>חגורת גב אווירירית ללא תמיכות</t>
+        </is>
+      </c>
+      <c r="C67" s="36" t="n"/>
+      <c r="D67" s="36" t="n"/>
+      <c r="E67" s="36" t="n"/>
+      <c r="F67" s="37" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="35" t="inlineStr">
+        <is>
+          <t>מועמדים אפשריים מטבלת האביזרים (אותו אזור אנטומי):</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="38" t="inlineStr">
+        <is>
+          <t>גיליון</t>
+        </is>
+      </c>
+      <c r="B70" s="38" t="inlineStr">
+        <is>
+          <t>שורה</t>
+        </is>
+      </c>
+      <c r="C70" s="38" t="inlineStr">
+        <is>
+          <t>התוויה רפואית (טבלת המחירים)</t>
+        </is>
+      </c>
+      <c r="D70" s="38" t="inlineStr">
+        <is>
+          <t>עצמית / כללית / כולל</t>
+        </is>
+      </c>
+      <c r="E70" s="38" t="inlineStr">
+        <is>
+          <t>ליבואן ללא/כולל מע"מ</t>
+        </is>
+      </c>
+      <c r="F70" s="38" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B71" s="39" t="n">
+        <v>10</v>
+      </c>
+      <c r="C71" s="39" t="inlineStr">
+        <is>
+          <t>חגורת גב גמישה עם תמיכה + כרית (מעל 24 ס"מ)</t>
+        </is>
+      </c>
+      <c r="D71" s="39" t="inlineStr">
+        <is>
+          <t>63 / 146 / 209</t>
+        </is>
+      </c>
+      <c r="E71" s="39" t="inlineStr">
+        <is>
+          <t>135 / 159</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B72" s="39" t="n">
+        <v>11</v>
+      </c>
+      <c r="C72" s="39" t="inlineStr">
+        <is>
+          <t>חגורת גב גמישה עם תמיכה + כרית (מעל 24 ס"מ)</t>
+        </is>
+      </c>
+      <c r="D72" s="39" t="inlineStr">
+        <is>
+          <t>43 / 101 / 144</t>
+        </is>
+      </c>
+      <c r="E72" s="39" t="inlineStr">
+        <is>
+          <t>80 / 94</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B73" s="39" t="n">
+        <v>12</v>
+      </c>
+      <c r="C73" s="39" t="inlineStr">
+        <is>
+          <t>חגורת גב לשברים תואם JEWETT</t>
+        </is>
+      </c>
+      <c r="D73" s="39" t="inlineStr">
+        <is>
+          <t>174 / 407 / 581</t>
+        </is>
+      </c>
+      <c r="E73" s="39" t="inlineStr">
+        <is>
+          <t>450 / 531</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B74" s="39" t="n">
+        <v>13</v>
+      </c>
+      <c r="C74" s="39" t="inlineStr">
+        <is>
+          <t>חגורת גב לשברים תואם JEWETT</t>
+        </is>
+      </c>
+      <c r="D74" s="39" t="inlineStr">
+        <is>
+          <t>121 / 283 / 404</t>
+        </is>
+      </c>
+      <c r="E74" s="39" t="inlineStr">
+        <is>
+          <t>300 / 354</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B75" s="39" t="n">
+        <v>14</v>
+      </c>
+      <c r="C75" s="39" t="inlineStr">
+        <is>
+          <t>חגורת גב חיזוקים גמישים וסגירה כפולה (מעל 24 ס"מ)</t>
+        </is>
+      </c>
+      <c r="D75" s="39" t="inlineStr">
+        <is>
+          <t>37 / 87 / 124</t>
+        </is>
+      </c>
+      <c r="E75" s="39" t="inlineStr">
+        <is>
+          <t>63 / 74</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B76" s="39" t="n">
+        <v>15</v>
+      </c>
+      <c r="C76" s="39" t="inlineStr">
+        <is>
+          <t>חגורת גב חיזוקים גמישים וסגירה כפולה (מעל 24 ס"מ)</t>
+        </is>
+      </c>
+      <c r="D76" s="39" t="inlineStr">
+        <is>
+          <t>49 / 114 / 163</t>
+        </is>
+      </c>
+      <c r="E76" s="39" t="inlineStr">
+        <is>
+          <t>96 / 113</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B77" s="39" t="n">
+        <v>16</v>
+      </c>
+      <c r="C77" s="39" t="inlineStr">
+        <is>
+          <t>חגורת גב חיזוקים גמישים וסגירה כפולה (מעל 24 ס"מ)</t>
+        </is>
+      </c>
+      <c r="D77" s="39" t="inlineStr">
+        <is>
+          <t>36 / 82 / 118</t>
+        </is>
+      </c>
+      <c r="E77" s="39" t="inlineStr">
+        <is>
+          <t>58 / 68</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B78" s="39" t="n">
+        <v>17</v>
+      </c>
+      <c r="C78" s="39" t="inlineStr">
+        <is>
+          <t>חגורת גב עם תמיכה לנשים בהריון</t>
+        </is>
+      </c>
+      <c r="D78" s="39" t="inlineStr">
+        <is>
+          <t>31 / 72 / 103</t>
+        </is>
+      </c>
+      <c r="E78" s="39" t="inlineStr">
+        <is>
+          <t>45 / 53</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B79" s="39" t="n">
+        <v>18</v>
+      </c>
+      <c r="C79" s="39" t="inlineStr">
+        <is>
+          <t>צווארון מורכב מסוג PMT, פילדלפיה, VISTA, עם ריפוד</t>
+        </is>
+      </c>
+      <c r="D79" s="39" t="inlineStr">
+        <is>
+          <t>95 / 221 / 316</t>
+        </is>
+      </c>
+      <c r="E79" s="39" t="inlineStr">
+        <is>
+          <t>225 / 266</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B80" s="39" t="n">
+        <v>19</v>
+      </c>
+      <c r="C80" s="39" t="inlineStr">
+        <is>
+          <t>צווארון מורכב מסוג PMT, פילדלפיה, VISTA, ללא ריפוד</t>
+        </is>
+      </c>
+      <c r="D80" s="39" t="inlineStr">
+        <is>
+          <t>31 / 72 / 103</t>
+        </is>
+      </c>
+      <c r="E80" s="39" t="inlineStr">
+        <is>
+          <t>45 / 53</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B81" s="39" t="n">
+        <v>20</v>
+      </c>
+      <c r="C81" s="39" t="inlineStr">
+        <is>
+          <t>צווארון מורכב מסוג PMT, פילדלפיה, VISTA, ללא ריפוד</t>
+        </is>
+      </c>
+      <c r="D81" s="39" t="inlineStr">
+        <is>
+          <t>31 / 72 / 103</t>
+        </is>
+      </c>
+      <c r="E81" s="39" t="inlineStr">
+        <is>
+          <t>45 / 53</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="33" t="inlineStr">
+        <is>
+          <t>אזור אנטומי: ברך  (מקורות מחיר שנבדקו: ברך)</t>
+        </is>
+      </c>
+      <c r="B84" s="34" t="n"/>
+      <c r="C84" s="34" t="n"/>
+      <c r="D84" s="34" t="n"/>
+      <c r="E84" s="34" t="n"/>
+      <c r="F84" s="34" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="35" t="inlineStr">
+        <is>
+          <t>שורות במכרז שטרם מולאו:</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="22" t="inlineStr">
+        <is>
+          <t>שורה 35</t>
+        </is>
+      </c>
+      <c r="B86" s="22" t="inlineStr">
+        <is>
+          <t>מגן ברך ללא סיליקון</t>
+        </is>
+      </c>
+      <c r="C86" s="36" t="n"/>
+      <c r="D86" s="36" t="n"/>
+      <c r="E86" s="36" t="n"/>
+      <c r="F86" s="37" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="22" t="inlineStr">
+        <is>
+          <t>שורה 38</t>
+        </is>
+      </c>
+      <c r="B87" s="22" t="inlineStr">
+        <is>
+          <t>מייצב ברך ללא צירים - אימבולייזר</t>
+        </is>
+      </c>
+      <c r="C87" s="36" t="n"/>
+      <c r="D87" s="36" t="n"/>
+      <c r="E87" s="36" t="n"/>
+      <c r="F87" s="37" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="22" t="inlineStr">
+        <is>
+          <t>שורה 43</t>
+        </is>
+      </c>
+      <c r="B88" s="22" t="inlineStr">
+        <is>
+          <t>אימבלוייזר לתינוקות לברך</t>
+        </is>
+      </c>
+      <c r="C88" s="36" t="n"/>
+      <c r="D88" s="36" t="n"/>
+      <c r="E88" s="36" t="n"/>
+      <c r="F88" s="37" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="35" t="inlineStr">
+        <is>
+          <t>מועמדים אפשריים מטבלת האביזרים (אותו אזור אנטומי):</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="38" t="inlineStr">
+        <is>
+          <t>גיליון</t>
+        </is>
+      </c>
+      <c r="B91" s="38" t="inlineStr">
+        <is>
+          <t>שורה</t>
+        </is>
+      </c>
+      <c r="C91" s="38" t="inlineStr">
+        <is>
+          <t>התוויה רפואית (טבלת המחירים)</t>
+        </is>
+      </c>
+      <c r="D91" s="38" t="inlineStr">
+        <is>
+          <t>עצמית / כללית / כולל</t>
+        </is>
+      </c>
+      <c r="E91" s="38" t="inlineStr">
+        <is>
+          <t>ליבואן ללא/כולל מע"מ</t>
+        </is>
+      </c>
+      <c r="F91" s="38" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="39" t="inlineStr">
+        <is>
+          <t>דף 03</t>
+        </is>
+      </c>
+      <c r="B92" s="39" t="n">
+        <v>2</v>
+      </c>
+      <c r="C92" s="39" t="inlineStr">
+        <is>
+          <t>תומך ברך רך עם טבעת סיליקון לפיקה</t>
+        </is>
+      </c>
+      <c r="D92" s="39" t="inlineStr">
+        <is>
+          <t>44 / 103 / 147</t>
+        </is>
+      </c>
+      <c r="E92" s="39" t="inlineStr">
+        <is>
+          <t>83 / 97</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="39" t="inlineStr">
+        <is>
+          <t>דף 03</t>
+        </is>
+      </c>
+      <c r="B93" s="39" t="n">
+        <v>3</v>
+      </c>
+      <c r="C93" s="39" t="inlineStr">
+        <is>
+          <t>תומך ברך רך עם טבעת סיליקון לפיקה</t>
+        </is>
+      </c>
+      <c r="D93" s="39" t="inlineStr">
+        <is>
+          <t>45 / 104 / 149</t>
+        </is>
+      </c>
+      <c r="E93" s="39" t="inlineStr">
+        <is>
+          <t>84 / 99</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="39" t="inlineStr">
+        <is>
+          <t>דף 03</t>
+        </is>
+      </c>
+      <c r="B94" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="C94" s="39" t="inlineStr">
+        <is>
+          <t>תומך ברך רך עם טבעת סיליקון לפיקה</t>
+        </is>
+      </c>
+      <c r="D94" s="39" t="inlineStr">
+        <is>
+          <t>26 / 59 / 85</t>
+        </is>
+      </c>
+      <c r="E94" s="39" t="inlineStr">
+        <is>
+          <t>30 / 35</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="39" t="inlineStr">
+        <is>
+          <t>דף 03</t>
+        </is>
+      </c>
+      <c r="B95" s="39" t="n">
+        <v>5</v>
+      </c>
+      <c r="C95" s="39" t="inlineStr">
+        <is>
+          <t>תומך ברך ארוך עם טבעת סיליקון לפיקה ותומכי צד קשיחים (לפחות 15 ס"מ מעל ומתחת לברך)</t>
+        </is>
+      </c>
+      <c r="D95" s="39" t="inlineStr">
+        <is>
+          <t>54 / 126 / 180</t>
+        </is>
+      </c>
+      <c r="E95" s="39" t="inlineStr">
+        <is>
+          <t>110 / 130</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="39" t="inlineStr">
+        <is>
+          <t>דף 03</t>
+        </is>
+      </c>
+      <c r="B96" s="39" t="n">
+        <v>6</v>
+      </c>
+      <c r="C96" s="39" t="inlineStr">
+        <is>
+          <t>תומך ברך ארוך עם טבעת סיליקון לפיקה ותומכי צד קשיחים (לפחות 15 ס"מ מעל ומתחת לברך)</t>
+        </is>
+      </c>
+      <c r="D96" s="39" t="inlineStr">
+        <is>
+          <t>38 / 90 / 128</t>
+        </is>
+      </c>
+      <c r="E96" s="39" t="inlineStr">
+        <is>
+          <t>66 / 78</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="39" t="inlineStr">
+        <is>
+          <t>דף 03</t>
+        </is>
+      </c>
+      <c r="B97" s="39" t="n">
+        <v>7</v>
+      </c>
+      <c r="C97" s="39" t="inlineStr">
+        <is>
+          <t>מקבע ברך ארוך עם צירים מתכווננים POST OP</t>
+        </is>
+      </c>
+      <c r="D97" s="39" t="inlineStr">
+        <is>
+          <t>98 / 229 / 327</t>
+        </is>
+      </c>
+      <c r="E97" s="39" t="inlineStr">
+        <is>
+          <t>235 / 277</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="39" t="inlineStr">
+        <is>
+          <t>דף 03</t>
+        </is>
+      </c>
+      <c r="B98" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="C98" s="39" t="inlineStr">
+        <is>
+          <t>מקבע ברך ארוך עם צירים מתכווננים POST OP</t>
+        </is>
+      </c>
+      <c r="D98" s="39" t="inlineStr">
+        <is>
+          <t>104 / 241 / 345</t>
+        </is>
+      </c>
+      <c r="E98" s="39" t="inlineStr">
+        <is>
+          <t>250 / 295</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="39" t="inlineStr">
+        <is>
+          <t>דף 03</t>
+        </is>
+      </c>
+      <c r="B99" s="39" t="n">
+        <v>9</v>
+      </c>
+      <c r="C99" s="39" t="inlineStr">
+        <is>
+          <t>חבק תת פיקתי</t>
+        </is>
+      </c>
+      <c r="D99" s="39" t="inlineStr">
+        <is>
+          <t>23 / 53 / 76</t>
+        </is>
+      </c>
+      <c r="E99" s="39" t="inlineStr">
+        <is>
+          <t>22 / 26</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="39" t="inlineStr">
+        <is>
+          <t>דף 03</t>
+        </is>
+      </c>
+      <c r="B100" s="39" t="n">
+        <v>10</v>
+      </c>
+      <c r="C100" s="39" t="inlineStr">
+        <is>
+          <t>חבק תת פיקתי</t>
+        </is>
+      </c>
+      <c r="D100" s="39" t="inlineStr">
+        <is>
+          <t>24 / 56 / 80</t>
+        </is>
+      </c>
+      <c r="E100" s="39" t="inlineStr">
+        <is>
+          <t>26 / 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="39" t="inlineStr">
+        <is>
+          <t>דף 03</t>
+        </is>
+      </c>
+      <c r="B101" s="39" t="n">
+        <v>11</v>
+      </c>
+      <c r="C101" s="39" t="inlineStr">
+        <is>
+          <t>מייצב ברך ליציבות קדמית וצידית עם מסגרת מתכת קלה / קיבוע כולל ציר מתכוונן</t>
+        </is>
+      </c>
+      <c r="D101" s="39" t="inlineStr">
+        <is>
+          <t>134 / 311 / 445</t>
+        </is>
+      </c>
+      <c r="E101" s="39" t="inlineStr">
+        <is>
+          <t>335 / 395</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="39" t="inlineStr">
+        <is>
+          <t>דף 03</t>
+        </is>
+      </c>
+      <c r="B102" s="39" t="n">
+        <v>12</v>
+      </c>
+      <c r="C102" s="39" t="inlineStr">
+        <is>
+          <t>מייצב ברך לחוסר יציבות אחורית עם מסגרת מתכת קלה/קרבון ומערכת להחזרת הברך אחורית</t>
+        </is>
+      </c>
+      <c r="D102" s="39" t="inlineStr">
+        <is>
+          <t>134 / 311 / 445</t>
+        </is>
+      </c>
+      <c r="E102" s="39" t="inlineStr">
+        <is>
+          <t>335 / 395</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="39" t="inlineStr">
+        <is>
+          <t>דף 03</t>
+        </is>
+      </c>
+      <c r="B103" s="39" t="n">
+        <v>13</v>
+      </c>
+      <c r="C103" s="39" t="inlineStr">
+        <is>
+          <t>מייצב ברך לחוסר יציבות אחורית עם מסגרת מתכת קלה/קרבון ומערכת להחזרת הברך אחורית</t>
+        </is>
+      </c>
+      <c r="D103" s="39" t="inlineStr">
+        <is>
+          <t>185 / 433 / 618</t>
+        </is>
+      </c>
+      <c r="E103" s="39" t="inlineStr">
+        <is>
+          <t>481 / 568</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="39" t="inlineStr">
+        <is>
+          <t>דף 03</t>
+        </is>
+      </c>
+      <c r="B104" s="39" t="n">
+        <v>14</v>
+      </c>
+      <c r="C104" s="39" t="inlineStr">
+        <is>
+          <t>מייצב ברך ליציבות קדמית אחורית וצידית רך וגמיש עם ציר מתכוונן</t>
+        </is>
+      </c>
+      <c r="D104" s="39" t="inlineStr">
+        <is>
+          <t>240 / 559 / 799</t>
+        </is>
+      </c>
+      <c r="E104" s="39" t="inlineStr">
+        <is>
+          <t>635 / 749</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="39" t="inlineStr">
+        <is>
+          <t>דף 03</t>
+        </is>
+      </c>
+      <c r="B105" s="39" t="n">
+        <v>15</v>
+      </c>
+      <c r="C105" s="39" t="inlineStr">
+        <is>
+          <t>מייצב ברך ליציבות קדמית אחורית וצידית רך וגמיש עם ציר מתכוונן</t>
+        </is>
+      </c>
+      <c r="D105" s="39" t="inlineStr">
+        <is>
+          <t>249 / 580 / 829</t>
+        </is>
+      </c>
+      <c r="E105" s="39" t="inlineStr">
+        <is>
+          <t>660 / 779</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="39" t="inlineStr">
+        <is>
+          <t>דף 03</t>
+        </is>
+      </c>
+      <c r="B106" s="39" t="n">
+        <v>16</v>
+      </c>
+      <c r="C106" s="39" t="inlineStr">
+        <is>
+          <t>מייצב ברך ליציבות קדמית אחורית וצידית רך וגמיש עם ציר מתכוונן</t>
+        </is>
+      </c>
+      <c r="D106" s="39" t="inlineStr">
+        <is>
+          <t>97 / 226 / 323</t>
+        </is>
+      </c>
+      <c r="E106" s="39" t="inlineStr">
+        <is>
+          <t>231 / 273</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="33" t="inlineStr">
+        <is>
+          <t>אזור אנטומי: כף רגל  (מקורות מחיר שנבדקו: כף רגל)</t>
+        </is>
+      </c>
+      <c r="B109" s="34" t="n"/>
+      <c r="C109" s="34" t="n"/>
+      <c r="D109" s="34" t="n"/>
+      <c r="E109" s="34" t="n"/>
+      <c r="F109" s="34" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="35" t="inlineStr">
+        <is>
+          <t>שורות במכרז שטרם מולאו:</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="22" t="inlineStr">
+        <is>
+          <t>שורה 50</t>
+        </is>
+      </c>
+      <c r="B111" s="22" t="inlineStr">
+        <is>
+          <t>סד לתמיכה ב-FOOT DROP ובכף הרגל קשיח/ גמיש , סד פיני לשיקום</t>
+        </is>
+      </c>
+      <c r="C111" s="36" t="n"/>
+      <c r="D111" s="36" t="n"/>
+      <c r="E111" s="36" t="n"/>
+      <c r="F111" s="37" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="22" t="inlineStr">
+        <is>
+          <t>שורה 51</t>
+        </is>
+      </c>
+      <c r="B112" s="22" t="inlineStr">
+        <is>
+          <t>סד לתמיכה ב-FOOT DROP - תמיכת קרסול ברצועות/ קפיץ (תואם דיקטוס)</t>
+        </is>
+      </c>
+      <c r="C112" s="36" t="n"/>
+      <c r="D112" s="36" t="n"/>
+      <c r="E112" s="36" t="n"/>
+      <c r="F112" s="37" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="22" t="inlineStr">
+        <is>
+          <t>שורה 52</t>
+        </is>
+      </c>
+      <c r="B113" s="22" t="inlineStr">
+        <is>
+          <t>נעל גבס</t>
+        </is>
+      </c>
+      <c r="C113" s="36" t="n"/>
+      <c r="D113" s="36" t="n"/>
+      <c r="E113" s="36" t="n"/>
+      <c r="F113" s="37" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="22" t="inlineStr">
+        <is>
+          <t>שורה 53</t>
+        </is>
+      </c>
+      <c r="B114" s="22" t="inlineStr">
+        <is>
+          <t>נעלי אחרי ניתוח POST OP</t>
+        </is>
+      </c>
+      <c r="C114" s="36" t="n"/>
+      <c r="D114" s="36" t="n"/>
+      <c r="E114" s="36" t="n"/>
+      <c r="F114" s="37" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="22" t="inlineStr">
+        <is>
+          <t>שורה 54</t>
+        </is>
+      </c>
+      <c r="B115" s="22" t="inlineStr">
+        <is>
+          <t>נעל לאחר ניתוח/ לריפוי פצע עם הגבהה קדמית</t>
+        </is>
+      </c>
+      <c r="C115" s="36" t="n"/>
+      <c r="D115" s="36" t="n"/>
+      <c r="E115" s="36" t="n"/>
+      <c r="F115" s="37" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="22" t="inlineStr">
+        <is>
+          <t>שורה 55</t>
+        </is>
+      </c>
+      <c r="B116" s="22" t="inlineStr">
+        <is>
+          <t>נעל לאחר ניתוח/ לריפוי פצע עם הגבהה אחורית</t>
+        </is>
+      </c>
+      <c r="C116" s="36" t="n"/>
+      <c r="D116" s="36" t="n"/>
+      <c r="E116" s="36" t="n"/>
+      <c r="F116" s="37" t="n"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="22" t="inlineStr">
+        <is>
+          <t>שורה 57</t>
+        </is>
+      </c>
+      <c r="B117" s="22" t="inlineStr">
+        <is>
+          <t>עקב סיליקון בלי נקודה כחולה</t>
+        </is>
+      </c>
+      <c r="C117" s="36" t="n"/>
+      <c r="D117" s="36" t="n"/>
+      <c r="E117" s="36" t="n"/>
+      <c r="F117" s="37" t="n"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="22" t="inlineStr">
+        <is>
+          <t>שורה 59</t>
+        </is>
+      </c>
+      <c r="B118" s="22" t="inlineStr">
+        <is>
+          <t>סד הלוקס ואלגוס</t>
+        </is>
+      </c>
+      <c r="C118" s="36" t="n"/>
+      <c r="D118" s="36" t="n"/>
+      <c r="E118" s="36" t="n"/>
+      <c r="F118" s="37" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="22" t="inlineStr">
+        <is>
+          <t>שורה 60</t>
+        </is>
+      </c>
+      <c r="B119" s="22" t="inlineStr">
+        <is>
+          <t>מדרס סיליקון מוכן עם נקודות מחוברות</t>
+        </is>
+      </c>
+      <c r="C119" s="36" t="n"/>
+      <c r="D119" s="36" t="n"/>
+      <c r="E119" s="36" t="n"/>
+      <c r="F119" s="37" t="n"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="22" t="inlineStr">
+        <is>
+          <t>שורה 61</t>
+        </is>
+      </c>
+      <c r="B120" s="22" t="inlineStr">
+        <is>
+          <t>מדרסי ג'ל</t>
+        </is>
+      </c>
+      <c r="C120" s="36" t="n"/>
+      <c r="D120" s="36" t="n"/>
+      <c r="E120" s="36" t="n"/>
+      <c r="F120" s="37" t="n"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="22" t="inlineStr">
+        <is>
+          <t>שורה 62</t>
+        </is>
+      </c>
+      <c r="B121" s="22" t="inlineStr">
+        <is>
+          <t>סד לילה לפסאיטיס- פלנטרית בכף הרגל</t>
+        </is>
+      </c>
+      <c r="C121" s="36" t="n"/>
+      <c r="D121" s="36" t="n"/>
+      <c r="E121" s="36" t="n"/>
+      <c r="F121" s="37" t="n"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="22" t="inlineStr">
+        <is>
+          <t>שורה 63</t>
+        </is>
+      </c>
+      <c r="B122" s="22" t="inlineStr">
+        <is>
+          <t>מדרס בהתאמה אישית</t>
+        </is>
+      </c>
+      <c r="C122" s="36" t="n"/>
+      <c r="D122" s="36" t="n"/>
+      <c r="E122" s="36" t="n"/>
+      <c r="F122" s="37" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="22" t="inlineStr">
+        <is>
+          <t>שורה 64</t>
+        </is>
+      </c>
+      <c r="B123" s="22" t="inlineStr">
+        <is>
+          <t>מדרסים מיוחדים - ביו מכני - מדרסים לסכרתיים - עיוות רגל</t>
+        </is>
+      </c>
+      <c r="C123" s="36" t="n"/>
+      <c r="D123" s="36" t="n"/>
+      <c r="E123" s="36" t="n"/>
+      <c r="F123" s="37" t="n"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="35" t="inlineStr">
+        <is>
+          <t>מועמדים אפשריים מטבלת האביזרים (אותו אזור אנטומי):</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="38" t="inlineStr">
+        <is>
+          <t>גיליון</t>
+        </is>
+      </c>
+      <c r="B126" s="38" t="inlineStr">
+        <is>
+          <t>שורה</t>
+        </is>
+      </c>
+      <c r="C126" s="38" t="inlineStr">
+        <is>
+          <t>התוויה רפואית (טבלת המחירים)</t>
+        </is>
+      </c>
+      <c r="D126" s="38" t="inlineStr">
+        <is>
+          <t>עצמית / כללית / כולל</t>
+        </is>
+      </c>
+      <c r="E126" s="38" t="inlineStr">
+        <is>
+          <t>ליבואן ללא/כולל מע"מ</t>
+        </is>
+      </c>
+      <c r="F126" s="38" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="39" t="inlineStr">
+        <is>
+          <t>דף 01</t>
+        </is>
+      </c>
+      <c r="B127" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="C127" s="39" t="inlineStr">
+        <is>
+          <t>סד לתמיכה ב DROP FOOT</t>
+        </is>
+      </c>
+      <c r="D127" s="39" t="inlineStr">
+        <is>
+          <t>38 / 89 / 127</t>
+        </is>
+      </c>
+      <c r="E127" s="39" t="inlineStr">
+        <is>
+          <t>65 / 77</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="39" t="inlineStr">
+        <is>
+          <t>דף 01</t>
+        </is>
+      </c>
+      <c r="B128" s="39" t="n">
+        <v>9</v>
+      </c>
+      <c r="C128" s="39" t="inlineStr">
+        <is>
+          <t>תבנית לסד לתמיכה ב DROP FOOT</t>
+        </is>
+      </c>
+      <c r="D128" s="39" t="inlineStr">
+        <is>
+          <t>43 / 101 / 144</t>
+        </is>
+      </c>
+      <c r="E128" s="39" t="inlineStr">
+        <is>
+          <t>80 / 94</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="39" t="inlineStr">
+        <is>
+          <t>דף 01</t>
+        </is>
+      </c>
+      <c r="B129" s="39" t="n">
+        <v>10</v>
+      </c>
+      <c r="C129" s="39" t="inlineStr">
+        <is>
+          <t>סד לתמיכה ב DROP FOOT - תמיכת קרסול קשיח</t>
+        </is>
+      </c>
+      <c r="D129" s="39" t="inlineStr">
+        <is>
+          <t>61 / 142 / 203</t>
+        </is>
+      </c>
+      <c r="E129" s="39" t="inlineStr">
+        <is>
+          <t>130 / 153</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="39" t="inlineStr">
+        <is>
+          <t>דף 01</t>
+        </is>
+      </c>
+      <c r="B130" s="39" t="n">
+        <v>11</v>
+      </c>
+      <c r="C130" s="39" t="inlineStr">
+        <is>
+          <t>סד לתמיכה ב DROP FOOT - תמיכת קרסול קשיח ומרופד</t>
+        </is>
+      </c>
+      <c r="D130" s="39" t="inlineStr">
+        <is>
+          <t>66 / 155 / 221</t>
+        </is>
+      </c>
+      <c r="E130" s="39" t="inlineStr">
+        <is>
+          <t>145 / 171</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="39" t="inlineStr">
+        <is>
+          <t>דף 01</t>
+        </is>
+      </c>
+      <c r="B131" s="39" t="n">
+        <v>12</v>
+      </c>
+      <c r="C131" s="39" t="inlineStr">
+        <is>
+          <t>דמוי נעל - off-loading device</t>
+        </is>
+      </c>
+      <c r="D131" s="39" t="inlineStr">
+        <is>
+          <t>27 / 64 / 91</t>
+        </is>
+      </c>
+      <c r="E131" s="39" t="inlineStr">
+        <is>
+          <t>35 / 41</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="39" t="inlineStr">
+        <is>
+          <t>דף 01</t>
+        </is>
+      </c>
+      <c r="B132" s="39" t="n">
+        <v>13</v>
+      </c>
+      <c r="C132" s="39" t="inlineStr">
+        <is>
+          <t>דמוי נעל - off-loading device</t>
+        </is>
+      </c>
+      <c r="D132" s="39" t="inlineStr">
+        <is>
+          <t>29 / 68 / 97</t>
+        </is>
+      </c>
+      <c r="E132" s="39" t="inlineStr">
+        <is>
+          <t>40 / 47</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="39" t="inlineStr">
+        <is>
+          <t>דף 01</t>
+        </is>
+      </c>
+      <c r="B133" s="39" t="n">
+        <v>14</v>
+      </c>
+      <c r="C133" s="39" t="inlineStr">
+        <is>
+          <t>נעלי ציר עד ג' שנים</t>
+        </is>
+      </c>
+      <c r="D133" s="39" t="inlineStr">
+        <is>
+          <t>298 / 696 / 994</t>
+        </is>
+      </c>
+      <c r="E133" s="39" t="inlineStr">
+        <is>
+          <t>800 / 944</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="39" t="inlineStr">
+        <is>
+          <t>דף 01</t>
+        </is>
+      </c>
+      <c r="B134" s="39" t="n">
+        <v>15</v>
+      </c>
+      <c r="C134" s="39" t="inlineStr">
+        <is>
+          <t>עקב סיליקון לדורבן</t>
+        </is>
+      </c>
+      <c r="D134" s="39" t="inlineStr">
+        <is>
+          <t>24 / 56 / 80</t>
+        </is>
+      </c>
+      <c r="E134" s="39" t="inlineStr">
+        <is>
+          <t>25 / 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="39" t="inlineStr">
+        <is>
+          <t>דף 01</t>
+        </is>
+      </c>
+      <c r="B135" s="39" t="n">
+        <v>16</v>
+      </c>
+      <c r="C135" s="39" t="inlineStr">
+        <is>
+          <t>עקב סיליקון לדורבן</t>
+        </is>
+      </c>
+      <c r="D135" s="39" t="inlineStr">
+        <is>
+          <t>25 / 57 / 82</t>
+        </is>
+      </c>
+      <c r="E135" s="39" t="inlineStr">
+        <is>
+          <t>27 / 32</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="33" t="inlineStr">
+        <is>
+          <t>אזור אנטומי: ירכיים  (מקורות מחיר שנבדקו: ירכיים)</t>
+        </is>
+      </c>
+      <c r="B138" s="34" t="n"/>
+      <c r="C138" s="34" t="n"/>
+      <c r="D138" s="34" t="n"/>
+      <c r="E138" s="34" t="n"/>
+      <c r="F138" s="34" t="n"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="35" t="inlineStr">
+        <is>
+          <t>שורות במכרז שטרם מולאו:</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="22" t="inlineStr">
+        <is>
+          <t>שורה 65</t>
+        </is>
+      </c>
+      <c r="B140" s="22" t="inlineStr">
+        <is>
+          <t>מגני ירכיים עם ריפוד / כרית מתנפחת למניעת שבר צוואר ירך</t>
+        </is>
+      </c>
+      <c r="C140" s="36" t="n"/>
+      <c r="D140" s="36" t="n"/>
+      <c r="E140" s="36" t="n"/>
+      <c r="F140" s="37" t="n"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="35" t="inlineStr">
+        <is>
+          <t>מועמדים אפשריים מטבלת האביזרים (אותו אזור אנטומי):</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="38" t="inlineStr">
+        <is>
+          <t>גיליון</t>
+        </is>
+      </c>
+      <c r="B143" s="38" t="inlineStr">
+        <is>
+          <t>שורה</t>
+        </is>
+      </c>
+      <c r="C143" s="38" t="inlineStr">
+        <is>
+          <t>התוויה רפואית (טבלת המחירים)</t>
+        </is>
+      </c>
+      <c r="D143" s="38" t="inlineStr">
+        <is>
+          <t>עצמית / כללית / כולל</t>
+        </is>
+      </c>
+      <c r="E143" s="38" t="inlineStr">
+        <is>
+          <t>ליבואן ללא/כולל מע"מ</t>
+        </is>
+      </c>
+      <c r="F143" s="38" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="39" t="inlineStr">
+        <is>
+          <t>דף 01</t>
+        </is>
+      </c>
+      <c r="B144" s="39" t="n">
+        <v>27</v>
+      </c>
+      <c r="C144" s="39" t="inlineStr">
+        <is>
+          <t>מגן ירכיים עם ריפוד / כרית</t>
+        </is>
+      </c>
+      <c r="D144" s="39" t="inlineStr">
+        <is>
+          <t>44 / 103 / 147</t>
+        </is>
+      </c>
+      <c r="E144" s="39" t="inlineStr">
+        <is>
+          <t>83 / 97</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="39" t="inlineStr">
+        <is>
+          <t>דף 01</t>
+        </is>
+      </c>
+      <c r="B145" s="39" t="n">
+        <v>28</v>
+      </c>
+      <c r="C145" s="39" t="inlineStr">
+        <is>
+          <t>מתנפחות למניעת שבר צוואר ירך</t>
+        </is>
+      </c>
+      <c r="D145" s="39" t="inlineStr">
+        <is>
+          <t>49 / 113 / 162</t>
+        </is>
+      </c>
+      <c r="E145" s="39" t="inlineStr">
+        <is>
+          <t>95 / 112</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="33" t="inlineStr">
+        <is>
+          <t>אזור אנטומי: בטן  (מקורות מחיר שנבדקו: חגורת בטן)</t>
+        </is>
+      </c>
+      <c r="B148" s="34" t="n"/>
+      <c r="C148" s="34" t="n"/>
+      <c r="D148" s="34" t="n"/>
+      <c r="E148" s="34" t="n"/>
+      <c r="F148" s="34" t="n"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="35" t="inlineStr">
+        <is>
+          <t>שורות במכרז שטרם מולאו:</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="22" t="inlineStr">
+        <is>
+          <t>שורה 75</t>
+        </is>
+      </c>
+      <c r="B150" s="22" t="inlineStr">
+        <is>
+          <t>חגורת גב לאחר ניתוח בטן / חזה</t>
+        </is>
+      </c>
+      <c r="C150" s="36" t="n"/>
+      <c r="D150" s="36" t="n"/>
+      <c r="E150" s="36" t="n"/>
+      <c r="F150" s="37" t="n"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="22" t="inlineStr">
+        <is>
+          <t>שורה 76</t>
+        </is>
+      </c>
+      <c r="B151" s="22" t="inlineStr">
+        <is>
+          <t>חגורת בטן לאחר ניתוח חזה / בטן</t>
+        </is>
+      </c>
+      <c r="C151" s="36" t="n"/>
+      <c r="D151" s="36" t="n"/>
+      <c r="E151" s="36" t="n"/>
+      <c r="F151" s="37" t="n"/>
+    </row>
+    <row r="153">
+      <c r="A153" s="35" t="inlineStr">
+        <is>
+          <t>מועמדים אפשריים מטבלת האביזרים (אותו אזור אנטומי):</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="38" t="inlineStr">
+        <is>
+          <t>גיליון</t>
+        </is>
+      </c>
+      <c r="B154" s="38" t="inlineStr">
+        <is>
+          <t>שורה</t>
+        </is>
+      </c>
+      <c r="C154" s="38" t="inlineStr">
+        <is>
+          <t>התוויה רפואית (טבלת המחירים)</t>
+        </is>
+      </c>
+      <c r="D154" s="38" t="inlineStr">
+        <is>
+          <t>עצמית / כללית / כולל</t>
+        </is>
+      </c>
+      <c r="E154" s="38" t="inlineStr">
+        <is>
+          <t>ליבואן ללא/כולל מע"מ</t>
+        </is>
+      </c>
+      <c r="F154" s="38" t="inlineStr"/>
+    </row>
+    <row r="155">
+      <c r="A155" s="39" t="inlineStr">
+        <is>
+          <t>דף 01</t>
+        </is>
+      </c>
+      <c r="B155" s="39" t="n">
+        <v>26</v>
+      </c>
+      <c r="C155" s="39" t="inlineStr">
+        <is>
+          <t>חגורת בטן סטומה (מדף)</t>
+        </is>
+      </c>
+      <c r="D155" s="39" t="inlineStr">
+        <is>
+          <t>104 / 241 / 345</t>
+        </is>
+      </c>
+      <c r="E155" s="39" t="inlineStr">
+        <is>
+          <t>250 / 295</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="33" t="inlineStr">
+        <is>
+          <t>אזור אנטומי: מותניים  (מקורות מחיר שנבדקו: גב)</t>
+        </is>
+      </c>
+      <c r="B158" s="34" t="n"/>
+      <c r="C158" s="34" t="n"/>
+      <c r="D158" s="34" t="n"/>
+      <c r="E158" s="34" t="n"/>
+      <c r="F158" s="34" t="n"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="35" t="inlineStr">
+        <is>
+          <t>שורות במכרז שטרם מולאו:</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="22" t="inlineStr">
+        <is>
+          <t>שורה 77</t>
+        </is>
+      </c>
+      <c r="B160" s="22" t="inlineStr">
+        <is>
+          <t>סד למניעת פריקה התפתחותית במפרק הירכיים DDH</t>
+        </is>
+      </c>
+      <c r="C160" s="36" t="n"/>
+      <c r="D160" s="36" t="n"/>
+      <c r="E160" s="36" t="n"/>
+      <c r="F160" s="37" t="n"/>
+    </row>
+    <row r="162">
+      <c r="A162" s="35" t="inlineStr">
+        <is>
+          <t>מועמדים אפשריים מטבלת האביזרים (אותו אזור אנטומי):</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="38" t="inlineStr">
+        <is>
+          <t>גיליון</t>
+        </is>
+      </c>
+      <c r="B163" s="38" t="inlineStr">
+        <is>
+          <t>שורה</t>
+        </is>
+      </c>
+      <c r="C163" s="38" t="inlineStr">
+        <is>
+          <t>התוויה רפואית (טבלת המחירים)</t>
+        </is>
+      </c>
+      <c r="D163" s="38" t="inlineStr">
+        <is>
+          <t>עצמית / כללית / כולל</t>
+        </is>
+      </c>
+      <c r="E163" s="38" t="inlineStr">
+        <is>
+          <t>ליבואן ללא/כולל מע"מ</t>
+        </is>
+      </c>
+      <c r="F163" s="38" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="A164" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B164" s="39" t="n">
+        <v>10</v>
+      </c>
+      <c r="C164" s="39" t="inlineStr">
+        <is>
+          <t>חגורת גב גמישה עם תמיכה + כרית (מעל 24 ס"מ)</t>
+        </is>
+      </c>
+      <c r="D164" s="39" t="inlineStr">
+        <is>
+          <t>63 / 146 / 209</t>
+        </is>
+      </c>
+      <c r="E164" s="39" t="inlineStr">
+        <is>
+          <t>135 / 159</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B165" s="39" t="n">
+        <v>11</v>
+      </c>
+      <c r="C165" s="39" t="inlineStr">
+        <is>
+          <t>חגורת גב גמישה עם תמיכה + כרית (מעל 24 ס"מ)</t>
+        </is>
+      </c>
+      <c r="D165" s="39" t="inlineStr">
+        <is>
+          <t>43 / 101 / 144</t>
+        </is>
+      </c>
+      <c r="E165" s="39" t="inlineStr">
+        <is>
+          <t>80 / 94</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B166" s="39" t="n">
+        <v>12</v>
+      </c>
+      <c r="C166" s="39" t="inlineStr">
+        <is>
+          <t>חגורת גב לשברים תואם JEWETT</t>
+        </is>
+      </c>
+      <c r="D166" s="39" t="inlineStr">
+        <is>
+          <t>174 / 407 / 581</t>
+        </is>
+      </c>
+      <c r="E166" s="39" t="inlineStr">
+        <is>
+          <t>450 / 531</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B167" s="39" t="n">
+        <v>13</v>
+      </c>
+      <c r="C167" s="39" t="inlineStr">
+        <is>
+          <t>חגורת גב לשברים תואם JEWETT</t>
+        </is>
+      </c>
+      <c r="D167" s="39" t="inlineStr">
+        <is>
+          <t>121 / 283 / 404</t>
+        </is>
+      </c>
+      <c r="E167" s="39" t="inlineStr">
+        <is>
+          <t>300 / 354</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B168" s="39" t="n">
+        <v>14</v>
+      </c>
+      <c r="C168" s="39" t="inlineStr">
+        <is>
+          <t>חגורת גב חיזוקים גמישים וסגירה כפולה (מעל 24 ס"מ)</t>
+        </is>
+      </c>
+      <c r="D168" s="39" t="inlineStr">
+        <is>
+          <t>37 / 87 / 124</t>
+        </is>
+      </c>
+      <c r="E168" s="39" t="inlineStr">
+        <is>
+          <t>63 / 74</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B169" s="39" t="n">
+        <v>15</v>
+      </c>
+      <c r="C169" s="39" t="inlineStr">
+        <is>
+          <t>חגורת גב חיזוקים גמישים וסגירה כפולה (מעל 24 ס"מ)</t>
+        </is>
+      </c>
+      <c r="D169" s="39" t="inlineStr">
+        <is>
+          <t>49 / 114 / 163</t>
+        </is>
+      </c>
+      <c r="E169" s="39" t="inlineStr">
+        <is>
+          <t>96 / 113</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B170" s="39" t="n">
+        <v>16</v>
+      </c>
+      <c r="C170" s="39" t="inlineStr">
+        <is>
+          <t>חגורת גב חיזוקים גמישים וסגירה כפולה (מעל 24 ס"מ)</t>
+        </is>
+      </c>
+      <c r="D170" s="39" t="inlineStr">
+        <is>
+          <t>36 / 82 / 118</t>
+        </is>
+      </c>
+      <c r="E170" s="39" t="inlineStr">
+        <is>
+          <t>58 / 68</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B171" s="39" t="n">
+        <v>17</v>
+      </c>
+      <c r="C171" s="39" t="inlineStr">
+        <is>
+          <t>חגורת גב עם תמיכה לנשים בהריון</t>
+        </is>
+      </c>
+      <c r="D171" s="39" t="inlineStr">
+        <is>
+          <t>31 / 72 / 103</t>
+        </is>
+      </c>
+      <c r="E171" s="39" t="inlineStr">
+        <is>
+          <t>45 / 53</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="33" t="inlineStr">
+        <is>
+          <t>אזור אנטומי: אגן  (מקורות מחיר שנבדקו: חגורת בטן, גב)</t>
+        </is>
+      </c>
+      <c r="B174" s="34" t="n"/>
+      <c r="C174" s="34" t="n"/>
+      <c r="D174" s="34" t="n"/>
+      <c r="E174" s="34" t="n"/>
+      <c r="F174" s="34" t="n"/>
+    </row>
+    <row r="175">
+      <c r="A175" s="35" t="inlineStr">
+        <is>
+          <t>שורות במכרז שטרם מולאו:</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="22" t="inlineStr">
+        <is>
+          <t>שורה 78</t>
+        </is>
+      </c>
+      <c r="B176" s="22" t="inlineStr">
+        <is>
+          <t>חגורת אגן ( אורט' - חגורת היריון)</t>
+        </is>
+      </c>
+      <c r="C176" s="36" t="n"/>
+      <c r="D176" s="36" t="n"/>
+      <c r="E176" s="36" t="n"/>
+      <c r="F176" s="37" t="n"/>
+    </row>
+    <row r="178">
+      <c r="A178" s="35" t="inlineStr">
+        <is>
+          <t>מועמדים אפשריים מטבלת האביזרים (אותו אזור אנטומי):</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="38" t="inlineStr">
+        <is>
+          <t>גיליון</t>
+        </is>
+      </c>
+      <c r="B179" s="38" t="inlineStr">
+        <is>
+          <t>שורה</t>
+        </is>
+      </c>
+      <c r="C179" s="38" t="inlineStr">
+        <is>
+          <t>התוויה רפואית (טבלת המחירים)</t>
+        </is>
+      </c>
+      <c r="D179" s="38" t="inlineStr">
+        <is>
+          <t>עצמית / כללית / כולל</t>
+        </is>
+      </c>
+      <c r="E179" s="38" t="inlineStr">
+        <is>
+          <t>ליבואן ללא/כולל מע"מ</t>
+        </is>
+      </c>
+      <c r="F179" s="38" t="inlineStr"/>
+    </row>
+    <row r="180">
+      <c r="A180" s="39" t="inlineStr">
+        <is>
+          <t>דף 01</t>
+        </is>
+      </c>
+      <c r="B180" s="39" t="n">
+        <v>26</v>
+      </c>
+      <c r="C180" s="39" t="inlineStr">
+        <is>
+          <t>חגורת בטן סטומה (מדף)</t>
+        </is>
+      </c>
+      <c r="D180" s="39" t="inlineStr">
+        <is>
+          <t>104 / 241 / 345</t>
+        </is>
+      </c>
+      <c r="E180" s="39" t="inlineStr">
+        <is>
+          <t>250 / 295</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B181" s="39" t="n">
+        <v>10</v>
+      </c>
+      <c r="C181" s="39" t="inlineStr">
+        <is>
+          <t>חגורת גב גמישה עם תמיכה + כרית (מעל 24 ס"מ)</t>
+        </is>
+      </c>
+      <c r="D181" s="39" t="inlineStr">
+        <is>
+          <t>63 / 146 / 209</t>
+        </is>
+      </c>
+      <c r="E181" s="39" t="inlineStr">
+        <is>
+          <t>135 / 159</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B182" s="39" t="n">
+        <v>11</v>
+      </c>
+      <c r="C182" s="39" t="inlineStr">
+        <is>
+          <t>חגורת גב גמישה עם תמיכה + כרית (מעל 24 ס"מ)</t>
+        </is>
+      </c>
+      <c r="D182" s="39" t="inlineStr">
+        <is>
+          <t>43 / 101 / 144</t>
+        </is>
+      </c>
+      <c r="E182" s="39" t="inlineStr">
+        <is>
+          <t>80 / 94</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B183" s="39" t="n">
+        <v>12</v>
+      </c>
+      <c r="C183" s="39" t="inlineStr">
+        <is>
+          <t>חגורת גב לשברים תואם JEWETT</t>
+        </is>
+      </c>
+      <c r="D183" s="39" t="inlineStr">
+        <is>
+          <t>174 / 407 / 581</t>
+        </is>
+      </c>
+      <c r="E183" s="39" t="inlineStr">
+        <is>
+          <t>450 / 531</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B184" s="39" t="n">
+        <v>13</v>
+      </c>
+      <c r="C184" s="39" t="inlineStr">
+        <is>
+          <t>חגורת גב לשברים תואם JEWETT</t>
+        </is>
+      </c>
+      <c r="D184" s="39" t="inlineStr">
+        <is>
+          <t>121 / 283 / 404</t>
+        </is>
+      </c>
+      <c r="E184" s="39" t="inlineStr">
+        <is>
+          <t>300 / 354</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B185" s="39" t="n">
+        <v>14</v>
+      </c>
+      <c r="C185" s="39" t="inlineStr">
+        <is>
+          <t>חגורת גב חיזוקים גמישים וסגירה כפולה (מעל 24 ס"מ)</t>
+        </is>
+      </c>
+      <c r="D185" s="39" t="inlineStr">
+        <is>
+          <t>37 / 87 / 124</t>
+        </is>
+      </c>
+      <c r="E185" s="39" t="inlineStr">
+        <is>
+          <t>63 / 74</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B186" s="39" t="n">
+        <v>15</v>
+      </c>
+      <c r="C186" s="39" t="inlineStr">
+        <is>
+          <t>חגורת גב חיזוקים גמישים וסגירה כפולה (מעל 24 ס"מ)</t>
+        </is>
+      </c>
+      <c r="D186" s="39" t="inlineStr">
+        <is>
+          <t>49 / 114 / 163</t>
+        </is>
+      </c>
+      <c r="E186" s="39" t="inlineStr">
+        <is>
+          <t>96 / 113</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B187" s="39" t="n">
+        <v>16</v>
+      </c>
+      <c r="C187" s="39" t="inlineStr">
+        <is>
+          <t>חגורת גב חיזוקים גמישים וסגירה כפולה (מעל 24 ס"מ)</t>
+        </is>
+      </c>
+      <c r="D187" s="39" t="inlineStr">
+        <is>
+          <t>36 / 82 / 118</t>
+        </is>
+      </c>
+      <c r="E187" s="39" t="inlineStr">
+        <is>
+          <t>58 / 68</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="39" t="inlineStr">
+        <is>
+          <t>דף 02</t>
+        </is>
+      </c>
+      <c r="B188" s="39" t="n">
+        <v>17</v>
+      </c>
+      <c r="C188" s="39" t="inlineStr">
+        <is>
+          <t>חגורת גב עם תמיכה לנשים בהריון</t>
+        </is>
+      </c>
+      <c r="D188" s="39" t="inlineStr">
+        <is>
+          <t>31 / 72 / 103</t>
+        </is>
+      </c>
+      <c r="E188" s="39" t="inlineStr">
+        <is>
+          <t>45 / 53</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="33" t="inlineStr">
+        <is>
+          <t>אזור אנטומי: חזה  (מקורות מחיר שנבדקו: חגורת שבר, חגורת בטן)</t>
+        </is>
+      </c>
+      <c r="B191" s="34" t="n"/>
+      <c r="C191" s="34" t="n"/>
+      <c r="D191" s="34" t="n"/>
+      <c r="E191" s="34" t="n"/>
+      <c r="F191" s="34" t="n"/>
+    </row>
+    <row r="192">
+      <c r="A192" s="35" t="inlineStr">
+        <is>
+          <t>שורות במכרז שטרם מולאו:</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="22" t="inlineStr">
+        <is>
+          <t>שורה 79</t>
+        </is>
+      </c>
+      <c r="B193" s="22" t="inlineStr">
+        <is>
+          <t>חגורת חזה / שבר צלעות</t>
+        </is>
+      </c>
+      <c r="C193" s="36" t="n"/>
+      <c r="D193" s="36" t="n"/>
+      <c r="E193" s="36" t="n"/>
+      <c r="F193" s="37" t="n"/>
+    </row>
+    <row r="195">
+      <c r="A195" s="35" t="inlineStr">
+        <is>
+          <t>מועמדים אפשריים מטבלת האביזרים (אותו אזור אנטומי):</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="38" t="inlineStr">
+        <is>
+          <t>גיליון</t>
+        </is>
+      </c>
+      <c r="B196" s="38" t="inlineStr">
+        <is>
+          <t>שורה</t>
+        </is>
+      </c>
+      <c r="C196" s="38" t="inlineStr">
+        <is>
+          <t>התוויה רפואית (טבלת המחירים)</t>
+        </is>
+      </c>
+      <c r="D196" s="38" t="inlineStr">
+        <is>
+          <t>עצמית / כללית / כולל</t>
+        </is>
+      </c>
+      <c r="E196" s="38" t="inlineStr">
+        <is>
+          <t>ליבואן ללא/כולל מע"מ</t>
+        </is>
+      </c>
+      <c r="F196" s="38" t="inlineStr"/>
+    </row>
+    <row r="197">
+      <c r="A197" s="39" t="inlineStr">
+        <is>
+          <t>דף 01</t>
+        </is>
+      </c>
+      <c r="B197" s="39" t="n">
+        <v>24</v>
+      </c>
+      <c r="C197" s="39" t="inlineStr">
+        <is>
+          <t>חגורת שבר הבקע חד צדדית</t>
+        </is>
+      </c>
+      <c r="D197" s="39" t="inlineStr">
+        <is>
+          <t>96 / 225 / 321</t>
+        </is>
+      </c>
+      <c r="E197" s="39" t="inlineStr">
+        <is>
+          <t>230 / 271</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="39" t="inlineStr">
+        <is>
+          <t>דף 01</t>
+        </is>
+      </c>
+      <c r="B198" s="39" t="n">
+        <v>25</v>
+      </c>
+      <c r="C198" s="39" t="inlineStr">
+        <is>
+          <t>חגורת שבר הרניה דו"צ</t>
+        </is>
+      </c>
+      <c r="D198" s="39" t="inlineStr">
+        <is>
+          <t>69 / 160 / 229</t>
+        </is>
+      </c>
+      <c r="E198" s="39" t="inlineStr">
+        <is>
+          <t>152 / 179</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="39" t="inlineStr">
+        <is>
+          <t>דף 01</t>
+        </is>
+      </c>
+      <c r="B199" s="39" t="n">
+        <v>26</v>
+      </c>
+      <c r="C199" s="39" t="inlineStr">
+        <is>
+          <t>חגורת בטן סטומה (מדף)</t>
+        </is>
+      </c>
+      <c r="D199" s="39" t="inlineStr">
+        <is>
+          <t>104 / 241 / 345</t>
+        </is>
+      </c>
+      <c r="E199" s="39" t="inlineStr">
+        <is>
+          <t>250 / 295</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="35">
+    <mergeCell ref="B113:F113"/>
+    <mergeCell ref="B7:F7"/>
+    <mergeCell ref="B25:F25"/>
+    <mergeCell ref="B193:F193"/>
+    <mergeCell ref="B66:F66"/>
+    <mergeCell ref="B150:F150"/>
+    <mergeCell ref="B121:F121"/>
+    <mergeCell ref="B122:F122"/>
+    <mergeCell ref="B115:F115"/>
+    <mergeCell ref="B140:F140"/>
+    <mergeCell ref="B27:F27"/>
+    <mergeCell ref="B43:F43"/>
+    <mergeCell ref="B176:F176"/>
+    <mergeCell ref="B86:F86"/>
+    <mergeCell ref="B117:F117"/>
+    <mergeCell ref="B111:F111"/>
+    <mergeCell ref="B151:F151"/>
+    <mergeCell ref="B120:F120"/>
+    <mergeCell ref="B67:F67"/>
+    <mergeCell ref="B119:F119"/>
+    <mergeCell ref="B88:F88"/>
+    <mergeCell ref="B44:F44"/>
+    <mergeCell ref="B87:F87"/>
+    <mergeCell ref="B116:F116"/>
+    <mergeCell ref="B112:F112"/>
+    <mergeCell ref="B118:F118"/>
+    <mergeCell ref="B65:F65"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="B64:F64"/>
+    <mergeCell ref="B114:F114"/>
+    <mergeCell ref="B45:F45"/>
+    <mergeCell ref="B63:F63"/>
+    <mergeCell ref="B123:F123"/>
+    <mergeCell ref="B160:F160"/>
+    <mergeCell ref="B26:F26"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Fill row 78 (pregnancy belt match), document reasoning for remaining 34 rows
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E9QvuhBZminJvrtKVH8YY8
</commit_message>
<xml_diff>
--- a/kirill/outputs/2026-09-03-קופח-מכרזים-מולא-מטבלאות-אביזרים.xlsx
+++ b/kirill/outputs/2026-09-03-קופח-מכרזים-מולא-מטבלאות-אביזרים.xlsx
@@ -111,7 +111,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -162,6 +162,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF9E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
   </fills>
@@ -250,7 +260,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -323,6 +333,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="9" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="10" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3665,6 +3681,21 @@
           <t>קיים במגוון</t>
         </is>
       </c>
+      <c r="M78" t="n">
+        <v>31</v>
+      </c>
+      <c r="N78" t="n">
+        <v>72</v>
+      </c>
+      <c r="O78" t="n">
+        <v>103</v>
+      </c>
+      <c r="P78" t="n">
+        <v>45</v>
+      </c>
+      <c r="Q78" t="n">
+        <v>53</v>
+      </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="10">
       <c r="A79" s="15" t="n"/>
@@ -4553,55 +4584,79 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="22" t="n">
+      <c r="A7" s="40" t="n">
         <v>10</v>
       </c>
-      <c r="B7" s="22" t="inlineStr">
+      <c r="B7" s="40" t="inlineStr">
         <is>
           <t>אימבלוייזר לתינוקות לשורש כף יד</t>
         </is>
       </c>
-      <c r="C7" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — לא נמצאה שום התאמה (לא מדויקת ולא קרובה) בטבלת המחירים</t>
-        </is>
-      </c>
-      <c r="D7" s="24" t="inlineStr"/>
-      <c r="E7" s="24" t="inlineStr"/>
+      <c r="C7" s="41" t="inlineStr">
+        <is>
+          <t>נבדק - לא הוכרע (אין מוצר מקביל קלינית באזור)</t>
+        </is>
+      </c>
+      <c r="D7" s="42" t="inlineStr">
+        <is>
+          <t>סבב 2 (אזור אנטומי + שיקול קליני)</t>
+        </is>
+      </c>
+      <c r="E7" s="42" t="inlineStr">
+        <is>
+          <t>אימבלוייזר "לתינוקות" - כל המועמדים הם מכשירי מבוגרים, אין גרסה ייעודית לתינוקות בטבלת המחירים (הבדל גיל/מידה מהותי)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="22" t="n">
+      <c r="A8" s="40" t="n">
         <v>11</v>
       </c>
-      <c r="B8" s="22" t="inlineStr">
+      <c r="B8" s="40" t="inlineStr">
         <is>
           <t>חבק שורש כף יד ללא סד</t>
         </is>
       </c>
-      <c r="C8" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — לא נמצאה שום התאמה (לא מדויקת ולא קרובה) בטבלת המחירים</t>
-        </is>
-      </c>
-      <c r="D8" s="24" t="inlineStr"/>
-      <c r="E8" s="24" t="inlineStr"/>
+      <c r="C8" s="41" t="inlineStr">
+        <is>
+          <t>נבדק - לא הוכרע (אין מוצר מקביל קלינית באזור)</t>
+        </is>
+      </c>
+      <c r="D8" s="42" t="inlineStr">
+        <is>
+          <t>סבב 2 (אזור אנטומי + שיקול קליני)</t>
+        </is>
+      </c>
+      <c r="E8" s="42" t="inlineStr">
+        <is>
+          <t>תובע חבק "ללא סד" (ללא קיבוע קשיח) - כל המועמדים הם מכשירים עם קיבוע/תמיכה קשיחה (עם/בלי אגודל, מקבע קשיח) - היפוך מהותי של המאפיין המבוקש</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="22" t="n">
+      <c r="A9" s="40" t="n">
         <v>12</v>
       </c>
-      <c r="B9" s="22" t="inlineStr">
+      <c r="B9" s="40" t="inlineStr">
         <is>
           <t>תומך פעיל למרפק עם סיליקון (לפחות 10 ס"מ מעל ומתחת לקו המפרק)</t>
         </is>
       </c>
-      <c r="C9" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — לא נמצאה שום התאמה (לא מדויקת ולא קרובה) בטבלת המחירים</t>
-        </is>
-      </c>
-      <c r="D9" s="24" t="inlineStr"/>
-      <c r="E9" s="24" t="inlineStr"/>
+      <c r="C9" s="41" t="inlineStr">
+        <is>
+          <t>נבדק - לא הוכרע (אין מוצר מקביל קלינית באזור)</t>
+        </is>
+      </c>
+      <c r="D9" s="42" t="inlineStr">
+        <is>
+          <t>סבב 2 (אזור אנטומי + שיקול קליני)</t>
+        </is>
+      </c>
+      <c r="E9" s="42" t="inlineStr">
+        <is>
+          <t>שרוול/תומך עם סיליקון 10 ס"מ מעל/מתחת למפרק (סוג sleeve) - המועמדים הם רצועות/כריות ל"מרפק טניס" (סוג device שונה לחלוטין, לא sleeve מעגלי)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="22" t="n">
@@ -4625,55 +4680,79 @@
       <c r="E10" s="24" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="22" t="n">
+      <c r="A11" s="40" t="n">
         <v>14</v>
       </c>
-      <c r="B11" s="22" t="inlineStr">
+      <c r="B11" s="40" t="inlineStr">
         <is>
           <t>מגן מרפק עם חיזוקי מתכת וציר יישור/ כיפוף מייצב POST OP</t>
         </is>
       </c>
-      <c r="C11" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — לא נמצאה שום התאמה (לא מדויקת ולא קרובה) בטבלת המחירים</t>
-        </is>
-      </c>
-      <c r="D11" s="24" t="inlineStr"/>
-      <c r="E11" s="24" t="inlineStr"/>
+      <c r="C11" s="41" t="inlineStr">
+        <is>
+          <t>נבדק - לא הוכרע (אין מוצר מקביל קלינית באזור)</t>
+        </is>
+      </c>
+      <c r="D11" s="42" t="inlineStr">
+        <is>
+          <t>סבב 2 (אזור אנטומי + שיקול קליני)</t>
+        </is>
+      </c>
+      <c r="E11" s="42" t="inlineStr">
+        <is>
+          <t>מגן מרפק עם חיזוקי מתכת+ציר, POST OP - אין מועמד עם מתכת/ציר; המועמדים הם רצועות מרפק-טניס בסיסיות בלבד</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="22" t="n">
+      <c r="A12" s="40" t="n">
         <v>15</v>
       </c>
-      <c r="B12" s="22" t="inlineStr">
+      <c r="B12" s="40" t="inlineStr">
         <is>
           <t>שרוול למרפק אלסטי</t>
         </is>
       </c>
-      <c r="C12" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — לא נמצאה שום התאמה (לא מדויקת ולא קרובה) בטבלת המחירים</t>
-        </is>
-      </c>
-      <c r="D12" s="24" t="inlineStr"/>
-      <c r="E12" s="24" t="inlineStr"/>
+      <c r="C12" s="41" t="inlineStr">
+        <is>
+          <t>נבדק - לא הוכרע (אין מוצר מקביל קלינית באזור)</t>
+        </is>
+      </c>
+      <c r="D12" s="42" t="inlineStr">
+        <is>
+          <t>סבב 2 (אזור אנטומי + שיקול קליני)</t>
+        </is>
+      </c>
+      <c r="E12" s="42" t="inlineStr">
+        <is>
+          <t>שרוול מרפק אלסטי (sleeve) - המועמדים הם רצועות ממוקדות למרפק טניס, לא שרוול אלסטי מלא</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="22" t="n">
+      <c r="A13" s="28" t="n">
         <v>16</v>
       </c>
-      <c r="B13" s="22" t="inlineStr">
+      <c r="B13" s="28" t="inlineStr">
         <is>
           <t>קיבוע אמה צמודה לבטן לאחר ניתוח</t>
         </is>
       </c>
-      <c r="C13" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — לא נמצאה שום התאמה (לא מדויקת ולא קרובה) בטבלת המחירים</t>
-        </is>
-      </c>
-      <c r="D13" s="24" t="inlineStr"/>
-      <c r="E13" s="24" t="inlineStr"/>
+      <c r="C13" s="29" t="inlineStr">
+        <is>
+          <t>נבדק - לא הוכרע (מועמד קליני סביר, אך כמה מחירים מתחרים)</t>
+        </is>
+      </c>
+      <c r="D13" s="30" t="inlineStr">
+        <is>
+          <t>סבב 2 (אזור אנטומי + שיקול קליני)</t>
+        </is>
+      </c>
+      <c r="E13" s="30" t="inlineStr">
+        <is>
+          <t>מועמד קליני סביר: "קיבוע אחרי צניחה/ניתוח לאחר ניתוח" (גם קיבוע לאחר ניתוח) - אך יש לו 3 ערכי-מחיר שונים (מתוך 4 שורות) בטבלת המקור - לא ניתן לבחור</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="28" t="n">
@@ -4776,38 +4855,54 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="22" t="n">
+      <c r="A18" s="40" t="n">
         <v>21</v>
       </c>
-      <c r="B18" s="22" t="inlineStr">
+      <c r="B18" s="40" t="inlineStr">
         <is>
           <t>שמינייה לכתף / עצם הבריח</t>
         </is>
       </c>
-      <c r="C18" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — לא נמצאה שום התאמה (לא מדויקת ולא קרובה) בטבלת המחירים</t>
-        </is>
-      </c>
-      <c r="D18" s="24" t="inlineStr"/>
-      <c r="E18" s="24" t="inlineStr"/>
+      <c r="C18" s="41" t="inlineStr">
+        <is>
+          <t>נבדק - לא הוכרע (אין מוצר מקביל קלינית באזור)</t>
+        </is>
+      </c>
+      <c r="D18" s="42" t="inlineStr">
+        <is>
+          <t>סבב 2 (אזור אנטומי + שיקול קליני)</t>
+        </is>
+      </c>
+      <c r="E18" s="42" t="inlineStr">
+        <is>
+          <t>שמינייה לכתף/עצם בריח (figure-8 clavicle brace) - התקן ייעודי שאין לו מקבילה ברשימה (מקבעי כתף/זרוע מורכבים יותר, לא שמינייה)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="22" t="n">
+      <c r="A19" s="40" t="n">
         <v>22</v>
       </c>
-      <c r="B19" s="22" t="inlineStr">
+      <c r="B19" s="40" t="inlineStr">
         <is>
           <t>מתלה ליד /זרוע</t>
         </is>
       </c>
-      <c r="C19" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — לא נמצאה שום התאמה (לא מדויקת ולא קרובה) בטבלת המחירים</t>
-        </is>
-      </c>
-      <c r="D19" s="24" t="inlineStr"/>
-      <c r="E19" s="24" t="inlineStr"/>
+      <c r="C19" s="41" t="inlineStr">
+        <is>
+          <t>נבדק - לא הוכרע (אין מוצר מקביל קלינית באזור)</t>
+        </is>
+      </c>
+      <c r="D19" s="42" t="inlineStr">
+        <is>
+          <t>סבב 2 (אזור אנטומי + שיקול קליני)</t>
+        </is>
+      </c>
+      <c r="E19" s="42" t="inlineStr">
+        <is>
+          <t>מתלה יד/זרוע (sling בסיסי) - אין מתלה בסיסי ברשימה, רק מקבעים מורכבים יותר</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="28" t="n">
@@ -4860,21 +4955,29 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="22" t="n">
+      <c r="A22" s="28" t="n">
         <v>25</v>
       </c>
-      <c r="B22" s="22" t="inlineStr">
+      <c r="B22" s="28" t="inlineStr">
         <is>
           <t>חגורת Jewett 3 POINTS</t>
         </is>
       </c>
-      <c r="C22" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — לא נמצאה שום התאמה (לא מדויקת ולא קרובה) בטבלת המחירים</t>
-        </is>
-      </c>
-      <c r="D22" s="24" t="inlineStr"/>
-      <c r="E22" s="24" t="inlineStr"/>
+      <c r="C22" s="29" t="inlineStr">
+        <is>
+          <t>נבדק - לא הוכרע (מועמד קליני סביר, אך כמה מחירים מתחרים)</t>
+        </is>
+      </c>
+      <c r="D22" s="30" t="inlineStr">
+        <is>
+          <t>סבב 2 (אזור אנטומי + שיקול קליני)</t>
+        </is>
+      </c>
+      <c r="E22" s="30" t="inlineStr">
+        <is>
+          <t>מועמד קליני מדויק: "חגורת גב לשברים תואם JEWETT" - התאמה ישירה בשם ההתקן! אך יש 2 ערכי-מחיר שונים בטבלת המקור - לא ניתן לבחור בלי הכרעה איזה ספק</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="28" t="n">
@@ -4927,21 +5030,29 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="22" t="n">
+      <c r="A25" s="40" t="n">
         <v>28</v>
       </c>
-      <c r="B25" s="22" t="inlineStr">
+      <c r="B25" s="40" t="inlineStr">
         <is>
           <t>כיסוי למחוכים לספונדליזיס (ניתן בשב"ן רק בהתוויות שאינן בסל)</t>
         </is>
       </c>
-      <c r="C25" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — לא נמצאה שום התאמה (לא מדויקת ולא קרובה) בטבלת המחירים</t>
-        </is>
-      </c>
-      <c r="D25" s="24" t="inlineStr"/>
-      <c r="E25" s="24" t="inlineStr"/>
+      <c r="C25" s="41" t="inlineStr">
+        <is>
+          <t>נבדק - לא הוכרע (אין מוצר מקביל קלינית באזור)</t>
+        </is>
+      </c>
+      <c r="D25" s="42" t="inlineStr">
+        <is>
+          <t>סבב 2 (אזור אנטומי + שיקול קליני)</t>
+        </is>
+      </c>
+      <c r="E25" s="42" t="inlineStr">
+        <is>
+          <t>כיסוי למחוך ספונדליזיס (פריט אביזר-לוואי ספציפי, לא המחוך עצמו) - אין מקבילה</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="22" t="n">
@@ -4986,55 +5097,79 @@
       <c r="E27" s="24" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="22" t="n">
+      <c r="A28" s="40" t="n">
         <v>31</v>
       </c>
-      <c r="B28" s="22" t="inlineStr">
+      <c r="B28" s="40" t="inlineStr">
         <is>
           <t>חגורה מייצבת -חזה צוואר /SOMI</t>
         </is>
       </c>
-      <c r="C28" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — לא נמצאה שום התאמה (לא מדויקת ולא קרובה) בטבלת המחירים</t>
-        </is>
-      </c>
-      <c r="D28" s="24" t="inlineStr"/>
-      <c r="E28" s="24" t="inlineStr"/>
+      <c r="C28" s="41" t="inlineStr">
+        <is>
+          <t>נבדק - לא הוכרע (אין מוצר מקביל קלינית באזור)</t>
+        </is>
+      </c>
+      <c r="D28" s="42" t="inlineStr">
+        <is>
+          <t>סבב 2 (אזור אנטומי + שיקול קליני)</t>
+        </is>
+      </c>
+      <c r="E28" s="42" t="inlineStr">
+        <is>
+          <t>חגורת SOMI (שלד חזה-צוואר) - התקן שונה מבנית מצווארונים (PMT/פילדלפיה/VISTA) שברשימה - לא אותה משפחת מכשור</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="22" t="n">
+      <c r="A29" s="40" t="n">
         <v>32</v>
       </c>
-      <c r="B29" s="22" t="inlineStr">
+      <c r="B29" s="40" t="inlineStr">
         <is>
           <t>צווארון רך</t>
         </is>
       </c>
-      <c r="C29" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — לא נמצאה שום התאמה (לא מדויקת ולא קרובה) בטבלת המחירים</t>
-        </is>
-      </c>
-      <c r="D29" s="24" t="inlineStr"/>
-      <c r="E29" s="24" t="inlineStr"/>
+      <c r="C29" s="41" t="inlineStr">
+        <is>
+          <t>נבדק - לא הוכרע (אין מוצר מקביל קלינית באזור)</t>
+        </is>
+      </c>
+      <c r="D29" s="42" t="inlineStr">
+        <is>
+          <t>סבב 2 (אזור אנטומי + שיקול קליני)</t>
+        </is>
+      </c>
+      <c r="E29" s="42" t="inlineStr">
+        <is>
+          <t>צווארון רך - המועמדים הם צווארונים "מורכבים" (קשיחים) עם/בלי ריפוד - היפוך מהותי (רך מול קשיח, כמו מקרה DROP FOOT)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="22" t="n">
+      <c r="A30" s="40" t="n">
         <v>33</v>
       </c>
-      <c r="B30" s="22" t="inlineStr">
+      <c r="B30" s="40" t="inlineStr">
         <is>
           <t>חגורת גב אווירירית ללא תמיכות</t>
         </is>
       </c>
-      <c r="C30" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — לא נמצאה שום התאמה (לא מדויקת ולא קרובה) בטבלת המחירים</t>
-        </is>
-      </c>
-      <c r="D30" s="24" t="inlineStr"/>
-      <c r="E30" s="24" t="inlineStr"/>
+      <c r="C30" s="41" t="inlineStr">
+        <is>
+          <t>נבדק - לא הוכרע (אין מוצר מקביל קלינית באזור)</t>
+        </is>
+      </c>
+      <c r="D30" s="42" t="inlineStr">
+        <is>
+          <t>סבב 2 (אזור אנטומי + שיקול קליני)</t>
+        </is>
+      </c>
+      <c r="E30" s="42" t="inlineStr">
+        <is>
+          <t>חגורת גב אווירירית ללא תמיכות - המועמדים הם חגורות עם חיזוקים/תמיכות (ההפך המבוקש), ואין גרסה "אווירירית" ברשימה</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="28" t="n">
@@ -5062,21 +5197,29 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="22" t="n">
+      <c r="A32" s="40" t="n">
         <v>35</v>
       </c>
-      <c r="B32" s="22" t="inlineStr">
+      <c r="B32" s="40" t="inlineStr">
         <is>
           <t>מגן ברך ללא סיליקון</t>
         </is>
       </c>
-      <c r="C32" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — לא נמצאה שום התאמה (לא מדויקת ולא קרובה) בטבלת המחירים</t>
-        </is>
-      </c>
-      <c r="D32" s="24" t="inlineStr"/>
-      <c r="E32" s="24" t="inlineStr"/>
+      <c r="C32" s="41" t="inlineStr">
+        <is>
+          <t>נבדק - לא הוכרע (אין מוצר מקביל קלינית באזור)</t>
+        </is>
+      </c>
+      <c r="D32" s="42" t="inlineStr">
+        <is>
+          <t>סבב 2 (אזור אנטומי + שיקול קליני)</t>
+        </is>
+      </c>
+      <c r="E32" s="42" t="inlineStr">
+        <is>
+          <t>מגן ברך ללא סיליקון - כל המועמדים הם עם טבעת סיליקון או מסגרות מתכת - היפוך מהותי של המאפיין המבוקש</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="28" t="n">
@@ -5125,21 +5268,29 @@
       <c r="E34" s="24" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="22" t="n">
+      <c r="A35" s="40" t="n">
         <v>38</v>
       </c>
-      <c r="B35" s="22" t="inlineStr">
+      <c r="B35" s="40" t="inlineStr">
         <is>
           <t>מייצב ברך ללא צירים - אימבולייזר</t>
         </is>
       </c>
-      <c r="C35" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — לא נמצאה שום התאמה (לא מדויקת ולא קרובה) בטבלת המחירים</t>
-        </is>
-      </c>
-      <c r="D35" s="24" t="inlineStr"/>
-      <c r="E35" s="24" t="inlineStr"/>
+      <c r="C35" s="41" t="inlineStr">
+        <is>
+          <t>נבדק - לא הוכרע (אין מוצר מקביל קלינית באזור)</t>
+        </is>
+      </c>
+      <c r="D35" s="42" t="inlineStr">
+        <is>
+          <t>סבב 2 (אזור אנטומי + שיקול קליני)</t>
+        </is>
+      </c>
+      <c r="E35" s="42" t="inlineStr">
+        <is>
+          <t>מייצב ברך ללא צירים (אימבולייזר) - המועמדים הרלוונטיים ביותר הם עם צירים מתכווננים (ההפך המבוקש)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="28" t="n">
@@ -5230,21 +5381,29 @@
       <c r="E39" s="24" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="22" t="n">
+      <c r="A40" s="40" t="n">
         <v>43</v>
       </c>
-      <c r="B40" s="22" t="inlineStr">
+      <c r="B40" s="40" t="inlineStr">
         <is>
           <t>אימבלוייזר לתינוקות לברך</t>
         </is>
       </c>
-      <c r="C40" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — לא נמצאה שום התאמה (לא מדויקת ולא קרובה) בטבלת המחירים</t>
-        </is>
-      </c>
-      <c r="D40" s="24" t="inlineStr"/>
-      <c r="E40" s="24" t="inlineStr"/>
+      <c r="C40" s="41" t="inlineStr">
+        <is>
+          <t>נבדק - לא הוכרע (אין מוצר מקביל קלינית באזור)</t>
+        </is>
+      </c>
+      <c r="D40" s="42" t="inlineStr">
+        <is>
+          <t>סבב 2 (אזור אנטומי + שיקול קליני)</t>
+        </is>
+      </c>
+      <c r="E40" s="42" t="inlineStr">
+        <is>
+          <t>אימבלוייזר "לתינוקות" לברך - אותה בעיית גיל/מידה כמו שורה 10, אין גרסה ייעודית לתינוקות</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="28" t="n">
@@ -5389,106 +5548,154 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="22" t="n">
+      <c r="A47" s="43" t="n">
         <v>50</v>
       </c>
-      <c r="B47" s="22" t="inlineStr">
+      <c r="B47" s="43" t="inlineStr">
         <is>
           <t>סד לתמיכה ב-FOOT DROP ובכף הרגל קשיח/ גמיש , סד פיני לשיקום</t>
         </is>
       </c>
-      <c r="C47" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — לא נמצאה שום התאמה (לא מדויקת ולא קרובה) בטבלת המחירים</t>
-        </is>
-      </c>
-      <c r="D47" s="24" t="inlineStr"/>
-      <c r="E47" s="24" t="inlineStr"/>
+      <c r="C47" s="44" t="inlineStr">
+        <is>
+          <t>נבדק - לא הוכרע (הבדל קליני מהותי במנגנון/סוג ההתקן)</t>
+        </is>
+      </c>
+      <c r="D47" s="45" t="inlineStr">
+        <is>
+          <t>סבב 2 (אזור אנטומי + שיקול קליני)</t>
+        </is>
+      </c>
+      <c r="E47" s="45" t="inlineStr">
+        <is>
+          <t>נבדק לעומק בסבב קודם: "קשיח/גמיש + סד פיני לשיקום" (קטגוריית-על) מול מועמדים ספציפיים "קשיח" בלבד - הבדל מהותי בהיקף/סוג ההתקן, לא הוכרע</t>
+        </is>
+      </c>
     </row>
     <row r="48">
-      <c r="A48" s="22" t="n">
+      <c r="A48" s="43" t="n">
         <v>51</v>
       </c>
-      <c r="B48" s="22" t="inlineStr">
+      <c r="B48" s="43" t="inlineStr">
         <is>
           <t>סד לתמיכה ב-FOOT DROP - תמיכת קרסול ברצועות/ קפיץ (תואם דיקטוס)</t>
         </is>
       </c>
-      <c r="C48" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — לא נמצאה שום התאמה (לא מדויקת ולא קרובה) בטבלת המחירים</t>
-        </is>
-      </c>
-      <c r="D48" s="24" t="inlineStr"/>
-      <c r="E48" s="24" t="inlineStr"/>
+      <c r="C48" s="44" t="inlineStr">
+        <is>
+          <t>נבדק - לא הוכרע (הבדל קליני מהותי במנגנון/סוג ההתקן)</t>
+        </is>
+      </c>
+      <c r="D48" s="45" t="inlineStr">
+        <is>
+          <t>סבב 2 (אזור אנטומי + שיקול קליני)</t>
+        </is>
+      </c>
+      <c r="E48" s="45" t="inlineStr">
+        <is>
+          <t>נבדק לעומק בסבב קודם: "תמיכת קרסול ברצועות/קפיץ" מול מועמד "תמיכת קרסול קשיח" - מנגנון שונה מהותית (גמיש/קפיצי מול קשיח), לא הוכרע</t>
+        </is>
+      </c>
     </row>
     <row r="49">
-      <c r="A49" s="22" t="n">
+      <c r="A49" s="43" t="n">
         <v>52</v>
       </c>
-      <c r="B49" s="22" t="inlineStr">
+      <c r="B49" s="43" t="inlineStr">
         <is>
           <t>נעל גבס</t>
         </is>
       </c>
-      <c r="C49" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — לא נמצאה שום התאמה (לא מדויקת ולא קרובה) בטבלת המחירים</t>
-        </is>
-      </c>
-      <c r="D49" s="24" t="inlineStr"/>
-      <c r="E49" s="24" t="inlineStr"/>
+      <c r="C49" s="44" t="inlineStr">
+        <is>
+          <t>נבדק - לא הוכרע (מטרה קלינית לא ודאית + ריבוי מחירים)</t>
+        </is>
+      </c>
+      <c r="D49" s="45" t="inlineStr">
+        <is>
+          <t>סבב 2 (אזור אנטומי + שיקול קליני)</t>
+        </is>
+      </c>
+      <c r="E49" s="45" t="inlineStr">
+        <is>
+          <t>"נעל גבס" (ללבישה מעל גבס) מול "דמוי נעל - off-loading device" (התקן פיזור-לחץ, לאו דווקא לגבס) - מטרה קלינית שונה, לא בטוח שזו אותה קטגוריה; ובנוסף למועמד 2 ערכי-מחיר שונים</t>
+        </is>
+      </c>
     </row>
     <row r="50">
-      <c r="A50" s="22" t="n">
+      <c r="A50" s="28" t="n">
         <v>53</v>
       </c>
-      <c r="B50" s="22" t="inlineStr">
+      <c r="B50" s="28" t="inlineStr">
         <is>
           <t>נעלי אחרי ניתוח POST OP</t>
         </is>
       </c>
-      <c r="C50" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — לא נמצאה שום התאמה (לא מדויקת ולא קרובה) בטבלת המחירים</t>
-        </is>
-      </c>
-      <c r="D50" s="24" t="inlineStr"/>
-      <c r="E50" s="24" t="inlineStr"/>
+      <c r="C50" s="29" t="inlineStr">
+        <is>
+          <t>נבדק - לא הוכרע (מועמד קליני סביר, אך כמה מחירים מתחרים)</t>
+        </is>
+      </c>
+      <c r="D50" s="30" t="inlineStr">
+        <is>
+          <t>סבב 2 (אזור אנטומי + שיקול קליני)</t>
+        </is>
+      </c>
+      <c r="E50" s="30" t="inlineStr">
+        <is>
+          <t>מועמד קליני סביר: "דמוי נעל - off-loading device" (נעל פוסט-ניתוחית סטנדרטית בשוק) - אך יש לו 2 ערכי-מחיר שונים בטבלה - לא ניתן לבחור</t>
+        </is>
+      </c>
     </row>
     <row r="51">
-      <c r="A51" s="22" t="n">
+      <c r="A51" s="28" t="n">
         <v>54</v>
       </c>
-      <c r="B51" s="22" t="inlineStr">
+      <c r="B51" s="28" t="inlineStr">
         <is>
           <t>נעל לאחר ניתוח/ לריפוי פצע עם הגבהה קדמית</t>
         </is>
       </c>
-      <c r="C51" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — לא נמצאה שום התאמה (לא מדויקת ולא קרובה) בטבלת המחירים</t>
-        </is>
-      </c>
-      <c r="D51" s="24" t="inlineStr"/>
-      <c r="E51" s="24" t="inlineStr"/>
+      <c r="C51" s="29" t="inlineStr">
+        <is>
+          <t>נבדק - לא הוכרע (מועמד קליני סביר, אך כמה מחירים מתחרים)</t>
+        </is>
+      </c>
+      <c r="D51" s="30" t="inlineStr">
+        <is>
+          <t>סבב 2 (אזור אנטומי + שיקול קליני)</t>
+        </is>
+      </c>
+      <c r="E51" s="30" t="inlineStr">
+        <is>
+          <t>מועמד אפשרי: "דמוי נעל - off-loading device" - לא ברור אם תואם ספציפית "הגבהה קדמית" (המועמד לא מציין כיוון הגבהה), ובנוסף 2 ערכי-מחיר שונים</t>
+        </is>
+      </c>
     </row>
     <row r="52">
-      <c r="A52" s="22" t="n">
+      <c r="A52" s="28" t="n">
         <v>55</v>
       </c>
-      <c r="B52" s="22" t="inlineStr">
+      <c r="B52" s="28" t="inlineStr">
         <is>
           <t>נעל לאחר ניתוח/ לריפוי פצע עם הגבהה אחורית</t>
         </is>
       </c>
-      <c r="C52" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — לא נמצאה שום התאמה (לא מדויקת ולא קרובה) בטבלת המחירים</t>
-        </is>
-      </c>
-      <c r="D52" s="24" t="inlineStr"/>
-      <c r="E52" s="24" t="inlineStr"/>
+      <c r="C52" s="29" t="inlineStr">
+        <is>
+          <t>נבדק - לא הוכרע (מועמד קליני סביר, אך כמה מחירים מתחרים)</t>
+        </is>
+      </c>
+      <c r="D52" s="30" t="inlineStr">
+        <is>
+          <t>סבב 2 (אזור אנטומי + שיקול קליני)</t>
+        </is>
+      </c>
+      <c r="E52" s="30" t="inlineStr">
+        <is>
+          <t>מועמד אפשרי: "דמוי נעל - off-loading device" - לא ברור אם תואם ספציפית "הגבהה אחורית", ובנוסף 2 ערכי-מחיר שונים</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="22" t="n">
@@ -5512,21 +5719,29 @@
       <c r="E53" s="24" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" s="22" t="n">
+      <c r="A54" s="28" t="n">
         <v>57</v>
       </c>
-      <c r="B54" s="22" t="inlineStr">
+      <c r="B54" s="28" t="inlineStr">
         <is>
           <t>עקב סיליקון בלי נקודה כחולה</t>
         </is>
       </c>
-      <c r="C54" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — לא נמצאה שום התאמה (לא מדויקת ולא קרובה) בטבלת המחירים</t>
-        </is>
-      </c>
-      <c r="D54" s="24" t="inlineStr"/>
-      <c r="E54" s="24" t="inlineStr"/>
+      <c r="C54" s="29" t="inlineStr">
+        <is>
+          <t>נבדק - לא הוכרע (מועמד קליני סביר, אך כמה מחירים מתחרים)</t>
+        </is>
+      </c>
+      <c r="D54" s="30" t="inlineStr">
+        <is>
+          <t>סבב 2 (אזור אנטומי + שיקול קליני)</t>
+        </is>
+      </c>
+      <c r="E54" s="30" t="inlineStr">
+        <is>
+          <t>מועמד אפשרי: "עקב סיליקון לדורבן" - אך זה ייעודי לדורבן (אינדיקציה ספציפית) בעוד השורה במכרז היא כללית ("בלי נקודה כחולה" = מאפיין ייצור, לא אינדיקציה) - התאמה לא ודאית; ובנוסף 2 ערכי-מחיר שונים</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="28" t="n">
@@ -5554,123 +5769,179 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="22" t="n">
+      <c r="A56" s="40" t="n">
         <v>59</v>
       </c>
-      <c r="B56" s="22" t="inlineStr">
+      <c r="B56" s="40" t="inlineStr">
         <is>
           <t>סד הלוקס ואלגוס</t>
         </is>
       </c>
-      <c r="C56" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — לא נמצאה שום התאמה (לא מדויקת ולא קרובה) בטבלת המחירים</t>
-        </is>
-      </c>
-      <c r="D56" s="24" t="inlineStr"/>
-      <c r="E56" s="24" t="inlineStr"/>
+      <c r="C56" s="41" t="inlineStr">
+        <is>
+          <t>נבדק - לא הוכרע (אין מוצר מקביל קלינית באזור)</t>
+        </is>
+      </c>
+      <c r="D56" s="42" t="inlineStr">
+        <is>
+          <t>סבב 2 (אזור אנטומי + שיקול קליני)</t>
+        </is>
+      </c>
+      <c r="E56" s="42" t="inlineStr">
+        <is>
+          <t>סד הלוקס ואלגוס (בקע בוהן/bunion) - התקן ייעודי לחלוטין, אין מקבילה ברשימת המועמדים (כף רגל) כלל</t>
+        </is>
+      </c>
     </row>
     <row r="57">
-      <c r="A57" s="22" t="n">
+      <c r="A57" s="40" t="n">
         <v>60</v>
       </c>
-      <c r="B57" s="22" t="inlineStr">
+      <c r="B57" s="40" t="inlineStr">
         <is>
           <t>מדרס סיליקון מוכן עם נקודות מחוברות</t>
         </is>
       </c>
-      <c r="C57" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — לא נמצאה שום התאמה (לא מדויקת ולא קרובה) בטבלת המחירים</t>
-        </is>
-      </c>
-      <c r="D57" s="24" t="inlineStr"/>
-      <c r="E57" s="24" t="inlineStr"/>
+      <c r="C57" s="41" t="inlineStr">
+        <is>
+          <t>נבדק - לא הוכרע (אין מוצר מקביל קלינית באזור)</t>
+        </is>
+      </c>
+      <c r="D57" s="42" t="inlineStr">
+        <is>
+          <t>סבב 2 (אזור אנטומי + שיקול קליני)</t>
+        </is>
+      </c>
+      <c r="E57" s="42" t="inlineStr">
+        <is>
+          <t>מדרס סיליקון עם נקודות מחוברות - אין קטגוריית מדרסים/אורתוטיקה כלל ברשימת המועמדים</t>
+        </is>
+      </c>
     </row>
     <row r="58">
-      <c r="A58" s="22" t="n">
+      <c r="A58" s="40" t="n">
         <v>61</v>
       </c>
-      <c r="B58" s="22" t="inlineStr">
+      <c r="B58" s="40" t="inlineStr">
         <is>
           <t>מדרסי ג'ל</t>
         </is>
       </c>
-      <c r="C58" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — לא נמצאה שום התאמה (לא מדויקת ולא קרובה) בטבלת המחירים</t>
-        </is>
-      </c>
-      <c r="D58" s="24" t="inlineStr"/>
-      <c r="E58" s="24" t="inlineStr"/>
+      <c r="C58" s="41" t="inlineStr">
+        <is>
+          <t>נבדק - לא הוכרע (אין מוצר מקביל קלינית באזור)</t>
+        </is>
+      </c>
+      <c r="D58" s="42" t="inlineStr">
+        <is>
+          <t>סבב 2 (אזור אנטומי + שיקול קליני)</t>
+        </is>
+      </c>
+      <c r="E58" s="42" t="inlineStr">
+        <is>
+          <t>מדרסי ג'ל - אין קטגוריית מדרסים ברשימת המועמדים</t>
+        </is>
+      </c>
     </row>
     <row r="59">
-      <c r="A59" s="22" t="n">
+      <c r="A59" s="40" t="n">
         <v>62</v>
       </c>
-      <c r="B59" s="22" t="inlineStr">
+      <c r="B59" s="40" t="inlineStr">
         <is>
           <t>סד לילה לפסאיטיס- פלנטרית בכף הרגל</t>
         </is>
       </c>
-      <c r="C59" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — לא נמצאה שום התאמה (לא מדויקת ולא קרובה) בטבלת המחירים</t>
-        </is>
-      </c>
-      <c r="D59" s="24" t="inlineStr"/>
-      <c r="E59" s="24" t="inlineStr"/>
+      <c r="C59" s="41" t="inlineStr">
+        <is>
+          <t>נבדק - לא הוכרע (אין מוצר מקביל קלינית באזור)</t>
+        </is>
+      </c>
+      <c r="D59" s="42" t="inlineStr">
+        <is>
+          <t>סבב 2 (אזור אנטומי + שיקול קליני)</t>
+        </is>
+      </c>
+      <c r="E59" s="42" t="inlineStr">
+        <is>
+          <t>סד לילה לפסציאיטיס פלנטרית - התקן ללבישת לילה, שונה מבנית מסדי DROP FOOT/נעליים - אין מקבילה</t>
+        </is>
+      </c>
     </row>
     <row r="60">
-      <c r="A60" s="22" t="n">
+      <c r="A60" s="40" t="n">
         <v>63</v>
       </c>
-      <c r="B60" s="22" t="inlineStr">
+      <c r="B60" s="40" t="inlineStr">
         <is>
           <t>מדרס בהתאמה אישית</t>
         </is>
       </c>
-      <c r="C60" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — לא נמצאה שום התאמה (לא מדויקת ולא קרובה) בטבלת המחירים</t>
-        </is>
-      </c>
-      <c r="D60" s="24" t="inlineStr"/>
-      <c r="E60" s="24" t="inlineStr"/>
+      <c r="C60" s="41" t="inlineStr">
+        <is>
+          <t>נבדק - לא הוכרע (אין מוצר מקביל קלינית באזור)</t>
+        </is>
+      </c>
+      <c r="D60" s="42" t="inlineStr">
+        <is>
+          <t>סבב 2 (אזור אנטומי + שיקול קליני)</t>
+        </is>
+      </c>
+      <c r="E60" s="42" t="inlineStr">
+        <is>
+          <t>מדרס בהתאמה אישית - אין קטגוריית מדרסים ברשימת המועמדים</t>
+        </is>
+      </c>
     </row>
     <row r="61">
-      <c r="A61" s="22" t="n">
+      <c r="A61" s="40" t="n">
         <v>64</v>
       </c>
-      <c r="B61" s="22" t="inlineStr">
+      <c r="B61" s="40" t="inlineStr">
         <is>
           <t>מדרסים מיוחדים - ביו מכני - מדרסים לסכרתיים - עיוות רגל</t>
         </is>
       </c>
-      <c r="C61" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — לא נמצאה שום התאמה (לא מדויקת ולא קרובה) בטבלת המחירים</t>
-        </is>
-      </c>
-      <c r="D61" s="24" t="inlineStr"/>
-      <c r="E61" s="24" t="inlineStr"/>
+      <c r="C61" s="41" t="inlineStr">
+        <is>
+          <t>נבדק - לא הוכרע (אין מוצר מקביל קלינית באזור)</t>
+        </is>
+      </c>
+      <c r="D61" s="42" t="inlineStr">
+        <is>
+          <t>סבב 2 (אזור אנטומי + שיקול קליני)</t>
+        </is>
+      </c>
+      <c r="E61" s="42" t="inlineStr">
+        <is>
+          <t>מדרסים ביו-מכניים לסכרתיים - אין קטגוריית מדרסים ברשימת המועמדים</t>
+        </is>
+      </c>
     </row>
     <row r="62">
-      <c r="A62" s="22" t="n">
+      <c r="A62" s="43" t="n">
         <v>65</v>
       </c>
-      <c r="B62" s="22" t="inlineStr">
+      <c r="B62" s="43" t="inlineStr">
         <is>
           <t>מגני ירכיים עם ריפוד / כרית מתנפחת למניעת שבר צוואר ירך</t>
         </is>
       </c>
-      <c r="C62" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — לא נמצאה שום התאמה (לא מדויקת ולא קרובה) בטבלת המחירים</t>
-        </is>
-      </c>
-      <c r="D62" s="24" t="inlineStr"/>
-      <c r="E62" s="24" t="inlineStr"/>
+      <c r="C62" s="44" t="inlineStr">
+        <is>
+          <t>נבדק - לא הוכרע (2 וריאנטים אפשריים, לא ברור איזה)</t>
+        </is>
+      </c>
+      <c r="D62" s="45" t="inlineStr">
+        <is>
+          <t>סבב 2 (אזור אנטומי + שיקול קליני)</t>
+        </is>
+      </c>
+      <c r="E62" s="45" t="inlineStr">
+        <is>
+          <t>השורה במכרז משלבת 2 מאפיינים ("עם ריפוד / כרית מתנפחת") שמופיעים כשתי שורות-מוצר נפרדות בטבלת המחירים ("מגן ירכיים עם ריפוד/כרית" בסך 44/103/147/83/97 מול "מתנפחות למניעת שבר צוואר ירך" בסך 49/113/162/95/112) - לא ברור איזה משני הווריאנטים לבחור</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="25" t="n">
@@ -5898,89 +6169,129 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="22" t="n">
+      <c r="A72" s="40" t="n">
         <v>75</v>
       </c>
-      <c r="B72" s="22" t="inlineStr">
+      <c r="B72" s="40" t="inlineStr">
         <is>
           <t>חגורת גב לאחר ניתוח בטן / חזה</t>
         </is>
       </c>
-      <c r="C72" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — לא נמצאה שום התאמה (לא מדויקת ולא קרובה) בטבלת המחירים</t>
-        </is>
-      </c>
-      <c r="D72" s="24" t="inlineStr"/>
-      <c r="E72" s="24" t="inlineStr"/>
+      <c r="C72" s="41" t="inlineStr">
+        <is>
+          <t>נבדק - לא הוכרע (אין מוצר מקביל קלינית באזור)</t>
+        </is>
+      </c>
+      <c r="D72" s="42" t="inlineStr">
+        <is>
+          <t>סבב 2 (אזור אנטומי + שיקול קליני)</t>
+        </is>
+      </c>
+      <c r="E72" s="42" t="inlineStr">
+        <is>
+          <t>חגורת גב לאחר ניתוח בטן/חזה (תמיכה כללית) מול "חגורת בטן סטומה" (ייעודית לסטומה/פיום) - מטרה קלינית שונה מהותית</t>
+        </is>
+      </c>
     </row>
     <row r="73">
-      <c r="A73" s="22" t="n">
+      <c r="A73" s="40" t="n">
         <v>76</v>
       </c>
-      <c r="B73" s="22" t="inlineStr">
+      <c r="B73" s="40" t="inlineStr">
         <is>
           <t>חגורת בטן לאחר ניתוח חזה / בטן</t>
         </is>
       </c>
-      <c r="C73" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — לא נמצאה שום התאמה (לא מדויקת ולא קרובה) בטבלת המחירים</t>
-        </is>
-      </c>
-      <c r="D73" s="24" t="inlineStr"/>
-      <c r="E73" s="24" t="inlineStr"/>
+      <c r="C73" s="41" t="inlineStr">
+        <is>
+          <t>נבדק - לא הוכרע (אין מוצר מקביל קלינית באזור)</t>
+        </is>
+      </c>
+      <c r="D73" s="42" t="inlineStr">
+        <is>
+          <t>סבב 2 (אזור אנטומי + שיקול קליני)</t>
+        </is>
+      </c>
+      <c r="E73" s="42" t="inlineStr">
+        <is>
+          <t>אותה סיבה כמו שורה 75 - חגורת בטן כללית מול חגורת סטומה ייעודית</t>
+        </is>
+      </c>
     </row>
     <row r="74">
-      <c r="A74" s="22" t="n">
+      <c r="A74" s="40" t="n">
         <v>77</v>
       </c>
-      <c r="B74" s="22" t="inlineStr">
+      <c r="B74" s="40" t="inlineStr">
         <is>
           <t>סד למניעת פריקה התפתחותית במפרק הירכיים DDH</t>
         </is>
       </c>
-      <c r="C74" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — לא נמצאה שום התאמה (לא מדויקת ולא קרובה) בטבלת המחירים</t>
-        </is>
-      </c>
-      <c r="D74" s="24" t="inlineStr"/>
-      <c r="E74" s="24" t="inlineStr"/>
+      <c r="C74" s="41" t="inlineStr">
+        <is>
+          <t>נבדק - לא הוכרע (אין מוצר מקביל קלינית באזור)</t>
+        </is>
+      </c>
+      <c r="D74" s="42" t="inlineStr">
+        <is>
+          <t>סבב 2 (אזור אנטומי + שיקול קליני)</t>
+        </is>
+      </c>
+      <c r="E74" s="42" t="inlineStr">
+        <is>
+          <t>DDH (פריקה התפתחותית במפרק ירכיים אצל תינוקות) - מצב פדיאטרי-אורתופדי שונה לחלוטין; מיפוי אזור "מותניים"-&gt;"גב" לא רלוונטי כאן, אין מכשור מקביל בטבלת המחירים</t>
+        </is>
+      </c>
     </row>
     <row r="75">
-      <c r="A75" s="22" t="n">
+      <c r="A75" s="25" t="n">
         <v>78</v>
       </c>
-      <c r="B75" s="22" t="inlineStr">
+      <c r="B75" s="25" t="inlineStr">
         <is>
           <t>חגורת אגן ( אורט' - חגורת היריון)</t>
         </is>
       </c>
-      <c r="C75" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — לא נמצאה שום התאמה (לא מדויקת ולא קרובה) בטבלת המחירים</t>
-        </is>
-      </c>
-      <c r="D75" s="24" t="inlineStr"/>
-      <c r="E75" s="24" t="inlineStr"/>
+      <c r="C75" s="26" t="inlineStr">
+        <is>
+          <t>מולא (התאמה אזורית-קלינית, אושר 03/09)</t>
+        </is>
+      </c>
+      <c r="D75" s="27" t="inlineStr">
+        <is>
+          <t>סבב 2 (אזור אנטומי + שיקול קליני)</t>
+        </is>
+      </c>
+      <c r="E75" s="27" t="inlineStr">
+        <is>
+          <t>התאמה ברורה: "חגורת אגן (חגורת היריון)" = "חגורת גב עם תמיכה לנשים בהריון" - אותו מוצר בדיוק (חגורת היריון), ערך מחיר יחיד וחד-משמעי (31,72,103,45,53) - זהה למה שכבר אושר בשורה 27 לאותו מוצר</t>
+        </is>
+      </c>
     </row>
     <row r="76">
-      <c r="A76" s="22" t="n">
+      <c r="A76" s="40" t="n">
         <v>79</v>
       </c>
-      <c r="B76" s="22" t="inlineStr">
+      <c r="B76" s="40" t="inlineStr">
         <is>
           <t>חגורת חזה / שבר צלעות</t>
         </is>
       </c>
-      <c r="C76" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — לא נמצאה שום התאמה (לא מדויקת ולא קרובה) בטבלת המחירים</t>
-        </is>
-      </c>
-      <c r="D76" s="24" t="inlineStr"/>
-      <c r="E76" s="24" t="inlineStr"/>
+      <c r="C76" s="41" t="inlineStr">
+        <is>
+          <t>נבדק - לא הוכרע (אין מוצר מקביל קלינית באזור)</t>
+        </is>
+      </c>
+      <c r="D76" s="42" t="inlineStr">
+        <is>
+          <t>סבב 2 (אזור אנטומי + שיקול קליני)</t>
+        </is>
+      </c>
+      <c r="E76" s="42" t="inlineStr">
+        <is>
+          <t>חגורת חזה/שבר צלעות - כל המועמדים (מקבוצת "חגורת שבר" בטבלת המחירים) הם בפועל חגורות בקע/הרניה, לא חגורות צלעות/חזה - מיפוי האזור החזיר קטגוריה לא רלוונטית, אין מוצר תואם בפועל</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:E76"/>

</xml_diff>

<commit_message>
Fill 7 more rows per user's pricing decisions (25, 16, 53-55, 57, 65)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E9QvuhBZminJvrtKVH8YY8
</commit_message>
<xml_diff>
--- a/kirill/outputs/2026-09-03-קופח-מכרזים-מולא-מטבלאות-אביזרים.xlsx
+++ b/kirill/outputs/2026-09-03-קופח-מכרזים-מולא-מטבלאות-אביזרים.xlsx
@@ -1193,6 +1193,26 @@
           <t>קיים במגוון</t>
         </is>
       </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>מולא לפי המחיר הנמוך מבין 3 מחירים מתחרים בטבלת המקור (דף 02!22: 30/70/100/42/50). קיימים גם: 32/73/105/47/55 (דף 02!21,24) ו-32/74/106/48/56 (דף 02!23).</t>
+        </is>
+      </c>
+      <c r="M16" t="n">
+        <v>30</v>
+      </c>
+      <c r="N16" t="n">
+        <v>70</v>
+      </c>
+      <c r="O16" t="n">
+        <v>100</v>
+      </c>
+      <c r="P16" t="n">
+        <v>42</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="10">
       <c r="A17" s="15" t="inlineStr">
@@ -1553,8 +1573,23 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>דוגמא והצעת מחיר -E-LIFE</t>
-        </is>
+          <t>דוגמא והצעת מחיר -E-LIFE | מולא לפי המחיר הנמוך מבין 2 מחירים מתחרים בטבלת המקור (דף 02!13: 121/283/404/300/354). קיים מחיר חלופי גבוה יותר: 174/407/581/450/531 (דף 02!12).</t>
+        </is>
+      </c>
+      <c r="M25" t="n">
+        <v>121</v>
+      </c>
+      <c r="N25" t="n">
+        <v>283</v>
+      </c>
+      <c r="O25" t="n">
+        <v>404</v>
+      </c>
+      <c r="P25" t="n">
+        <v>300</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>354</v>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="10">
@@ -2683,8 +2718,23 @@
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>לא נמצאה חלופה מתאימה DARCO</t>
-        </is>
+          <t>לא נמצאה חלופה מתאימה DARCO | מולא לפי המחיר הנמוך מבין 2 מחירים מתחרים בטבלת המקור (דף 01!12: 27/64/91/35/41). קיים מחיר חלופי גבוה יותר: 29/68/97/40/47 (דף 01!13).</t>
+        </is>
+      </c>
+      <c r="M53" t="n">
+        <v>27</v>
+      </c>
+      <c r="N53" t="n">
+        <v>64</v>
+      </c>
+      <c r="O53" t="n">
+        <v>91</v>
+      </c>
+      <c r="P53" t="n">
+        <v>35</v>
+      </c>
+      <c r="Q53" t="n">
+        <v>41</v>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="10">
@@ -2716,8 +2766,23 @@
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>לא נמצאה חלופה מתאימה DARCO</t>
-        </is>
+          <t>לא נמצאה חלופה מתאימה DARCO | מולא לפי המחיר הנמוך מבין 2 מחירים מתחרים בטבלת המקור (דף 01!12: 27/64/91/35/41). קיים מחיר חלופי גבוה יותר: 29/68/97/40/47 (דף 01!13).</t>
+        </is>
+      </c>
+      <c r="M54" t="n">
+        <v>27</v>
+      </c>
+      <c r="N54" t="n">
+        <v>64</v>
+      </c>
+      <c r="O54" t="n">
+        <v>91</v>
+      </c>
+      <c r="P54" t="n">
+        <v>35</v>
+      </c>
+      <c r="Q54" t="n">
+        <v>41</v>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="10">
@@ -2749,8 +2814,23 @@
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>לא נמצאה חלופה מתאימה DARCO</t>
-        </is>
+          <t>לא נמצאה חלופה מתאימה DARCO | מולא לפי המחיר הנמוך מבין 2 מחירים מתחרים בטבלת המקור (דף 01!12: 27/64/91/35/41). קיים מחיר חלופי גבוה יותר: 29/68/97/40/47 (דף 01!13).</t>
+        </is>
+      </c>
+      <c r="M55" t="n">
+        <v>27</v>
+      </c>
+      <c r="N55" t="n">
+        <v>64</v>
+      </c>
+      <c r="O55" t="n">
+        <v>91</v>
+      </c>
+      <c r="P55" t="n">
+        <v>35</v>
+      </c>
+      <c r="Q55" t="n">
+        <v>41</v>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="10">
@@ -2811,8 +2891,23 @@
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>לא התחלנו תהליך</t>
-        </is>
+          <t>לא התחלנו תהליך | מולא לפי המחיר הנמוך מבין 2 מחירים מתחרים בטבלת המקור (דף 01!15: 24/56/80/25/30). קיים מחיר חלופי גבוה יותר: 25/57/82/27/32 (דף 01!16).</t>
+        </is>
+      </c>
+      <c r="M57" t="n">
+        <v>24</v>
+      </c>
+      <c r="N57" t="n">
+        <v>56</v>
+      </c>
+      <c r="O57" t="n">
+        <v>80</v>
+      </c>
+      <c r="P57" t="n">
+        <v>25</v>
+      </c>
+      <c r="Q57" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="10">
@@ -3072,6 +3167,21 @@
         <is>
           <t>פריט נתפר במפעל</t>
         </is>
+      </c>
+      <c r="M65" t="n">
+        <v>44</v>
+      </c>
+      <c r="N65" t="n">
+        <v>103</v>
+      </c>
+      <c r="O65" t="n">
+        <v>147</v>
+      </c>
+      <c r="P65" t="n">
+        <v>83</v>
+      </c>
+      <c r="Q65" t="n">
+        <v>97</v>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="10">
@@ -4730,27 +4840,27 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="28" t="n">
+      <c r="A13" s="25" t="n">
         <v>16</v>
       </c>
-      <c r="B13" s="28" t="inlineStr">
+      <c r="B13" s="25" t="inlineStr">
         <is>
           <t>קיבוע אמה צמודה לבטן לאחר ניתוח</t>
         </is>
       </c>
-      <c r="C13" s="29" t="inlineStr">
-        <is>
-          <t>נבדק - לא הוכרע (מועמד קליני סביר, אך כמה מחירים מתחרים)</t>
-        </is>
-      </c>
-      <c r="D13" s="30" t="inlineStr">
-        <is>
-          <t>סבב 2 (אזור אנטומי + שיקול קליני)</t>
-        </is>
-      </c>
-      <c r="E13" s="30" t="inlineStr">
-        <is>
-          <t>מועמד קליני סביר: "קיבוע אחרי צניחה/ניתוח לאחר ניתוח" (גם קיבוע לאחר ניתוח) - אך יש לו 3 ערכי-מחיר שונים (מתוך 4 שורות) בטבלת המקור - לא ניתן לבחור</t>
+      <c r="C13" s="26" t="inlineStr">
+        <is>
+          <t>מולא - הוכרע ע"י המשתמש (מחיר נמוך + הערה)</t>
+        </is>
+      </c>
+      <c r="D13" s="27" t="inlineStr">
+        <is>
+          <t>דף 02!22</t>
+        </is>
+      </c>
+      <c r="E13" s="27" t="inlineStr">
+        <is>
+          <t>(30, 70, 100, 42, 50) — נבחר כי הוא הנמוך מבין 3 מחירים; החלופות תועדו בהערה בעמודה L</t>
         </is>
       </c>
     </row>
@@ -4955,27 +5065,27 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="28" t="n">
+      <c r="A22" s="25" t="n">
         <v>25</v>
       </c>
-      <c r="B22" s="28" t="inlineStr">
+      <c r="B22" s="25" t="inlineStr">
         <is>
           <t>חגורת Jewett 3 POINTS</t>
         </is>
       </c>
-      <c r="C22" s="29" t="inlineStr">
-        <is>
-          <t>נבדק - לא הוכרע (מועמד קליני סביר, אך כמה מחירים מתחרים)</t>
-        </is>
-      </c>
-      <c r="D22" s="30" t="inlineStr">
-        <is>
-          <t>סבב 2 (אזור אנטומי + שיקול קליני)</t>
-        </is>
-      </c>
-      <c r="E22" s="30" t="inlineStr">
-        <is>
-          <t>מועמד קליני מדויק: "חגורת גב לשברים תואם JEWETT" - התאמה ישירה בשם ההתקן! אך יש 2 ערכי-מחיר שונים בטבלת המקור - לא ניתן לבחור בלי הכרעה איזה ספק</t>
+      <c r="C22" s="26" t="inlineStr">
+        <is>
+          <t>מולא - הוכרע ע"י המשתמש (מחיר נמוך + הערה)</t>
+        </is>
+      </c>
+      <c r="D22" s="27" t="inlineStr">
+        <is>
+          <t>דף 02!13</t>
+        </is>
+      </c>
+      <c r="E22" s="27" t="inlineStr">
+        <is>
+          <t>(121, 283, 404, 300, 354) — נבחר כי הוא הנמוך מבין 2 מחירים; חלופה גבוהה 174/407/581/450/531 תועדה בהערה בעמודה L</t>
         </is>
       </c>
     </row>
@@ -5623,77 +5733,77 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="28" t="n">
+      <c r="A50" s="25" t="n">
         <v>53</v>
       </c>
-      <c r="B50" s="28" t="inlineStr">
+      <c r="B50" s="25" t="inlineStr">
         <is>
           <t>נעלי אחרי ניתוח POST OP</t>
         </is>
       </c>
-      <c r="C50" s="29" t="inlineStr">
-        <is>
-          <t>נבדק - לא הוכרע (מועמד קליני סביר, אך כמה מחירים מתחרים)</t>
-        </is>
-      </c>
-      <c r="D50" s="30" t="inlineStr">
-        <is>
-          <t>סבב 2 (אזור אנטומי + שיקול קליני)</t>
-        </is>
-      </c>
-      <c r="E50" s="30" t="inlineStr">
-        <is>
-          <t>מועמד קליני סביר: "דמוי נעל - off-loading device" (נעל פוסט-ניתוחית סטנדרטית בשוק) - אך יש לו 2 ערכי-מחיר שונים בטבלה - לא ניתן לבחור</t>
+      <c r="C50" s="26" t="inlineStr">
+        <is>
+          <t>מולא - הוכרע ע"י המשתמש (מחיר נמוך + הערה)</t>
+        </is>
+      </c>
+      <c r="D50" s="27" t="inlineStr">
+        <is>
+          <t>דף 01!12</t>
+        </is>
+      </c>
+      <c r="E50" s="27" t="inlineStr">
+        <is>
+          <t>(27, 64, 91, 35, 41) — נבחר כי הוא הנמוך מבין 2 מחירים; חלופה גבוהה 29/68/97/40/47 תועדה בהערה בעמודה L</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="28" t="n">
+      <c r="A51" s="25" t="n">
         <v>54</v>
       </c>
-      <c r="B51" s="28" t="inlineStr">
+      <c r="B51" s="25" t="inlineStr">
         <is>
           <t>נעל לאחר ניתוח/ לריפוי פצע עם הגבהה קדמית</t>
         </is>
       </c>
-      <c r="C51" s="29" t="inlineStr">
-        <is>
-          <t>נבדק - לא הוכרע (מועמד קליני סביר, אך כמה מחירים מתחרים)</t>
-        </is>
-      </c>
-      <c r="D51" s="30" t="inlineStr">
-        <is>
-          <t>סבב 2 (אזור אנטומי + שיקול קליני)</t>
-        </is>
-      </c>
-      <c r="E51" s="30" t="inlineStr">
-        <is>
-          <t>מועמד אפשרי: "דמוי נעל - off-loading device" - לא ברור אם תואם ספציפית "הגבהה קדמית" (המועמד לא מציין כיוון הגבהה), ובנוסף 2 ערכי-מחיר שונים</t>
+      <c r="C51" s="26" t="inlineStr">
+        <is>
+          <t>מולא - הוכרע ע"י המשתמש (מחיר נמוך + הערה)</t>
+        </is>
+      </c>
+      <c r="D51" s="27" t="inlineStr">
+        <is>
+          <t>דף 01!12</t>
+        </is>
+      </c>
+      <c r="E51" s="27" t="inlineStr">
+        <is>
+          <t>(27, 64, 91, 35, 41) — נבחר כי הוא הנמוך מבין 2 מחירים; חלופה גבוהה 29/68/97/40/47 תועדה בהערה בעמודה L</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="28" t="n">
+      <c r="A52" s="25" t="n">
         <v>55</v>
       </c>
-      <c r="B52" s="28" t="inlineStr">
+      <c r="B52" s="25" t="inlineStr">
         <is>
           <t>נעל לאחר ניתוח/ לריפוי פצע עם הגבהה אחורית</t>
         </is>
       </c>
-      <c r="C52" s="29" t="inlineStr">
-        <is>
-          <t>נבדק - לא הוכרע (מועמד קליני סביר, אך כמה מחירים מתחרים)</t>
-        </is>
-      </c>
-      <c r="D52" s="30" t="inlineStr">
-        <is>
-          <t>סבב 2 (אזור אנטומי + שיקול קליני)</t>
-        </is>
-      </c>
-      <c r="E52" s="30" t="inlineStr">
-        <is>
-          <t>מועמד אפשרי: "דמוי נעל - off-loading device" - לא ברור אם תואם ספציפית "הגבהה אחורית", ובנוסף 2 ערכי-מחיר שונים</t>
+      <c r="C52" s="26" t="inlineStr">
+        <is>
+          <t>מולא - הוכרע ע"י המשתמש (מחיר נמוך + הערה)</t>
+        </is>
+      </c>
+      <c r="D52" s="27" t="inlineStr">
+        <is>
+          <t>דף 01!12</t>
+        </is>
+      </c>
+      <c r="E52" s="27" t="inlineStr">
+        <is>
+          <t>(27, 64, 91, 35, 41) — נבחר כי הוא הנמוך מבין 2 מחירים; חלופה גבוהה 29/68/97/40/47 תועדה בהערה בעמודה L</t>
         </is>
       </c>
     </row>
@@ -5719,27 +5829,27 @@
       <c r="E53" s="24" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" s="28" t="n">
+      <c r="A54" s="25" t="n">
         <v>57</v>
       </c>
-      <c r="B54" s="28" t="inlineStr">
+      <c r="B54" s="25" t="inlineStr">
         <is>
           <t>עקב סיליקון בלי נקודה כחולה</t>
         </is>
       </c>
-      <c r="C54" s="29" t="inlineStr">
-        <is>
-          <t>נבדק - לא הוכרע (מועמד קליני סביר, אך כמה מחירים מתחרים)</t>
-        </is>
-      </c>
-      <c r="D54" s="30" t="inlineStr">
-        <is>
-          <t>סבב 2 (אזור אנטומי + שיקול קליני)</t>
-        </is>
-      </c>
-      <c r="E54" s="30" t="inlineStr">
-        <is>
-          <t>מועמד אפשרי: "עקב סיליקון לדורבן" - אך זה ייעודי לדורבן (אינדיקציה ספציפית) בעוד השורה במכרז היא כללית ("בלי נקודה כחולה" = מאפיין ייצור, לא אינדיקציה) - התאמה לא ודאית; ובנוסף 2 ערכי-מחיר שונים</t>
+      <c r="C54" s="26" t="inlineStr">
+        <is>
+          <t>מולא - הוכרע ע"י המשתמש (מחיר נמוך + הערה)</t>
+        </is>
+      </c>
+      <c r="D54" s="27" t="inlineStr">
+        <is>
+          <t>דף 01!15</t>
+        </is>
+      </c>
+      <c r="E54" s="27" t="inlineStr">
+        <is>
+          <t>(24, 56, 80, 25, 30) — נבחר כי הוא הנמוך מבין 2 מחירים; חלופה גבוהה 25/57/82/27/32 תועדה בהערה בעמודה L (לעקביות/שקיפות)</t>
         </is>
       </c>
     </row>
@@ -5919,27 +6029,27 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="43" t="n">
+      <c r="A62" s="25" t="n">
         <v>65</v>
       </c>
-      <c r="B62" s="43" t="inlineStr">
+      <c r="B62" s="25" t="inlineStr">
         <is>
           <t>מגני ירכיים עם ריפוד / כרית מתנפחת למניעת שבר צוואר ירך</t>
         </is>
       </c>
-      <c r="C62" s="44" t="inlineStr">
-        <is>
-          <t>נבדק - לא הוכרע (2 וריאנטים אפשריים, לא ברור איזה)</t>
-        </is>
-      </c>
-      <c r="D62" s="45" t="inlineStr">
-        <is>
-          <t>סבב 2 (אזור אנטומי + שיקול קליני)</t>
-        </is>
-      </c>
-      <c r="E62" s="45" t="inlineStr">
-        <is>
-          <t>השורה במכרז משלבת 2 מאפיינים ("עם ריפוד / כרית מתנפחת") שמופיעים כשתי שורות-מוצר נפרדות בטבלת המחירים ("מגן ירכיים עם ריפוד/כרית" בסך 44/103/147/83/97 מול "מתנפחות למניעת שבר צוואר ירך" בסך 49/113/162/95/112) - לא ברור איזה משני הווריאנטים לבחור</t>
+      <c r="C62" s="26" t="inlineStr">
+        <is>
+          <t>מולא - הוכרע ע"י המשתמש ("קח שורה 27")</t>
+        </is>
+      </c>
+      <c r="D62" s="27" t="inlineStr">
+        <is>
+          <t>דף 01!27</t>
+        </is>
+      </c>
+      <c r="E62" s="27" t="inlineStr">
+        <is>
+          <t>(44, 103, 147, 83, 97) — "מגן ירכיים עם ריפוד / כרית" — הזוהתה כ-"שורה 27" בטבלת האביזרים לפי בקשת המשתמש</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fill groups 1+2 (24/26 rows), 46/75 total filled
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E9QvuhBZminJvrtKVH8YY8
</commit_message>
<xml_diff>
--- a/kirill/outputs/2026-09-03-קופח-מכרזים-מולא-מטבלאות-אביזרים.xlsx
+++ b/kirill/outputs/2026-09-03-קופח-מכרזים-מולא-מטבלאות-אביזרים.xlsx
@@ -755,8 +755,23 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>לא התחלנו תהליך</t>
-        </is>
+          <t>לא התחלנו תהליך | מולא לפי מועמד קרוב-ניסוח ("תומך/מייצב פעיל לשורש כף היד עם אגודל") - הבדל רווח בלבד. מהמועמד היו 2 מחירים - נבחר הנמוך (דף 03!18: 39/91/130/68/80). חלופה גבוהה: 40/95/135/72/85 (דף 03!17).</t>
+        </is>
+      </c>
+      <c r="M5" t="n">
+        <v>39</v>
+      </c>
+      <c r="N5" t="n">
+        <v>91</v>
+      </c>
+      <c r="O5" t="n">
+        <v>130</v>
+      </c>
+      <c r="P5" t="n">
+        <v>68</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>80</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="10">
@@ -788,8 +803,23 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>לא התחלנו תהליך</t>
-        </is>
+          <t>לא התחלנו תהליך | מולא לפי מועמד קרוב-ניסוח ("תומך/מייצב פעיל לשורש כף היד ללא אגודל") - הבדל רווח בלבד. מהמועמד היו 2 מחירים - נבחר הנמוך (דף 03!20: 27/63/90/34/40). חלופה גבוהה: 40/93/133/70/83 (דף 03!19).</t>
+        </is>
+      </c>
+      <c r="M6" t="n">
+        <v>27</v>
+      </c>
+      <c r="N6" t="n">
+        <v>63</v>
+      </c>
+      <c r="O6" t="n">
+        <v>90</v>
+      </c>
+      <c r="P6" t="n">
+        <v>34</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>40</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="10">
@@ -878,6 +908,26 @@
           <t>קיים במגוון</t>
         </is>
       </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>מולא לפי המחיר הנמוך מבין 5 מחירים מתחרים (דף 03!22: 27/64/91/35/41). חלופות: 30/68/98/41/48 (23), 28/67/95/38/45 (24), 28/65/93/37/43 (25), 53/123/176/107/126 (26).</t>
+        </is>
+      </c>
+      <c r="M8" t="n">
+        <v>27</v>
+      </c>
+      <c r="N8" t="n">
+        <v>64</v>
+      </c>
+      <c r="O8" t="n">
+        <v>91</v>
+      </c>
+      <c r="P8" t="n">
+        <v>35</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>41</v>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="10">
       <c r="A9" s="15" t="inlineStr">
@@ -928,8 +978,23 @@
       </c>
       <c r="L9" s="15" t="inlineStr">
         <is>
-          <t>מוצר חדש בתהליך -HSY</t>
-        </is>
+          <t>מוצר חדש בתהליך -HSY | מולא לפי המחיר הנמוך מבין 2 מחירים מתחרים (דף 02!2: 27/64/91/35/41). חלופה גבוהה: 34/81/115/55/65 (דף 02!3).</t>
+        </is>
+      </c>
+      <c r="M9" t="n">
+        <v>27</v>
+      </c>
+      <c r="N9" t="n">
+        <v>64</v>
+      </c>
+      <c r="O9" t="n">
+        <v>91</v>
+      </c>
+      <c r="P9" t="n">
+        <v>35</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>41</v>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="10">
@@ -1251,8 +1316,23 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>דוגמא והצעת מחיר -HSY</t>
-        </is>
+          <t>דוגמא והצעת מחיר -HSY | מולא לפי המחיר הנמוך מבין 2 מחירים מתחרים (דף 02!30: 77/180/257/175/207). חלופה גבוהה: 101/236/337/243/287 (דף 02!29).</t>
+        </is>
+      </c>
+      <c r="M17" t="n">
+        <v>77</v>
+      </c>
+      <c r="N17" t="n">
+        <v>180</v>
+      </c>
+      <c r="O17" t="n">
+        <v>257</v>
+      </c>
+      <c r="P17" t="n">
+        <v>175</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>207</v>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="10">
@@ -1292,8 +1372,23 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>דוגמא והצעת מחיר -HSY</t>
-        </is>
+          <t>דוגמא והצעת מחיר -HSY | מולא לפי המחיר הנמוך מבין 2 מחירים מתחרים (דף 02!27: 165/387/552/425/502). חלופה גבוהה: 167/390/557/430/507 (דף 02!28).</t>
+        </is>
+      </c>
+      <c r="M18" t="n">
+        <v>165</v>
+      </c>
+      <c r="N18" t="n">
+        <v>387</v>
+      </c>
+      <c r="O18" t="n">
+        <v>552</v>
+      </c>
+      <c r="P18" t="n">
+        <v>425</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>502</v>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="10">
@@ -1500,8 +1595,23 @@
       </c>
       <c r="L23" s="15" t="inlineStr">
         <is>
-          <t>מוצר חדש בתהליך -HSY</t>
-        </is>
+          <t>מוצר חדש בתהליך -HSY | מולא לפי המחיר הנמוך מבין 2 מחירים מתחרים (דף 02!11: 43/101/144/80/94). חלופה גבוהה: 63/146/209/135/159 (דף 02!10).</t>
+        </is>
+      </c>
+      <c r="M23" t="n">
+        <v>43</v>
+      </c>
+      <c r="N23" t="n">
+        <v>101</v>
+      </c>
+      <c r="O23" t="n">
+        <v>144</v>
+      </c>
+      <c r="P23" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>94</v>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="10">
@@ -1542,6 +1652,26 @@
         <is>
           <t>חדש במגוון</t>
         </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>מולא לפי המחיר הנמוך מבין 2 מחירים מתחרים (דף 02!13: 121/283/404/300/354). חלופה גבוהה: 174/407/581/450/531 (דף 02!12).</t>
+        </is>
+      </c>
+      <c r="M24" t="n">
+        <v>121</v>
+      </c>
+      <c r="N24" t="n">
+        <v>283</v>
+      </c>
+      <c r="O24" t="n">
+        <v>404</v>
+      </c>
+      <c r="P24" t="n">
+        <v>300</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>354</v>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="10">
@@ -1641,8 +1771,23 @@
       </c>
       <c r="L26" s="15" t="inlineStr">
         <is>
-          <t>מוצר חדש בתהליך בדיקה-HSY</t>
-        </is>
+          <t>מוצר חדש בתהליך בדיקה-HSY | מולא לפי המחיר הנמוך מבין 3 מחירים מתחרים (דף 02!16: 36/82/118/58/68). חלופות: 37/87/124/63/74 (14), 49/114/163/96/113 (15).</t>
+        </is>
+      </c>
+      <c r="M26" t="n">
+        <v>36</v>
+      </c>
+      <c r="N26" t="n">
+        <v>82</v>
+      </c>
+      <c r="O26" t="n">
+        <v>118</v>
+      </c>
+      <c r="P26" t="n">
+        <v>58</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>68</v>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="10">
@@ -1766,6 +1911,21 @@
           <t>חדש במגוון</t>
         </is>
       </c>
+      <c r="M29" t="n">
+        <v>95</v>
+      </c>
+      <c r="N29" t="n">
+        <v>221</v>
+      </c>
+      <c r="O29" t="n">
+        <v>316</v>
+      </c>
+      <c r="P29" t="n">
+        <v>225</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>266</v>
+      </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="10">
       <c r="A30" s="15" t="inlineStr">
@@ -1799,6 +1959,21 @@
           <t>לא נמצאה חלופה מתאימה</t>
         </is>
       </c>
+      <c r="M30" t="n">
+        <v>31</v>
+      </c>
+      <c r="N30" t="n">
+        <v>72</v>
+      </c>
+      <c r="O30" t="n">
+        <v>103</v>
+      </c>
+      <c r="P30" t="n">
+        <v>45</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>53</v>
+      </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="10">
       <c r="A31" s="15" t="n"/>
@@ -1940,6 +2115,26 @@
           <t>קיים במגוון</t>
         </is>
       </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>מולא לפי המחיר הנמוך מבין 2 מחירים מתחרים (דף 03!9: 23/53/76/22/26). חלופה גבוהה: 24/56/80/26/30 (דף 03!10).</t>
+        </is>
+      </c>
+      <c r="M34" t="n">
+        <v>23</v>
+      </c>
+      <c r="N34" t="n">
+        <v>53</v>
+      </c>
+      <c r="O34" t="n">
+        <v>76</v>
+      </c>
+      <c r="P34" t="n">
+        <v>22</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="10">
       <c r="A35" s="15" t="n"/>
@@ -2016,8 +2211,23 @@
       </c>
       <c r="L36" s="15" t="inlineStr">
         <is>
-          <t>המוצרים מכילים כרית ג'ל ולא סיליקון</t>
-        </is>
+          <t>המוצרים מכילים כרית ג'ל ולא סיליקון | מולא לפי המחיר הנמוך מבין 3 מחירים מתחרים (דף 03!4: 26/59/85/30/35). חלופות: 44/103/147/83/97 (2), 45/104/149/84/99 (3).</t>
+        </is>
+      </c>
+      <c r="M36" t="n">
+        <v>26</v>
+      </c>
+      <c r="N36" t="n">
+        <v>59</v>
+      </c>
+      <c r="O36" t="n">
+        <v>85</v>
+      </c>
+      <c r="P36" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>35</v>
       </c>
     </row>
     <row r="37" ht="26.45" customHeight="1" s="10">
@@ -2058,6 +2268,26 @@
         <is>
           <t>חדש במגוון</t>
         </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>מולא לפי מועמד קרוב-ניסוח ("...מעל ומתחת לברך" במקום "...לקו המפרק" - אותו איבר בהקשר זה). מהמועמד היו 2 מחירים - נבחר הנמוך (דף 03!6: 38/90/128/66/78). חלופה גבוהה: 54/126/180/110/130 (דף 03!5).</t>
+        </is>
+      </c>
+      <c r="M37" t="n">
+        <v>38</v>
+      </c>
+      <c r="N37" t="n">
+        <v>90</v>
+      </c>
+      <c r="O37" t="n">
+        <v>128</v>
+      </c>
+      <c r="P37" t="n">
+        <v>66</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>78</v>
       </c>
     </row>
     <row r="38" ht="26.45" customHeight="1" s="10">
@@ -2126,8 +2356,23 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>דוגמא והצעת מחיר -HSY</t>
-        </is>
+          <t>דוגמא והצעת מחיר -HSY | מולא לפי המחיר הנמוך מבין 2 מחירים מתחרים (דף 03!7: 98/229/327/235/277). חלופה גבוהה: 104/241/345/250/295 (דף 03!8).</t>
+        </is>
+      </c>
+      <c r="M39" t="n">
+        <v>98</v>
+      </c>
+      <c r="N39" t="n">
+        <v>229</v>
+      </c>
+      <c r="O39" t="n">
+        <v>327</v>
+      </c>
+      <c r="P39" t="n">
+        <v>235</v>
+      </c>
+      <c r="Q39" t="n">
+        <v>277</v>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="10">
@@ -2170,6 +2415,21 @@
           <t>דוגמא והצעת מחיר -E-LIFE</t>
         </is>
       </c>
+      <c r="M40" t="n">
+        <v>134</v>
+      </c>
+      <c r="N40" t="n">
+        <v>311</v>
+      </c>
+      <c r="O40" t="n">
+        <v>445</v>
+      </c>
+      <c r="P40" t="n">
+        <v>335</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>395</v>
+      </c>
     </row>
     <row r="41" ht="26.45" customHeight="1" s="10">
       <c r="A41" s="15" t="inlineStr">
@@ -2208,8 +2468,23 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>דוגמא והצעת מחיר -E-LIFE</t>
-        </is>
+          <t>דוגמא והצעת מחיר -E-LIFE | מולא לפי מועמד קרוב-ניסוח ("...להחזרת הברך אחורית" - ככל הנראה טעות הקלדה במקור עבור "מגירה אחורית", מונח אורתופדי תקין). מהמועמד היו 2 מחירים - נבחר הנמוך (דף 03!12: 134/311/445/335/395). חלופה גבוהה: 185/433/618/481/568 (דף 03!13).</t>
+        </is>
+      </c>
+      <c r="M41" t="n">
+        <v>134</v>
+      </c>
+      <c r="N41" t="n">
+        <v>311</v>
+      </c>
+      <c r="O41" t="n">
+        <v>445</v>
+      </c>
+      <c r="P41" t="n">
+        <v>335</v>
+      </c>
+      <c r="Q41" t="n">
+        <v>395</v>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="10">
@@ -2249,8 +2524,23 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>דוגמא והצעת מחיר -E-LIFE</t>
-        </is>
+          <t>דוגמא והצעת מחיר -E-LIFE | מולא לפי מועמד קרוב-ניסוח ("וצידית" מול "וצדית" - איות בלבד). מהמועמד היו 3 מחירים - נבחר הנמוך (דף 03!16: 97/226/323/231/273). חלופות גבוהות: 240/559/799/635/749 (דף 03!14) ו-249/580/829/660/779 (דף 03!15).</t>
+        </is>
+      </c>
+      <c r="M42" t="n">
+        <v>97</v>
+      </c>
+      <c r="N42" t="n">
+        <v>226</v>
+      </c>
+      <c r="O42" t="n">
+        <v>323</v>
+      </c>
+      <c r="P42" t="n">
+        <v>231</v>
+      </c>
+      <c r="Q42" t="n">
+        <v>273</v>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="10">
@@ -2330,8 +2620,23 @@
       </c>
       <c r="L44" s="15" t="inlineStr">
         <is>
-          <t>מוצר חדש בתהליך -HSY</t>
-        </is>
+          <t>מוצר חדש בתהליך -HSY | מולא לפי המחיר הנמוך מבין 2 מחירים מתחרים (דף 02!32: 28/67/95/38/45). חלופה גבוהה: 33/76/109/50/59 (דף 02!31).</t>
+        </is>
+      </c>
+      <c r="M44" t="n">
+        <v>28</v>
+      </c>
+      <c r="N44" t="n">
+        <v>67</v>
+      </c>
+      <c r="O44" t="n">
+        <v>95</v>
+      </c>
+      <c r="P44" t="n">
+        <v>38</v>
+      </c>
+      <c r="Q44" t="n">
+        <v>45</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="10">
@@ -2426,8 +2731,23 @@
       </c>
       <c r="L46" s="15" t="inlineStr">
         <is>
-          <t>מוצר חדש בתהליך -HSY</t>
-        </is>
+          <t>מוצר חדש בתהליך -HSY | מולא לפי המחיר הנמוך מבין 2 מחירים מתחרים (דף 01!2: 71/165/236/158/186). חלופה גבוהה: 72/167/239/160/189 (דף 01!3).</t>
+        </is>
+      </c>
+      <c r="M46" t="n">
+        <v>71</v>
+      </c>
+      <c r="N46" t="n">
+        <v>165</v>
+      </c>
+      <c r="O46" t="n">
+        <v>236</v>
+      </c>
+      <c r="P46" t="n">
+        <v>158</v>
+      </c>
+      <c r="Q46" t="n">
+        <v>186</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="10">
@@ -2468,6 +2788,26 @@
         <is>
           <t>קיים במגוון</t>
         </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>מולא לפי מועמד קרוב-ניסוח (רווח סביב "/" בלבד). מהמועמד היו 3 מחירים - נבחר הנמוך (דף 02!34: 21/48/69/17/19). חלופות גבוהות: 21/50/71/18/21 (דף 02!33) ו-31/72/103/45/53 (דף 02!35).</t>
+        </is>
+      </c>
+      <c r="M47" t="n">
+        <v>21</v>
+      </c>
+      <c r="N47" t="n">
+        <v>48</v>
+      </c>
+      <c r="O47" t="n">
+        <v>69</v>
+      </c>
+      <c r="P47" t="n">
+        <v>17</v>
+      </c>
+      <c r="Q47" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" s="10">
@@ -2509,8 +2849,23 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>לא נמצאה חלופה מתאימה</t>
-        </is>
+          <t>לא נמצאה חלופה מתאימה | מולא לפי מועמד קרוב-ניסוח ("קרסולייה" מול "קרסוליה" - איות בלבד). מהמועמד היו 2 מחירים - נבחר הנמוך (דף 01!4: 44/102/146/81/96). חלופה גבוהה: 45/105/150/85/100 (דף 01!5).</t>
+        </is>
+      </c>
+      <c r="M48" t="n">
+        <v>44</v>
+      </c>
+      <c r="N48" t="n">
+        <v>102</v>
+      </c>
+      <c r="O48" t="n">
+        <v>146</v>
+      </c>
+      <c r="P48" t="n">
+        <v>81</v>
+      </c>
+      <c r="Q48" t="n">
+        <v>96</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="10">
@@ -2945,6 +3300,26 @@
           <t>קיים במגוון</t>
         </is>
       </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>מולא לפי המחיר הנמוך מבין 2 מחירים מתחרים (דף 01!15: 24/56/80/25/30). חלופה גבוהה: 25/57/82/27/32 (דף 01!16).</t>
+        </is>
+      </c>
+      <c r="M58" t="n">
+        <v>24</v>
+      </c>
+      <c r="N58" t="n">
+        <v>56</v>
+      </c>
+      <c r="O58" t="n">
+        <v>80</v>
+      </c>
+      <c r="P58" t="n">
+        <v>25</v>
+      </c>
+      <c r="Q58" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="10">
       <c r="A59" s="15" t="n"/>
@@ -3441,8 +3816,23 @@
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>פרוייקט סורסינג נעצר - קיימות הצעות ודוגמאות</t>
-        </is>
+          <t>פרוייקט סורסינג נעצר - קיימות הצעות ודוגמאות | מולא לפי המחיר הנמוך מבין 2 מחירים מתחרים (דף 01!21: 49/113/162/95/112). חלופה גבוהה: 54/126/180/110/130 (דף 01!22).</t>
+        </is>
+      </c>
+      <c r="M70" t="n">
+        <v>49</v>
+      </c>
+      <c r="N70" t="n">
+        <v>113</v>
+      </c>
+      <c r="O70" t="n">
+        <v>162</v>
+      </c>
+      <c r="P70" t="n">
+        <v>95</v>
+      </c>
+      <c r="Q70" t="n">
+        <v>112</v>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="10">
@@ -4577,46 +4967,46 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="22" t="n">
+      <c r="A2" s="25" t="n">
         <v>5</v>
       </c>
-      <c r="B2" s="22" t="inlineStr">
+      <c r="B2" s="25" t="inlineStr">
         <is>
           <t>תומך/ מייצב פעיל לשורש כף היד עם אגודל (עם סיליקון)</t>
         </is>
       </c>
-      <c r="C2" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — נמצאה התאמה קרובה (לא מדויקת) בטבלת המחירים, ייתכן טעות כתיב/ניסוח שונה — דורש אימות ידני</t>
-        </is>
-      </c>
-      <c r="D2" s="24" t="inlineStr">
-        <is>
-          <t>תומך/מייצב פעיל לשורש כף היד עם אגודל (עם סיליקון); תומך/מייצב פעיל לשורש כף היד ללא אגודל (עם סיליקון)</t>
-        </is>
-      </c>
-      <c r="E2" s="24" t="inlineStr"/>
+      <c r="C2" s="26" t="inlineStr">
+        <is>
+          <t>מולא - הוכרע ע"י המשתמש (התאמת ניסוח קרוב + מחיר נמוך במידת הצורך)</t>
+        </is>
+      </c>
+      <c r="D2" s="27" t="inlineStr">
+        <is>
+          <t>ראו עמודה L (הערות) בגיליון נספח יא לפרטי המקור המדויק</t>
+        </is>
+      </c>
+      <c r="E2" s="27" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="22" t="n">
+      <c r="A3" s="25" t="n">
         <v>6</v>
       </c>
-      <c r="B3" s="22" t="inlineStr">
+      <c r="B3" s="25" t="inlineStr">
         <is>
           <t>תומך/ מייצב פעיל לשורש כף היד ללא אגודל (עם סיליקון)</t>
         </is>
       </c>
-      <c r="C3" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — נמצאה התאמה קרובה (לא מדויקת) בטבלת המחירים, ייתכן טעות כתיב/ניסוח שונה — דורש אימות ידני</t>
-        </is>
-      </c>
-      <c r="D3" s="24" t="inlineStr">
-        <is>
-          <t>תומך/מייצב פעיל לשורש כף היד ללא אגודל (עם סיליקון); תומך/מייצב פעיל לשורש כף היד עם אגודל (עם סיליקון)</t>
-        </is>
-      </c>
-      <c r="E3" s="24" t="inlineStr"/>
+      <c r="C3" s="26" t="inlineStr">
+        <is>
+          <t>מולא - הוכרע ע"י המשתמש (התאמת ניסוח קרוב + מחיר נמוך במידת הצורך)</t>
+        </is>
+      </c>
+      <c r="D3" s="27" t="inlineStr">
+        <is>
+          <t>ראו עמודה L (הערות) בגיליון נספח יא לפרטי המקור המדויק</t>
+        </is>
+      </c>
+      <c r="E3" s="27" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="25" t="n">
@@ -4644,50 +5034,50 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="28" t="n">
+      <c r="A5" s="25" t="n">
         <v>8</v>
       </c>
-      <c r="B5" s="28" t="inlineStr">
+      <c r="B5" s="25" t="inlineStr">
         <is>
           <t>מגן שורש כף יד ללא קיבוע של האגודל (מקבע קשיח)</t>
         </is>
       </c>
-      <c r="C5" s="29" t="inlineStr">
-        <is>
-          <t>לא מולא — התאמה טקסטואלית מדויקת אך 5 שורות מחיר שונות בטבלת המקור (ספקים/מוצרים שונים, מחירים שונים) — נדרשת בחירה ידנית</t>
-        </is>
-      </c>
-      <c r="D5" s="30" t="inlineStr">
-        <is>
-          <t>דף 03!22; דף 03!23; דף 03!24; דף 03!25; דף 03!26</t>
-        </is>
-      </c>
-      <c r="E5" s="30" t="inlineStr">
+      <c r="C5" s="26" t="inlineStr">
+        <is>
+          <t>מולא - הוכרע ע"י המשתמש (התאמת ניסוח קרוב + מחיר נמוך במידת הצורך)</t>
+        </is>
+      </c>
+      <c r="D5" s="27" t="inlineStr">
+        <is>
+          <t>ראו עמודה L (הערות) בגיליון נספח יא לפרטי המקור המדויק</t>
+        </is>
+      </c>
+      <c r="E5" s="27" t="inlineStr">
         <is>
           <t>(27, 64, 91, 35, 41) | (30, 68, 98, 41, 48) | (28, 67, 95, 38, 45) | (28, 65, 93, 37, 43) | (53, 123, 176, 107, 126)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="28" t="n">
+      <c r="A6" s="25" t="n">
         <v>9</v>
       </c>
-      <c r="B6" s="28" t="inlineStr">
+      <c r="B6" s="25" t="inlineStr">
         <is>
           <t>מייצב אגודל ללא שורש כף יד</t>
         </is>
       </c>
-      <c r="C6" s="29" t="inlineStr">
-        <is>
-          <t>לא מולא — התאמה טקסטואלית מדויקת אך 2 שורות מחיר שונות בטבלת המקור (ספקים/מוצרים שונים, מחירים שונים) — נדרשת בחירה ידנית</t>
-        </is>
-      </c>
-      <c r="D6" s="30" t="inlineStr">
-        <is>
-          <t>דף 02!2; דף 02!3</t>
-        </is>
-      </c>
-      <c r="E6" s="30" t="inlineStr">
+      <c r="C6" s="26" t="inlineStr">
+        <is>
+          <t>מולא - הוכרע ע"י המשתמש (התאמת ניסוח קרוב + מחיר נמוך במידת הצורך)</t>
+        </is>
+      </c>
+      <c r="D6" s="27" t="inlineStr">
+        <is>
+          <t>ראו עמודה L (הערות) בגיליון נספח יא לפרטי המקור המדויק</t>
+        </is>
+      </c>
+      <c r="E6" s="27" t="inlineStr">
         <is>
           <t>(27, 64, 91, 35, 41) | (34, 81, 115, 55, 65)</t>
         </is>
@@ -4769,25 +5159,29 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="22" t="n">
+      <c r="A10" s="43" t="n">
         <v>13</v>
       </c>
-      <c r="B10" s="22" t="inlineStr">
+      <c r="B10" s="43" t="inlineStr">
         <is>
           <t>רצועה למרפק עם כרית ולחץ מבוקר למרפק טניס</t>
         </is>
       </c>
-      <c r="C10" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — נמצאה התאמה קרובה (לא מדויקת) בטבלת המחירים, ייתכן טעות כתיב/ניסוח שונה — דורש אימות ידני</t>
-        </is>
-      </c>
-      <c r="D10" s="24" t="inlineStr">
+      <c r="C10" s="44" t="inlineStr">
+        <is>
+          <t>נבדק - לא הוכרע (ספק קליני אמיתי, לא רק ניסוח)</t>
+        </is>
+      </c>
+      <c r="D10" s="45" t="inlineStr">
         <is>
           <t>רצועה למרפק עם כרית ורצועה מתחת למרפק טניס</t>
         </is>
       </c>
-      <c r="E10" s="24" t="inlineStr"/>
+      <c r="E10" s="45" t="inlineStr">
+        <is>
+          <t>לא מולא - ספק אמיתי: "עם כרית ולחץ מבוקר" (מנגנון לחץ) מול מועמד "עם כרית ורצועה מתחת" (מנגנון רצועה) - ייתכן שאלה שני סוגי רצועת מרפק-טניס שונים מכנית, לא רק ניסוח שונה. הושאר לבדיקת המשתמש.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="40" t="n">
@@ -4865,50 +5259,50 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="28" t="n">
+      <c r="A14" s="25" t="n">
         <v>17</v>
       </c>
-      <c r="B14" s="28" t="inlineStr">
+      <c r="B14" s="25" t="inlineStr">
         <is>
           <t>מקבע כתף בדרגות אבדוקציה שונות לאחר שבר, פריקה או ניתוח</t>
         </is>
       </c>
-      <c r="C14" s="29" t="inlineStr">
-        <is>
-          <t>לא מולא — התאמה טקסטואלית מדויקת אך 2 שורות מחיר שונות בטבלת המקור (ספקים/מוצרים שונים, מחירים שונים) — נדרשת בחירה ידנית</t>
-        </is>
-      </c>
-      <c r="D14" s="30" t="inlineStr">
-        <is>
-          <t>דף 02!29; דף 02!30</t>
-        </is>
-      </c>
-      <c r="E14" s="30" t="inlineStr">
+      <c r="C14" s="26" t="inlineStr">
+        <is>
+          <t>מולא - הוכרע ע"י המשתמש (התאמת ניסוח קרוב + מחיר נמוך במידת הצורך)</t>
+        </is>
+      </c>
+      <c r="D14" s="27" t="inlineStr">
+        <is>
+          <t>ראו עמודה L (הערות) בגיליון נספח יא לפרטי המקור המדויק</t>
+        </is>
+      </c>
+      <c r="E14" s="27" t="inlineStr">
         <is>
           <t>(101, 236, 337, 243, 287) | (77, 180, 257, 175, 207)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="28" t="n">
+      <c r="A15" s="25" t="n">
         <v>18</v>
       </c>
-      <c r="B15" s="28" t="inlineStr">
+      <c r="B15" s="25" t="inlineStr">
         <is>
           <t>מקבע כתף בדרגות רוטציה (סיבוב) משתנות לאחר שבר, פריקה או ניתוח</t>
         </is>
       </c>
-      <c r="C15" s="29" t="inlineStr">
-        <is>
-          <t>לא מולא — התאמה טקסטואלית מדויקת אך 2 שורות מחיר שונות בטבלת המקור (ספקים/מוצרים שונים, מחירים שונים) — נדרשת בחירה ידנית</t>
-        </is>
-      </c>
-      <c r="D15" s="30" t="inlineStr">
-        <is>
-          <t>דף 02!27; דף 02!28</t>
-        </is>
-      </c>
-      <c r="E15" s="30" t="inlineStr">
+      <c r="C15" s="26" t="inlineStr">
+        <is>
+          <t>מולא - הוכרע ע"י המשתמש (התאמת ניסוח קרוב + מחיר נמוך במידת הצורך)</t>
+        </is>
+      </c>
+      <c r="D15" s="27" t="inlineStr">
+        <is>
+          <t>ראו עמודה L (הערות) בגיליון נספח יא לפרטי המקור המדויק</t>
+        </is>
+      </c>
+      <c r="E15" s="27" t="inlineStr">
         <is>
           <t>(165, 387, 552, 425, 502) | (167, 390, 557, 430, 507)</t>
         </is>
@@ -5015,50 +5409,50 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="28" t="n">
+      <c r="A20" s="25" t="n">
         <v>23</v>
       </c>
-      <c r="B20" s="28" t="inlineStr">
+      <c r="B20" s="25" t="inlineStr">
         <is>
           <t>חגורת גב גמישה עם תמיכה + כרית (מעל 24 ס"מ)</t>
         </is>
       </c>
-      <c r="C20" s="29" t="inlineStr">
-        <is>
-          <t>לא מולא — התאמה טקסטואלית מדויקת אך 2 שורות מחיר שונות בטבלת המקור (ספקים/מוצרים שונים, מחירים שונים) — נדרשת בחירה ידנית</t>
-        </is>
-      </c>
-      <c r="D20" s="30" t="inlineStr">
-        <is>
-          <t>דף 02!10; דף 02!11</t>
-        </is>
-      </c>
-      <c r="E20" s="30" t="inlineStr">
+      <c r="C20" s="26" t="inlineStr">
+        <is>
+          <t>מולא - הוכרע ע"י המשתמש (התאמת ניסוח קרוב + מחיר נמוך במידת הצורך)</t>
+        </is>
+      </c>
+      <c r="D20" s="27" t="inlineStr">
+        <is>
+          <t>ראו עמודה L (הערות) בגיליון נספח יא לפרטי המקור המדויק</t>
+        </is>
+      </c>
+      <c r="E20" s="27" t="inlineStr">
         <is>
           <t>(63, 146, 209, 135, 159) | (43, 101, 144, 80, 94)</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="28" t="n">
+      <c r="A21" s="25" t="n">
         <v>24</v>
       </c>
-      <c r="B21" s="28" t="inlineStr">
+      <c r="B21" s="25" t="inlineStr">
         <is>
           <t>חגורת גב לשברים תואם JEWETT</t>
         </is>
       </c>
-      <c r="C21" s="29" t="inlineStr">
-        <is>
-          <t>לא מולא — התאמה טקסטואלית מדויקת אך 2 שורות מחיר שונות בטבלת המקור (ספקים/מוצרים שונים, מחירים שונים) — נדרשת בחירה ידנית</t>
-        </is>
-      </c>
-      <c r="D21" s="30" t="inlineStr">
-        <is>
-          <t>דף 02!12; דף 02!13</t>
-        </is>
-      </c>
-      <c r="E21" s="30" t="inlineStr">
+      <c r="C21" s="26" t="inlineStr">
+        <is>
+          <t>מולא - הוכרע ע"י המשתמש (התאמת ניסוח קרוב + מחיר נמוך במידת הצורך)</t>
+        </is>
+      </c>
+      <c r="D21" s="27" t="inlineStr">
+        <is>
+          <t>ראו עמודה L (הערות) בגיליון נספח יא לפרטי המקור המדויק</t>
+        </is>
+      </c>
+      <c r="E21" s="27" t="inlineStr">
         <is>
           <t>(174, 407, 581, 450, 531) | (121, 283, 404, 300, 354)</t>
         </is>
@@ -5090,25 +5484,25 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="28" t="n">
+      <c r="A23" s="25" t="n">
         <v>26</v>
       </c>
-      <c r="B23" s="28" t="inlineStr">
+      <c r="B23" s="25" t="inlineStr">
         <is>
           <t>חגורת גב חיזוקים גמישים וסגירה כפולה (מעל 24 ס"מ)</t>
         </is>
       </c>
-      <c r="C23" s="29" t="inlineStr">
-        <is>
-          <t>לא מולא — התאמה טקסטואלית מדויקת אך 3 שורות מחיר שונות בטבלת המקור (ספקים/מוצרים שונים, מחירים שונים) — נדרשת בחירה ידנית</t>
-        </is>
-      </c>
-      <c r="D23" s="30" t="inlineStr">
-        <is>
-          <t>דף 02!14; דף 02!15; דף 02!16</t>
-        </is>
-      </c>
-      <c r="E23" s="30" t="inlineStr">
+      <c r="C23" s="26" t="inlineStr">
+        <is>
+          <t>מולא - הוכרע ע"י המשתמש (התאמת ניסוח קרוב + מחיר נמוך במידת הצורך)</t>
+        </is>
+      </c>
+      <c r="D23" s="27" t="inlineStr">
+        <is>
+          <t>ראו עמודה L (הערות) בגיליון נספח יא לפרטי המקור המדויק</t>
+        </is>
+      </c>
+      <c r="E23" s="27" t="inlineStr">
         <is>
           <t>(37, 87, 124, 63, 74) | (49, 114, 163, 96, 113) | (36, 82, 118, 58, 68)</t>
         </is>
@@ -5165,46 +5559,46 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="22" t="n">
+      <c r="A26" s="25" t="n">
         <v>29</v>
       </c>
-      <c r="B26" s="22" t="inlineStr">
+      <c r="B26" s="25" t="inlineStr">
         <is>
           <t>צווארון מורכב כגון: PMT, פילדלפיה, VISTA, ASPEN - עם ריפוד</t>
         </is>
       </c>
-      <c r="C26" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — נמצאה התאמה קרובה (לא מדויקת) בטבלת המחירים, ייתכן טעות כתיב/ניסוח שונה — דורש אימות ידני</t>
-        </is>
-      </c>
-      <c r="D26" s="24" t="inlineStr">
-        <is>
-          <t>צווארון מורכב מסוג PMT, פילדלפיה, VISTA, עם ריפוד; צווארון מורכב מסוג PMT, פילדלפיה, VISTA, ללא ריפוד</t>
-        </is>
-      </c>
-      <c r="E26" s="24" t="inlineStr"/>
+      <c r="C26" s="26" t="inlineStr">
+        <is>
+          <t>מולא - הוכרע ע"י המשתמש (התאמת ניסוח קרוב + מחיר נמוך במידת הצורך)</t>
+        </is>
+      </c>
+      <c r="D26" s="27" t="inlineStr">
+        <is>
+          <t>ראו עמודה L (הערות) בגיליון נספח יא לפרטי המקור המדויק</t>
+        </is>
+      </c>
+      <c r="E26" s="27" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="22" t="n">
+      <c r="A27" s="25" t="n">
         <v>30</v>
       </c>
-      <c r="B27" s="22" t="inlineStr">
+      <c r="B27" s="25" t="inlineStr">
         <is>
           <t>צווארון מורכב כגון: PMT, פילדלפיה, VISTA, ASPEN - ללא ריפוד</t>
         </is>
       </c>
-      <c r="C27" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — נמצאה התאמה קרובה (לא מדויקת) בטבלת המחירים, ייתכן טעות כתיב/ניסוח שונה — דורש אימות ידני</t>
-        </is>
-      </c>
-      <c r="D27" s="24" t="inlineStr">
-        <is>
-          <t>צווארון מורכב מסוג PMT, פילדלפיה, VISTA, ללא ריפוד; צווארון מורכב מסוג PMT, פילדלפיה, VISTA, עם ריפוד</t>
-        </is>
-      </c>
-      <c r="E27" s="24" t="inlineStr"/>
+      <c r="C27" s="26" t="inlineStr">
+        <is>
+          <t>מולא - הוכרע ע"י המשתמש (התאמת ניסוח קרוב + מחיר נמוך במידת הצורך)</t>
+        </is>
+      </c>
+      <c r="D27" s="27" t="inlineStr">
+        <is>
+          <t>ראו עמודה L (הערות) בגיליון נספח יא לפרטי המקור המדויק</t>
+        </is>
+      </c>
+      <c r="E27" s="27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="40" t="n">
@@ -5282,25 +5676,25 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="28" t="n">
+      <c r="A31" s="25" t="n">
         <v>34</v>
       </c>
-      <c r="B31" s="28" t="inlineStr">
+      <c r="B31" s="25" t="inlineStr">
         <is>
           <t>חבק תת פיקתי</t>
         </is>
       </c>
-      <c r="C31" s="29" t="inlineStr">
-        <is>
-          <t>לא מולא — התאמה טקסטואלית מדויקת אך 2 שורות מחיר שונות בטבלת המקור (ספקים/מוצרים שונים, מחירים שונים) — נדרשת בחירה ידנית</t>
-        </is>
-      </c>
-      <c r="D31" s="30" t="inlineStr">
-        <is>
-          <t>דף 03!9; דף 03!10</t>
-        </is>
-      </c>
-      <c r="E31" s="30" t="inlineStr">
+      <c r="C31" s="26" t="inlineStr">
+        <is>
+          <t>מולא - הוכרע ע"י המשתמש (התאמת ניסוח קרוב + מחיר נמוך במידת הצורך)</t>
+        </is>
+      </c>
+      <c r="D31" s="27" t="inlineStr">
+        <is>
+          <t>ראו עמודה L (הערות) בגיליון נספח יא לפרטי המקור המדויק</t>
+        </is>
+      </c>
+      <c r="E31" s="27" t="inlineStr">
         <is>
           <t>(23, 53, 76, 22, 26) | (24, 56, 80, 26, 30)</t>
         </is>
@@ -5332,50 +5726,50 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="28" t="n">
+      <c r="A33" s="25" t="n">
         <v>36</v>
       </c>
-      <c r="B33" s="28" t="inlineStr">
+      <c r="B33" s="25" t="inlineStr">
         <is>
           <t>תומך ברך רך עם טבעת סיליקון לפיקה</t>
         </is>
       </c>
-      <c r="C33" s="29" t="inlineStr">
-        <is>
-          <t>לא מולא — התאמה טקסטואלית מדויקת אך 3 שורות מחיר שונות בטבלת המקור (ספקים/מוצרים שונים, מחירים שונים) — נדרשת בחירה ידנית</t>
-        </is>
-      </c>
-      <c r="D33" s="30" t="inlineStr">
-        <is>
-          <t>דף 03!2; דף 03!3; דף 03!4</t>
-        </is>
-      </c>
-      <c r="E33" s="30" t="inlineStr">
+      <c r="C33" s="26" t="inlineStr">
+        <is>
+          <t>מולא - הוכרע ע"י המשתמש (התאמת ניסוח קרוב + מחיר נמוך במידת הצורך)</t>
+        </is>
+      </c>
+      <c r="D33" s="27" t="inlineStr">
+        <is>
+          <t>ראו עמודה L (הערות) בגיליון נספח יא לפרטי המקור המדויק</t>
+        </is>
+      </c>
+      <c r="E33" s="27" t="inlineStr">
         <is>
           <t>(44, 103, 147, 83, 97) | (45, 104, 149, 84, 99) | (26, 59, 85, 30, 35)</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="22" t="n">
+      <c r="A34" s="25" t="n">
         <v>37</v>
       </c>
-      <c r="B34" s="22" t="inlineStr">
+      <c r="B34" s="25" t="inlineStr">
         <is>
           <t>תומך ברך ארוך עם טבעת סיליקון לפיקה ותומכי צד קשיחים (לפחות 15 ס"מ מעל ומתחת לקו המפרק)</t>
         </is>
       </c>
-      <c r="C34" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — נמצאה התאמה קרובה (לא מדויקת) בטבלת המחירים, ייתכן טעות כתיב/ניסוח שונה — דורש אימות ידני</t>
-        </is>
-      </c>
-      <c r="D34" s="24" t="inlineStr">
-        <is>
-          <t>תומך ברך ארוך עם טבעת סיליקון לפיקה ותומכי צד קשיחים (לפחות 15 ס"מ מעל ומתחת לברך)</t>
-        </is>
-      </c>
-      <c r="E34" s="24" t="inlineStr"/>
+      <c r="C34" s="26" t="inlineStr">
+        <is>
+          <t>מולא - הוכרע ע"י המשתמש (התאמת ניסוח קרוב + מחיר נמוך במידת הצורך)</t>
+        </is>
+      </c>
+      <c r="D34" s="27" t="inlineStr">
+        <is>
+          <t>ראו עמודה L (הערות) בגיליון נספח יא לפרטי המקור המדויק</t>
+        </is>
+      </c>
+      <c r="E34" s="27" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="40" t="n">
@@ -5403,92 +5797,92 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="28" t="n">
+      <c r="A36" s="25" t="n">
         <v>39</v>
       </c>
-      <c r="B36" s="28" t="inlineStr">
+      <c r="B36" s="25" t="inlineStr">
         <is>
           <t>מקבע ברך ארוך עם צירים מתכווננים POST OP</t>
         </is>
       </c>
-      <c r="C36" s="29" t="inlineStr">
-        <is>
-          <t>לא מולא — התאמה טקסטואלית מדויקת אך 2 שורות מחיר שונות בטבלת המקור (ספקים/מוצרים שונים, מחירים שונים) — נדרשת בחירה ידנית</t>
-        </is>
-      </c>
-      <c r="D36" s="30" t="inlineStr">
-        <is>
-          <t>דף 03!7; דף 03!8</t>
-        </is>
-      </c>
-      <c r="E36" s="30" t="inlineStr">
+      <c r="C36" s="26" t="inlineStr">
+        <is>
+          <t>מולא - הוכרע ע"י המשתמש (התאמת ניסוח קרוב + מחיר נמוך במידת הצורך)</t>
+        </is>
+      </c>
+      <c r="D36" s="27" t="inlineStr">
+        <is>
+          <t>ראו עמודה L (הערות) בגיליון נספח יא לפרטי המקור המדויק</t>
+        </is>
+      </c>
+      <c r="E36" s="27" t="inlineStr">
         <is>
           <t>(98, 229, 327, 235, 277) | (104, 241, 345, 250, 295)</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="22" t="n">
+      <c r="A37" s="25" t="n">
         <v>40</v>
       </c>
-      <c r="B37" s="22" t="inlineStr">
+      <c r="B37" s="25" t="inlineStr">
         <is>
           <t>מייצב ברך ליציבות קדמית וצידית עם מסגרת מתכת קלה / קרבון כולל ציר מתכוונן</t>
         </is>
       </c>
-      <c r="C37" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — נמצאה התאמה קרובה (לא מדויקת) בטבלת המחירים, ייתכן טעות כתיב/ניסוח שונה — דורש אימות ידני</t>
-        </is>
-      </c>
-      <c r="D37" s="24" t="inlineStr">
-        <is>
-          <t>מייצב ברך ליציבות קדמית וצידית עם מסגרת מתכת קלה / קיבוע כולל ציר מתכוונן</t>
-        </is>
-      </c>
-      <c r="E37" s="24" t="inlineStr"/>
+      <c r="C37" s="26" t="inlineStr">
+        <is>
+          <t>מולא - הוכרע ע"י המשתמש (התאמת ניסוח קרוב + מחיר נמוך במידת הצורך)</t>
+        </is>
+      </c>
+      <c r="D37" s="27" t="inlineStr">
+        <is>
+          <t>ראו עמודה L (הערות) בגיליון נספח יא לפרטי המקור המדויק</t>
+        </is>
+      </c>
+      <c r="E37" s="27" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="22" t="n">
+      <c r="A38" s="25" t="n">
         <v>41</v>
       </c>
-      <c r="B38" s="22" t="inlineStr">
+      <c r="B38" s="25" t="inlineStr">
         <is>
           <t>מייצב ברך לחוסר יציבות אחורית עם מסגרת מתכת קלה/קרבון ומערכת להחזרת מגירה אחורית</t>
         </is>
       </c>
-      <c r="C38" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — נמצאה התאמה קרובה (לא מדויקת) בטבלת המחירים, ייתכן טעות כתיב/ניסוח שונה — דורש אימות ידני</t>
-        </is>
-      </c>
-      <c r="D38" s="24" t="inlineStr">
-        <is>
-          <t>מייצב ברך לחוסר יציבות אחורית עם מסגרת מתכת קלה/קרבון ומערכת להחזרת הברך אחורית</t>
-        </is>
-      </c>
-      <c r="E38" s="24" t="inlineStr"/>
+      <c r="C38" s="26" t="inlineStr">
+        <is>
+          <t>מולא - הוכרע ע"י המשתמש (התאמת ניסוח קרוב + מחיר נמוך במידת הצורך)</t>
+        </is>
+      </c>
+      <c r="D38" s="27" t="inlineStr">
+        <is>
+          <t>ראו עמודה L (הערות) בגיליון נספח יא לפרטי המקור המדויק</t>
+        </is>
+      </c>
+      <c r="E38" s="27" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="22" t="n">
+      <c r="A39" s="25" t="n">
         <v>42</v>
       </c>
-      <c r="B39" s="22" t="inlineStr">
+      <c r="B39" s="25" t="inlineStr">
         <is>
           <t>מייצב ברך ליציבות קדמית אחורית וצדית רך וגמיש עם ציר מתכוונן</t>
         </is>
       </c>
-      <c r="C39" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — נמצאה התאמה קרובה (לא מדויקת) בטבלת המחירים, ייתכן טעות כתיב/ניסוח שונה — דורש אימות ידני</t>
-        </is>
-      </c>
-      <c r="D39" s="24" t="inlineStr">
-        <is>
-          <t>מייצב ברך ליציבות קדמית אחורית וצידית רך וגמיש עם ציר מתכוונן</t>
-        </is>
-      </c>
-      <c r="E39" s="24" t="inlineStr"/>
+      <c r="C39" s="26" t="inlineStr">
+        <is>
+          <t>מולא - הוכרע ע"י המשתמש (התאמת ניסוח קרוב + מחיר נמוך במידת הצורך)</t>
+        </is>
+      </c>
+      <c r="D39" s="27" t="inlineStr">
+        <is>
+          <t>ראו עמודה L (הערות) בגיליון נספח יא לפרטי המקור המדויק</t>
+        </is>
+      </c>
+      <c r="E39" s="27" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="40" t="n">
@@ -5516,25 +5910,25 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="28" t="n">
+      <c r="A41" s="25" t="n">
         <v>44</v>
       </c>
-      <c r="B41" s="28" t="inlineStr">
+      <c r="B41" s="25" t="inlineStr">
         <is>
           <t>מייצבים חצי קשיחים עם שרוכים ו/או רצועות</t>
         </is>
       </c>
-      <c r="C41" s="29" t="inlineStr">
-        <is>
-          <t>לא מולא — התאמה טקסטואלית מדויקת אך 2 שורות מחיר שונות בטבלת המקור (ספקים/מוצרים שונים, מחירים שונים) — נדרשת בחירה ידנית</t>
-        </is>
-      </c>
-      <c r="D41" s="30" t="inlineStr">
-        <is>
-          <t>דף 02!31; דף 02!32</t>
-        </is>
-      </c>
-      <c r="E41" s="30" t="inlineStr">
+      <c r="C41" s="26" t="inlineStr">
+        <is>
+          <t>מולא - הוכרע ע"י המשתמש (התאמת ניסוח קרוב + מחיר נמוך במידת הצורך)</t>
+        </is>
+      </c>
+      <c r="D41" s="27" t="inlineStr">
+        <is>
+          <t>ראו עמודה L (הערות) בגיליון נספח יא לפרטי המקור המדויק</t>
+        </is>
+      </c>
+      <c r="E41" s="27" t="inlineStr">
         <is>
           <t>(33, 76, 109, 50, 59) | (28, 67, 95, 38, 45)</t>
         </is>
@@ -5566,71 +5960,71 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="28" t="n">
+      <c r="A43" s="25" t="n">
         <v>46</v>
       </c>
-      <c r="B43" s="28" t="inlineStr">
+      <c r="B43" s="25" t="inlineStr">
         <is>
           <t>מגפיים לאחר שבר או ניתוח עם אפשרות להגבהה פנימית משתנה</t>
         </is>
       </c>
-      <c r="C43" s="29" t="inlineStr">
-        <is>
-          <t>לא מולא — התאמה טקסטואלית מדויקת אך 2 שורות מחיר שונות בטבלת המקור (ספקים/מוצרים שונים, מחירים שונים) — נדרשת בחירה ידנית</t>
-        </is>
-      </c>
-      <c r="D43" s="30" t="inlineStr">
-        <is>
-          <t>דף 01!2; דף 01!3</t>
-        </is>
-      </c>
-      <c r="E43" s="30" t="inlineStr">
+      <c r="C43" s="26" t="inlineStr">
+        <is>
+          <t>מולא - הוכרע ע"י המשתמש (התאמת ניסוח קרוב + מחיר נמוך במידת הצורך)</t>
+        </is>
+      </c>
+      <c r="D43" s="27" t="inlineStr">
+        <is>
+          <t>ראו עמודה L (הערות) בגיליון נספח יא לפרטי המקור המדויק</t>
+        </is>
+      </c>
+      <c r="E43" s="27" t="inlineStr">
         <is>
           <t>(71, 165, 236, 158, 186) | (72, 167, 239, 160, 189)</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="22" t="n">
+      <c r="A44" s="25" t="n">
         <v>47</v>
       </c>
-      <c r="B44" s="22" t="inlineStr">
+      <c r="B44" s="25" t="inlineStr">
         <is>
           <t>קרסוליה לטיפול בגידי קרסול / כף רגל</t>
         </is>
       </c>
-      <c r="C44" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — נמצאה התאמה קרובה (לא מדויקת) בטבלת המחירים, ייתכן טעות כתיב/ניסוח שונה — דורש אימות ידני</t>
-        </is>
-      </c>
-      <c r="D44" s="24" t="inlineStr">
-        <is>
-          <t>קרסוליה לטיפול בגידי קרסול/כף רגל</t>
-        </is>
-      </c>
-      <c r="E44" s="24" t="inlineStr"/>
+      <c r="C44" s="26" t="inlineStr">
+        <is>
+          <t>מולא - הוכרע ע"י המשתמש (התאמת ניסוח קרוב + מחיר נמוך במידת הצורך)</t>
+        </is>
+      </c>
+      <c r="D44" s="27" t="inlineStr">
+        <is>
+          <t>ראו עמודה L (הערות) בגיליון נספח יא לפרטי המקור המדויק</t>
+        </is>
+      </c>
+      <c r="E44" s="27" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="22" t="n">
+      <c r="A45" s="25" t="n">
         <v>48</v>
       </c>
-      <c r="B45" s="22" t="inlineStr">
+      <c r="B45" s="25" t="inlineStr">
         <is>
           <t>קרסולייה עם סיליקון לאכילס</t>
         </is>
       </c>
-      <c r="C45" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — נמצאה התאמה קרובה (לא מדויקת) בטבלת המחירים, ייתכן טעות כתיב/ניסוח שונה — דורש אימות ידני</t>
-        </is>
-      </c>
-      <c r="D45" s="24" t="inlineStr">
-        <is>
-          <t>קרסוליה עם סיליקון לאכילס</t>
-        </is>
-      </c>
-      <c r="E45" s="24" t="inlineStr"/>
+      <c r="C45" s="26" t="inlineStr">
+        <is>
+          <t>מולא - הוכרע ע"י המשתמש (התאמת ניסוח קרוב + מחיר נמוך במידת הצורך)</t>
+        </is>
+      </c>
+      <c r="D45" s="27" t="inlineStr">
+        <is>
+          <t>ראו עמודה L (הערות) בגיליון נספח יא לפרטי המקור המדויק</t>
+        </is>
+      </c>
+      <c r="E45" s="27" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="25" t="n">
@@ -5808,25 +6202,29 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="22" t="n">
+      <c r="A53" s="43" t="n">
         <v>56</v>
       </c>
-      <c r="B53" s="22" t="inlineStr">
+      <c r="B53" s="43" t="inlineStr">
         <is>
           <t>נעלי ציר עד גיל שנתיים</t>
         </is>
       </c>
-      <c r="C53" s="23" t="inlineStr">
-        <is>
-          <t>לא מולא — נמצאה התאמה קרובה (לא מדויקת) בטבלת המחירים, ייתכן טעות כתיב/ניסוח שונה — דורש אימות ידני</t>
-        </is>
-      </c>
-      <c r="D53" s="24" t="inlineStr">
+      <c r="C53" s="44" t="inlineStr">
+        <is>
+          <t>נבדק - לא הוכרע (ספק קליני אמיתי, לא רק ניסוח)</t>
+        </is>
+      </c>
+      <c r="D53" s="45" t="inlineStr">
         <is>
           <t>נעלי ציר עד ג' שנים</t>
         </is>
       </c>
-      <c r="E53" s="24" t="inlineStr"/>
+      <c r="E53" s="45" t="inlineStr">
+        <is>
+          <t>לא מולא - ספק אמיתי: "עד גיל שנתיים" (2 שנים) מול מועמד "עד ג' שנים" (3 שנים) - פער גילאים ממשי (לא טעות כתיב), עשוי להשפיע על זכאות/כיסוי. הושאר לבדיקת המשתמש.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="25" t="n">
@@ -5854,25 +6252,25 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="28" t="n">
+      <c r="A55" s="25" t="n">
         <v>58</v>
       </c>
-      <c r="B55" s="28" t="inlineStr">
+      <c r="B55" s="25" t="inlineStr">
         <is>
           <t>עקב סיליקון לדורבן</t>
         </is>
       </c>
-      <c r="C55" s="29" t="inlineStr">
-        <is>
-          <t>לא מולא — התאמה טקסטואלית מדויקת אך 2 שורות מחיר שונות בטבלת המקור (ספקים/מוצרים שונים, מחירים שונים) — נדרשת בחירה ידנית</t>
-        </is>
-      </c>
-      <c r="D55" s="30" t="inlineStr">
-        <is>
-          <t>דף 01!15; דף 01!16</t>
-        </is>
-      </c>
-      <c r="E55" s="30" t="inlineStr">
+      <c r="C55" s="26" t="inlineStr">
+        <is>
+          <t>מולא - הוכרע ע"י המשתמש (התאמת ניסוח קרוב + מחיר נמוך במידת הצורך)</t>
+        </is>
+      </c>
+      <c r="D55" s="27" t="inlineStr">
+        <is>
+          <t>ראו עמודה L (הערות) בגיליון נספח יא לפרטי המקור המדויק</t>
+        </is>
+      </c>
+      <c r="E55" s="27" t="inlineStr">
         <is>
           <t>(24, 56, 80, 25, 30) | (25, 57, 82, 27, 32)</t>
         </is>
@@ -6154,25 +6552,25 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="28" t="n">
+      <c r="A67" s="25" t="n">
         <v>70</v>
       </c>
-      <c r="B67" s="28" t="inlineStr">
+      <c r="B67" s="25" t="inlineStr">
         <is>
           <t>גרביים אלסטיות מכנסיים AT - ורידים, בצקות ורידיות, בצקות לימפאדמה</t>
         </is>
       </c>
-      <c r="C67" s="29" t="inlineStr">
-        <is>
-          <t>לא מולא — התאמה טקסטואלית מדויקת אך 2 שורות מחיר שונות בטבלת המקור (ספקים/מוצרים שונים, מחירים שונים) — נדרשת בחירה ידנית</t>
-        </is>
-      </c>
-      <c r="D67" s="30" t="inlineStr">
-        <is>
-          <t>דף 01!21; דף 01!22</t>
-        </is>
-      </c>
-      <c r="E67" s="30" t="inlineStr">
+      <c r="C67" s="26" t="inlineStr">
+        <is>
+          <t>מולא - הוכרע ע"י המשתמש (התאמת ניסוח קרוב + מחיר נמוך במידת הצורך)</t>
+        </is>
+      </c>
+      <c r="D67" s="27" t="inlineStr">
+        <is>
+          <t>ראו עמודה L (הערות) בגיליון נספח יא לפרטי המקור המדויק</t>
+        </is>
+      </c>
+      <c r="E67" s="27" t="inlineStr">
         <is>
           <t>(49, 113, 162, 95, 112) | (54, 126, 180, 110, 130)</t>
         </is>

</xml_diff>